<commit_message>
Add hydrograph storage routing to ponceau-fossé Excel model
Implement level-pool routing Q_in(t) → WSE(t) with pipe+ditch storage
and weir spill above elev_max; add Hydrogramme_entree and Routing_stockage
sheets to the workbook.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
+++ b/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
@@ -10,8 +10,10 @@
     <sheet name="Parametres" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resultat_Q9" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Courbe_de_tarage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hydrogramme_notes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Comparaison_modes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hydrogramme_entree" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Routing_stockage" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hydrogramme_notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Comparaison_modes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +51,9 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -104,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,6 +128,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2138,16 +2146,1176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Pourquoi un hydrogramme est mieux — et la différence hyétogramme / hydrogramme</t>
+          <t>Hydrogramme d'entrée Q(t) — triangle par défaut (pointe = 9 m³/s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Colonnes jaunes = hydrogramme utilisé pour le routing. Modifier t / Qin puis relancer: python build_excel.py (ou plus tard: calcul Excel direct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Options routing</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pond amont A (m²)</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0 = seulement stockage tuyau+fossé; &gt;0 ajoute un bassin amont simple</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q pointe triangle</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Montée (min)</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Descente (min)</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pas dt (min)</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>t (min)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Q_in (m³/s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1.125</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3.375</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>5.625</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>6.75</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7.875</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8.4375</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>7.875</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7.3125</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>6.75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>6.1875</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5.625</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5.0625</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>3.9375</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>3.375</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2.8125</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1.6875</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1.125</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0.5625</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Routing stockage — dS/dt = Q_in − Q_out(WSE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Méthode Euler + 1 correcteur; stockage ≈ volume ponceau + fossé trapézoïdal × L + pond amont (50 m²). TW=0.0 m (libre).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>t (min)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Q_in (m³/s)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Q_pipe (m³/s)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Q_overflow (m³/s)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Q_out (m³/s)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>HW (m)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>S (m³)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>WSE &gt; 37.4?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>35.36</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0.9012</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0.9012</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0.3575</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>35.7175</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>31.11</v>
+      </c>
+      <c r="I6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1.8738</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>1.8738</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.5367</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>35.8967</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>3.0938</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>3.0938</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.7483</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>36.1083</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>71.01000000000001</v>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>3.7839</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.4453</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>4.2292</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>1.2552</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>36.6152</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>132.02</v>
+      </c>
+      <c r="I9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>5.625</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>3.9565</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1.4971</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>5.4536</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>1.4555</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>36.8155</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>174.86</v>
+      </c>
+      <c r="I10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>4.065</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>2.5124</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>6.5774</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1.5858</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>36.9458</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>207.15</v>
+      </c>
+      <c r="I11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>7.875</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>4.1511</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>3.5437</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>7.6948</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>1.6919</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>37.0519</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>235.96</v>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>4.2237</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>4.585</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>8.8087</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>1.783</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>37.143</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>262.53</v>
+      </c>
+      <c r="I13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>8.4375</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>4.2066</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>4.3241</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>8.5306</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>1.7613</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>37.1213</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>256.06</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>7.875</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>4.1698</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>3.7961</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>7.9659</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>1.7152</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>37.0752</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>242.59</v>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>7.3125</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>3.2709</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>7.4009</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>1.6657</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>37.0257</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>228.62</v>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>4.0865</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>2.7499</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>6.8363</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>1.6121</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>36.9721</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>214.06</v>
+      </c>
+      <c r="I17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>6.1875</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>4.0382</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>2.234</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>6.2723</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1.5534</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>36.9134</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>198.78</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>5.625</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>3.9838</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>1.7252</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>5.709</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>1.488</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>36.848</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>182.59</v>
+      </c>
+      <c r="I19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>5.0625</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>3.9208</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>1.2261</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>5.1469</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>1.4133</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>36.7733</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>165.17</v>
+      </c>
+      <c r="I20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>3.8446</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0.7425</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>4.5871</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>1.3246</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>36.6846</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>145.94</v>
+      </c>
+      <c r="I21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>3.9375</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>3.7439</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.2899</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>4.0338</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>1.2102</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>36.5702</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="I22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>3.7052</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>3.7052</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.8875999999999999</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>36.2476</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>84.12</v>
+      </c>
+      <c r="I23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>2.8125</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>2.9803</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>2.9803</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0.7271</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>36.0871</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>68.92</v>
+      </c>
+      <c r="I24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>2.4552</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>2.4552</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>35.995</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>59.62</v>
+      </c>
+      <c r="I25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>1.6875</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>1.878</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>1.878</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.5374</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>35.8974</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>49.57</v>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1.2626</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>1.2626</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0.4286</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>35.7886</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="I27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0.6561</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0.6561</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.3031</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>35.6631</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="I28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0.09039999999999999</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0.09039999999999999</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0.1145</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>35.4745</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="I29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Résumé</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>WSE max</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>37.143</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>t au pic de niveau</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Q_in au même instant</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Q_out au même instant</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="n">
+        <v>8.808999999999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>S max (approx)</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="n">
+        <v>262.5</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ligne jaune = pas de temps du WSE max. Comparer au Resultat_Q9 (régime permanent): le pic transitoire peut être plus bas grâce au stockage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A38:I39"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Hyétogramme vs hydrogramme — et ce que fait ce classeur</t>
         </is>
       </c>
     </row>
@@ -2157,117 +3325,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1) Hyétogramme = pluie i(t)  [mm/h vs temps]</t>
+          <t>Hyétogramme = pluie i(t) [mm/h]. Hydrogramme = débit Q(t) [m³/s] à l'entrée du ponceau.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2) Hydrogramme = débit Q(t)  [m³/s vs temps]  ← c'est ce qu'il faut à l'entrée du ponceau</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Feuille Hydrogramme_entree : Q(t) triangulaire (pointe 9 m³/s, montée 40 min, descente 80 min).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Le modèle actuel suppose un Q CONSTANT (régime permanent). C'est utile pour:</t>
+          <t>Feuille Routing_stockage : résout dS/dt = Q_in − Q_out(WSE) avec S = f(HW).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • dimensionnement / vérification rapide à un débit de pointe</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • courbe de tarage Q vs niveau</t>
+          <t>Pour coller VOTRE hydrogramme: remplacez les Qin jaunes (idéalement via rebuild après édition du script,</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ou demandez une version 100% formules Excel).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Un hydrogramme d'entrée est mieux si vous voulez:</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • voir le niveau monter/descendre pendant l'orage</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • tenir compte du STOCKAGE dans le fossé / amont (routing)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • vérifier si le pic dépasse 37.4 m seulement quelques minutes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • coupler pluie → ruissellement (rationnel / SCS / SWMM) → Q(t) → ponceau+fossé</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Prochaine amélioration possible du classeur:</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • feuille Hydrogramme_entree avec colonnes: t (min), Q_in (m³/s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • routing niveau-stockage: dS/dt = Q_in - Q_out(WSE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • graphique WSE(t), Q_pipe(t), Q_overflow(t)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Pour l'instant: utilisez Resultat_Q9 + Courbe_de_tarage avec Q = débit de pointe.</t>
+          <t>Chaîne complète future: hyétogramme → ruissellement (rationnel/SCS) → hydrogramme → ce routing.</t>
         </is>
       </c>
     </row>
@@ -2276,7 +3378,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2294,7 +3396,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Comparaison overflow porous vs surface pour Q=9 (mêmes géométrie/S0)</t>
         </is>

</xml_diff>

<commit_message>
Document formulas and rating-curve method in Excel workbook
Add Formules_explications sheet, annotate Resultat/Courbe/Hydrogramme/
Routing with how each value is obtained, and use Excel formula for WSE.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
+++ b/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Parametres" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resultat_Q9" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Courbe_de_tarage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hydrogramme_entree" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Routing_stockage" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Hydrogramme_notes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Comparaison_modes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Formules_explications" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resultat_Q9" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Courbe_de_tarage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Hydrogramme_entree" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Routing_stockage" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Hydrogramme_notes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Comparaison_modes" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,8 +23,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="8">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +50,10 @@
       <i val="1"/>
       <color rgb="0064748B"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F5C5C"/>
     </font>
     <font>
       <b val="1"/>
@@ -109,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,18 +126,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -931,7 +943,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Cellules jaunes = entrées principales (recalculer via run_model.py / rebuild_excel.py après changement).</t>
+          <t>Cellules jaunes = entrées principales (recalculer via run_model.py / build_excel.py après changement).</t>
         </is>
       </c>
     </row>
@@ -949,221 +961,465 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Résultat pour Q permanent = 9 m³/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>Comment les valeurs sont calculées (formules + méthode)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Grandeur</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Valeur</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Unité</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Q design</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>m³/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>HW (profondeur amont)</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>1.797</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>WSE amont</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>37.157</v>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Q_ponceau</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>4.235</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>m³/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Q_débordement (fossé/rocher)</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>4.764</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>m³/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Q_total</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>m³/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Contrôle</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>compound/outlet+surface</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Capacité ponceau à la clé</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>3.598</v>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>m³/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Débordement actif?</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Dépasse elev_max 37.4?</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Interprétation: le ponceau seul (~3.6 m³/s à la clé, ~4.2 m³/s au WSE de calcul) est insuffisant pour 9 m³/s. L'excédent (~4.8 m³/s) passe dans le fossé au-dessus de la clé (mode surface / écoulement préférentiel dans le remblai 8–200 mm). WSE ≈ 37.16 m &lt; 37.4 m.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>Limite importante: ceci est un régime PERMANENT (Q constant). Pour un événement réel, un hydrogramme d'entrée Q(t) (et éventuellement stockage) est préférable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Sujet</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Formule / explication</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="35" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Important</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Les débits Q_ponceau / Q_débordement sont calculés dans Python (hydraulics.py), puis écrits dans Excel. Ce ne sont pas des formules Excel « live » (trop complexes: HDS-5 + Manning + routing). Relancer: python build_excel.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1. Cotes</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Profondeur d'eau amont au-dessus de l'invert du ponceau (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WSE</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>WSE = invert_amont + HW   →   35.36 + HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Clé (crown)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>elev_clé = invert_amont + D = 35.36 + 1.05 = 36.41 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>S0</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>S0 = (invert_amont − invert_aval) / L = (35.36 − 34.47) / 50.9 ≈ 0.0175 m/m</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>2. Courbe de tarage = quoi?</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13" ht="35" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Table qui donne le débit que le système PEUT évacuer pour chaque niveau d'eau HW. On fixe HW, on calcule Q. Ce n'est PAS un hydrogramme (qui est Q vs temps).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="35" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Pour HW = 0, 0.05, 0.10, … jusqu'à Hmax=37.4−35.36=2.04 m : Q_total(HW) = Q_pipe(HW) + Q_overflow(HW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3. Q_ponceau (FHWA HDS-5 + Manning)</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17" ht="35" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Contrôle d'entrée</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Forme 2 (SI):  HW/D = K [Q / (Ku·A·√D)]^M   (non submergé) ;  HW/D = c [Q/(Ku·A·√D)]² + Y  (submergé). Ku=1.811. Entrée biseautée: K=0.0018, M=2.5, c=0.030, Y=0.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Contrôle de sortie</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Plein tuyau: pertes H = (1+Ke) V²/(2g) + n² V² L / R^(4/3), R=D/4, Ke=0.2 (biseau). Partiellement plein: Manning circulaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Q retenu</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Q_pipe = min(Q_entrée, Q_sortie) au même HW  (le plus limitatif gouverne)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>4. Q_débordement (fossé / remblai)</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Seuil</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Débute quand HW &gt; D (au-dessus de la clé). y = HW − D</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Géométrie fossé</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Trapèze: A = (b + z·y)·y ; P = b + 2y√(1+z²) ; R = A/P   avec b=2 m, z=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mode surface (défaut)</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Manning: Q = (1/n) A R^(2/3) √S0   avec n≈0.045 (rocher 8–200 mm, écoulement préférentiel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Mode porous (option)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Wilkins approx.: V_bulk ≈ Cd·n_por·√(g·d50·S0/(1−n_por)) ; Q = A·V_bulk  (beaucoup plus petit — insuffisant seul pour 9 m³/s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>5. Régime permanent Q=9 (feuille Resultat_Q9)</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>On cherche HW tel que Q_pipe(HW)+Q_overflow(HW) = 9  (dichotomie / bisection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Résultat typique</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>WSE≈37.16 m ; Q_pipe≈4.2 ; Q_overflow≈4.8 m³/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" s="8" t="inlineStr"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>6. Hydrogramme d'entrée (triangle)</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Montée 0→Tmontée</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Q_in(t) = Qpointe · (t / Tmontée)     ex.: 9·(t/40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Descente après pic</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Q_in(t) = Qpointe · (1 − (t−Tmontée)/Tdescente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Exemple</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>t=20 min → Qin=9·20/40=4.5 ; t=40 → 9 ; t=60 → 9·(1−20/80)=6.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="35" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Pond amont A</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Surface fictive (m²) ajoutée au stockage: V_pond = A · HW. 0 = seulement tuyau+fossé. 50–500 = bassin/nappé amont simplifié.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" s="8" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>7. Routing stockage (feuille Routing_stockage)</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Bilan</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>dS/dt = Q_in − Q_out(WSE)    (continuité / level-pool)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="35" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Stockage S(HW)</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>S ≈ V_tuyau(HW)·(aire circulaire partielle × L) + V_fossé(max(0,HW−D)) + A_pond·HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Q_out</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Q_out = Q_pipe(HW) + Q_overflow(HW)  (+ déversoir large si WSE&gt;37.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="35" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Numérique</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Pas de temps subdivisés; estimateur/correcteur sur Q_out. Voir hydraulics.py → route_level_pool()</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ligne jaune</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Pas de temps où WSE est maximal</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" s="8" t="inlineStr"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>8. Fichiers source</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>hydraulics.py</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Toutes les formules hydrauliques</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>build_excel.py</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Remplit ce classeur à partir de hydraulics.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>run_model.py</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Affiche le résultat permanent dans le terminal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A20:C22"/>
-    <mergeCell ref="A16:C18"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1174,14 +1430,294 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Résultat pour Q permanent = 9 m³/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Grandeur</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Comment obtenu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Q design</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>m³/s</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Entrée utilisateur (débit de pointe permanent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>HW (profondeur amont)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>1.797</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Résolu pour Q_pipe+Q_overflow = 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>WSE amont</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>37.157</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>WSE = 35.36 + HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Q_ponceau</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>4.235</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>m³/s</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>min(contrôle entrée HDS-5, contrôle sortie Manning)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Q_débordement (fossé/rocher)</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>4.764</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>m³/s</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Manning trapèze au-dessus de la clé (mode surface)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Q_total</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>m³/s</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Q_pipe + Q_débordement</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Contrôle</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>compound/outlet+surface</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Quel mécanisme limite le débit</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Capacité ponceau à la clé</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>3.598</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>m³/s</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Q_pipe quand HW = D = 1.05 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Débordement actif?</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Oui si HW &gt; clé</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dépasse elev_max 37.4?</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Capacité insuffisante sous 37.4 si Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Interprétation: le ponceau seul (~3.6 m³/s à la clé, ~4.2 m³/s au WSE de calcul) est insuffisant pour 9 m³/s. L'excédent (~4.8 m³/s) passe dans le fossé au-dessus de la clé (mode surface / écoulement préférentiel dans le remblai 8–200 mm). WSE ≈ 37.16 m &lt; 37.4 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Voir aussi la feuille Formules_explications. Pour l'événement dans le temps: Hydrogramme_entree + Routing_stockage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A20:D21"/>
+    <mergeCell ref="A16:D18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1192,34 +1728,40 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>COMMENT LIRE: on impose HW (col A), on calcule les débits. WSE = 35.36+HW. Q_total = Q_ponceau + Q_débordement. Détail des formules → feuille Formules_explications §§2–4.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>HW (m)</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>WSE (m)</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Q_ponceau (m³/s)</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Q_débordement (m³/s)</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>Q_total (m³/s)</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>HW (m) imposé</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>WSE=35.36+HW</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Q_ponceau (HDS-5/Manning)</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Q_débord. (Manning fossé si HW&gt;D)</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Q_total = somme</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Contrôle</t>
         </is>
@@ -1229,8 +1771,9 @@
       <c r="A4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>35.36</v>
+      <c r="B4" s="12">
+        <f>35.36+A4</f>
+        <v/>
       </c>
       <c r="C4" s="4" t="n">
         <v>0</v>
@@ -1251,8 +1794,9 @@
       <c r="A5" s="4" t="n">
         <v>0.051</v>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>35.411</v>
+      <c r="B5" s="12">
+        <f>35.36+A5</f>
+        <v/>
       </c>
       <c r="C5" s="4" t="n">
         <v>0.0163</v>
@@ -1273,8 +1817,9 @@
       <c r="A6" s="4" t="n">
         <v>0.102</v>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>35.462</v>
+      <c r="B6" s="12">
+        <f>35.36+A6</f>
+        <v/>
       </c>
       <c r="C6" s="4" t="n">
         <v>0.0709</v>
@@ -1295,8 +1840,9 @@
       <c r="A7" s="4" t="n">
         <v>0.153</v>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>35.513</v>
+      <c r="B7" s="12">
+        <f>35.36+A7</f>
+        <v/>
       </c>
       <c r="C7" s="4" t="n">
         <v>0.1653</v>
@@ -1317,8 +1863,9 @@
       <c r="A8" s="4" t="n">
         <v>0.204</v>
       </c>
-      <c r="B8" s="4" t="n">
-        <v>35.564</v>
+      <c r="B8" s="12">
+        <f>35.36+A8</f>
+        <v/>
       </c>
       <c r="C8" s="4" t="n">
         <v>0.2982</v>
@@ -1339,8 +1886,9 @@
       <c r="A9" s="4" t="n">
         <v>0.255</v>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>35.615</v>
+      <c r="B9" s="12">
+        <f>35.36+A9</f>
+        <v/>
       </c>
       <c r="C9" s="4" t="n">
         <v>0.467</v>
@@ -1361,8 +1909,9 @@
       <c r="A10" s="4" t="n">
         <v>0.306</v>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>35.666</v>
+      <c r="B10" s="12">
+        <f>35.36+A10</f>
+        <v/>
       </c>
       <c r="C10" s="4" t="n">
         <v>0.6685</v>
@@ -1383,8 +1932,9 @@
       <c r="A11" s="4" t="n">
         <v>0.357</v>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>35.717</v>
+      <c r="B11" s="12">
+        <f>35.36+A11</f>
+        <v/>
       </c>
       <c r="C11" s="4" t="n">
         <v>0.8988</v>
@@ -1405,8 +1955,9 @@
       <c r="A12" s="4" t="n">
         <v>0.408</v>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>35.768</v>
+      <c r="B12" s="12">
+        <f>35.36+A12</f>
+        <v/>
       </c>
       <c r="C12" s="4" t="n">
         <v>1.1538</v>
@@ -1427,8 +1978,9 @@
       <c r="A13" s="4" t="n">
         <v>0.459</v>
       </c>
-      <c r="B13" s="4" t="n">
-        <v>35.819</v>
+      <c r="B13" s="12">
+        <f>35.36+A13</f>
+        <v/>
       </c>
       <c r="C13" s="4" t="n">
         <v>1.4286</v>
@@ -1449,8 +2001,9 @@
       <c r="A14" s="4" t="n">
         <v>0.51</v>
       </c>
-      <c r="B14" s="4" t="n">
-        <v>35.87</v>
+      <c r="B14" s="12">
+        <f>35.36+A14</f>
+        <v/>
       </c>
       <c r="C14" s="4" t="n">
         <v>1.7182</v>
@@ -1471,8 +2024,9 @@
       <c r="A15" s="4" t="n">
         <v>0.5610000000000001</v>
       </c>
-      <c r="B15" s="4" t="n">
-        <v>35.921</v>
+      <c r="B15" s="12">
+        <f>35.36+A15</f>
+        <v/>
       </c>
       <c r="C15" s="4" t="n">
         <v>2.0172</v>
@@ -1493,8 +2047,9 @@
       <c r="A16" s="4" t="n">
         <v>0.612</v>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>35.972</v>
+      <c r="B16" s="12">
+        <f>35.36+A16</f>
+        <v/>
       </c>
       <c r="C16" s="4" t="n">
         <v>2.3196</v>
@@ -1515,8 +2070,9 @@
       <c r="A17" s="4" t="n">
         <v>0.663</v>
       </c>
-      <c r="B17" s="4" t="n">
-        <v>36.023</v>
+      <c r="B17" s="12">
+        <f>35.36+A17</f>
+        <v/>
       </c>
       <c r="C17" s="4" t="n">
         <v>2.619</v>
@@ -1537,8 +2093,9 @@
       <c r="A18" s="4" t="n">
         <v>0.714</v>
       </c>
-      <c r="B18" s="4" t="n">
-        <v>36.074</v>
+      <c r="B18" s="12">
+        <f>35.36+A18</f>
+        <v/>
       </c>
       <c r="C18" s="4" t="n">
         <v>2.9086</v>
@@ -1559,8 +2116,9 @@
       <c r="A19" s="4" t="n">
         <v>0.765</v>
       </c>
-      <c r="B19" s="4" t="n">
-        <v>36.125</v>
+      <c r="B19" s="12">
+        <f>35.36+A19</f>
+        <v/>
       </c>
       <c r="C19" s="4" t="n">
         <v>3.1805</v>
@@ -1581,8 +2139,9 @@
       <c r="A20" s="4" t="n">
         <v>0.8159999999999999</v>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>36.176</v>
+      <c r="B20" s="12">
+        <f>35.36+A20</f>
+        <v/>
       </c>
       <c r="C20" s="4" t="n">
         <v>3.4261</v>
@@ -1603,8 +2162,9 @@
       <c r="A21" s="4" t="n">
         <v>0.867</v>
       </c>
-      <c r="B21" s="4" t="n">
-        <v>36.227</v>
+      <c r="B21" s="12">
+        <f>35.36+A21</f>
+        <v/>
       </c>
       <c r="C21" s="4" t="n">
         <v>3.6346</v>
@@ -1625,8 +2185,9 @@
       <c r="A22" s="4" t="n">
         <v>0.918</v>
       </c>
-      <c r="B22" s="4" t="n">
-        <v>36.278</v>
+      <c r="B22" s="12">
+        <f>35.36+A22</f>
+        <v/>
       </c>
       <c r="C22" s="4" t="n">
         <v>3.7922</v>
@@ -1647,8 +2208,9 @@
       <c r="A23" s="4" t="n">
         <v>0.969</v>
       </c>
-      <c r="B23" s="4" t="n">
-        <v>36.329</v>
+      <c r="B23" s="12">
+        <f>35.36+A23</f>
+        <v/>
       </c>
       <c r="C23" s="4" t="n">
         <v>3.8779</v>
@@ -1669,8 +2231,9 @@
       <c r="A24" s="4" t="n">
         <v>1.02</v>
       </c>
-      <c r="B24" s="4" t="n">
-        <v>36.38</v>
+      <c r="B24" s="12">
+        <f>35.36+A24</f>
+        <v/>
       </c>
       <c r="C24" s="4" t="n">
         <v>3.8445</v>
@@ -1691,8 +2254,9 @@
       <c r="A25" s="4" t="n">
         <v>1.071</v>
       </c>
-      <c r="B25" s="4" t="n">
-        <v>36.431</v>
+      <c r="B25" s="12">
+        <f>35.36+A25</f>
+        <v/>
       </c>
       <c r="C25" s="4" t="n">
         <v>3.6177</v>
@@ -1713,8 +2277,9 @@
       <c r="A26" s="4" t="n">
         <v>1.122</v>
       </c>
-      <c r="B26" s="4" t="n">
-        <v>36.482</v>
+      <c r="B26" s="12">
+        <f>35.36+A26</f>
+        <v/>
       </c>
       <c r="C26" s="4" t="n">
         <v>3.6645</v>
@@ -1735,8 +2300,9 @@
       <c r="A27" s="4" t="n">
         <v>1.173</v>
       </c>
-      <c r="B27" s="4" t="n">
-        <v>36.533</v>
+      <c r="B27" s="12">
+        <f>35.36+A27</f>
+        <v/>
       </c>
       <c r="C27" s="4" t="n">
         <v>3.7106</v>
@@ -1757,8 +2323,9 @@
       <c r="A28" s="4" t="n">
         <v>1.224</v>
       </c>
-      <c r="B28" s="4" t="n">
-        <v>36.584</v>
+      <c r="B28" s="12">
+        <f>35.36+A28</f>
+        <v/>
       </c>
       <c r="C28" s="4" t="n">
         <v>3.7562</v>
@@ -1779,8 +2346,9 @@
       <c r="A29" s="4" t="n">
         <v>1.275</v>
       </c>
-      <c r="B29" s="4" t="n">
-        <v>36.635</v>
+      <c r="B29" s="12">
+        <f>35.36+A29</f>
+        <v/>
       </c>
       <c r="C29" s="4" t="n">
         <v>3.8013</v>
@@ -1801,8 +2369,9 @@
       <c r="A30" s="4" t="n">
         <v>1.326</v>
       </c>
-      <c r="B30" s="4" t="n">
-        <v>36.686</v>
+      <c r="B30" s="12">
+        <f>35.36+A30</f>
+        <v/>
       </c>
       <c r="C30" s="4" t="n">
         <v>3.8458</v>
@@ -1823,8 +2392,9 @@
       <c r="A31" s="4" t="n">
         <v>1.377</v>
       </c>
-      <c r="B31" s="4" t="n">
-        <v>36.737</v>
+      <c r="B31" s="12">
+        <f>35.36+A31</f>
+        <v/>
       </c>
       <c r="C31" s="4" t="n">
         <v>3.8898</v>
@@ -1845,8 +2415,9 @@
       <c r="A32" s="4" t="n">
         <v>1.428</v>
       </c>
-      <c r="B32" s="4" t="n">
-        <v>36.788</v>
+      <c r="B32" s="12">
+        <f>35.36+A32</f>
+        <v/>
       </c>
       <c r="C32" s="4" t="n">
         <v>3.9333</v>
@@ -1867,8 +2438,9 @@
       <c r="A33" s="4" t="n">
         <v>1.479</v>
       </c>
-      <c r="B33" s="4" t="n">
-        <v>36.839</v>
+      <c r="B33" s="12">
+        <f>35.36+A33</f>
+        <v/>
       </c>
       <c r="C33" s="4" t="n">
         <v>3.9763</v>
@@ -1889,8 +2461,9 @@
       <c r="A34" s="4" t="n">
         <v>1.53</v>
       </c>
-      <c r="B34" s="4" t="n">
-        <v>36.89</v>
+      <c r="B34" s="12">
+        <f>35.36+A34</f>
+        <v/>
       </c>
       <c r="C34" s="4" t="n">
         <v>4.0189</v>
@@ -1911,8 +2484,9 @@
       <c r="A35" s="4" t="n">
         <v>1.581</v>
       </c>
-      <c r="B35" s="4" t="n">
-        <v>36.941</v>
+      <c r="B35" s="12">
+        <f>35.36+A35</f>
+        <v/>
       </c>
       <c r="C35" s="4" t="n">
         <v>4.061</v>
@@ -1933,8 +2507,9 @@
       <c r="A36" s="4" t="n">
         <v>1.632</v>
       </c>
-      <c r="B36" s="4" t="n">
-        <v>36.992</v>
+      <c r="B36" s="12">
+        <f>35.36+A36</f>
+        <v/>
       </c>
       <c r="C36" s="4" t="n">
         <v>4.1027</v>
@@ -1955,8 +2530,9 @@
       <c r="A37" s="4" t="n">
         <v>1.683</v>
       </c>
-      <c r="B37" s="4" t="n">
-        <v>37.043</v>
+      <c r="B37" s="12">
+        <f>35.36+A37</f>
+        <v/>
       </c>
       <c r="C37" s="4" t="n">
         <v>4.144</v>
@@ -1977,8 +2553,9 @@
       <c r="A38" s="4" t="n">
         <v>1.734</v>
       </c>
-      <c r="B38" s="4" t="n">
-        <v>37.094</v>
+      <c r="B38" s="12">
+        <f>35.36+A38</f>
+        <v/>
       </c>
       <c r="C38" s="4" t="n">
         <v>4.1848</v>
@@ -1999,8 +2576,9 @@
       <c r="A39" s="4" t="n">
         <v>1.785</v>
       </c>
-      <c r="B39" s="4" t="n">
-        <v>37.145</v>
+      <c r="B39" s="12">
+        <f>35.36+A39</f>
+        <v/>
       </c>
       <c r="C39" s="4" t="n">
         <v>4.2253</v>
@@ -2021,8 +2599,9 @@
       <c r="A40" s="4" t="n">
         <v>1.836</v>
       </c>
-      <c r="B40" s="4" t="n">
-        <v>37.196</v>
+      <c r="B40" s="12">
+        <f>35.36+A40</f>
+        <v/>
       </c>
       <c r="C40" s="4" t="n">
         <v>4.2654</v>
@@ -2043,8 +2622,9 @@
       <c r="A41" s="4" t="n">
         <v>1.887</v>
       </c>
-      <c r="B41" s="4" t="n">
-        <v>37.247</v>
+      <c r="B41" s="12">
+        <f>35.36+A41</f>
+        <v/>
       </c>
       <c r="C41" s="4" t="n">
         <v>4.3051</v>
@@ -2065,8 +2645,9 @@
       <c r="A42" s="4" t="n">
         <v>1.938</v>
       </c>
-      <c r="B42" s="4" t="n">
-        <v>37.298</v>
+      <c r="B42" s="12">
+        <f>35.36+A42</f>
+        <v/>
       </c>
       <c r="C42" s="4" t="n">
         <v>4.3445</v>
@@ -2087,8 +2668,9 @@
       <c r="A43" s="4" t="n">
         <v>1.989</v>
       </c>
-      <c r="B43" s="4" t="n">
-        <v>37.349</v>
+      <c r="B43" s="12">
+        <f>35.36+A43</f>
+        <v/>
       </c>
       <c r="C43" s="4" t="n">
         <v>4.3835</v>
@@ -2109,8 +2691,9 @@
       <c r="A44" s="4" t="n">
         <v>2.04</v>
       </c>
-      <c r="B44" s="4" t="n">
-        <v>37.4</v>
+      <c r="B44" s="12">
+        <f>35.36+A44</f>
+        <v/>
       </c>
       <c r="C44" s="4" t="n">
         <v>4.4221</v>
@@ -2131,16 +2714,26 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ligne jaune ≈ voisinage de Q_total ≈ 9 m³/s</t>
+          <t>Ligne jaune ≈ Q_total ≈ 9 m³/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Colonne B = formule Excel (=35.36+HW). Colonnes C–E = résultats Python (hydraulics.py).</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2156,7 +2749,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Hydrogramme d'entrée Q(t) — triangle par défaut (pointe = 9 m³/s)</t>
         </is>
@@ -2165,12 +2758,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Colonnes jaunes = hydrogramme utilisé pour le routing. Modifier t / Qin puis relancer: python build_excel.py (ou plus tard: calcul Excel direct).</t>
+          <t>FORMULE triangle: montée Qin=Qpointe*(t/Tmontée); descente Qin=Qpointe*(1-(t-Tmontée)/Tdescente). Ex: t=20 → 9*20/40=4.5. Colonnes jaunes générées par Python; pour changer: modifier B4–B8 puis relancer python build_excel.py. Détails → Formules_explications §§6–7.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Options routing</t>
         </is>
@@ -2182,7 +2775,7 @@
           <t>Pond amont A (m²)</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="15" t="n">
         <v>50</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -2197,7 +2790,7 @@
           <t>Q pointe triangle</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="15" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2207,7 +2800,7 @@
           <t>Montée (min)</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="15" t="n">
         <v>40</v>
       </c>
     </row>
@@ -2217,7 +2810,7 @@
           <t>Descente (min)</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="15" t="n">
         <v>80</v>
       </c>
     </row>
@@ -2227,18 +2820,18 @@
           <t>Pas dt (min)</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="15" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>t (min)</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Q_in (m³/s)</t>
         </is>
@@ -2452,7 +3045,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2473,7 +3066,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Routing stockage — dS/dt = Q_in − Q_out(WSE)</t>
         </is>
@@ -2488,47 +3081,47 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>t (min)</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Q_in (m³/s)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Q_pipe (m³/s)</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Q_overflow (m³/s)</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Q_out (m³/s)</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>HW (m)</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>WSE (m)</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>S (m³)</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>WSE &gt; 37.4?</t>
         </is>
@@ -3211,7 +3804,7 @@
     </row>
     <row r="30"/>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>Résumé</t>
         </is>
@@ -3223,7 +3816,7 @@
           <t>WSE max</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n">
+      <c r="B32" s="16" t="n">
         <v>37.143</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -3238,7 +3831,7 @@
           <t>t au pic de niveau</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="16" t="n">
         <v>40</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -3253,7 +3846,7 @@
           <t>Q_in au même instant</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B34" s="16" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3263,7 +3856,7 @@
           <t>Q_out au même instant</t>
         </is>
       </c>
-      <c r="B35" s="13" t="n">
+      <c r="B35" s="16" t="n">
         <v>8.808999999999999</v>
       </c>
     </row>
@@ -3273,7 +3866,7 @@
           <t>S max (approx)</t>
         </is>
       </c>
-      <c r="B36" s="13" t="n">
+      <c r="B36" s="16" t="n">
         <v>262.5</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -3300,7 +3893,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3313,7 +3906,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Hyétogramme vs hydrogramme — et ce que fait ce classeur</t>
         </is>
@@ -3378,7 +3971,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3396,7 +3989,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Comparaison overflow porous vs surface pour Q=9 (mêmes géométrie/S0)</t>
         </is>
@@ -3404,32 +3997,32 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Mode</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>WSE (m)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Q_pipe</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Q_overflow</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Q_total</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Sous 37.4?</t>
         </is>
@@ -3509,7 +4102,7 @@
     </row>
     <row r="7"/>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Note: mode porous (Wilkins) seul ne passe pas ~9 m³/s sous 37.4 m. Mode surface (fossé rugueux / macropores dans 8–200 mm) est le défaut pratique.</t>
         </is>

</xml_diff>

<commit_message>
Expand Excel overflow Manning formulas and Bernoulli note
Add step-by-step A, P, R, Q_overflow formulas with numeric example,
plus a clear section explaining why open-channel Manning is used above
the crown instead of a pure Bernoulli orifice equation.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
+++ b/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
@@ -961,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1150,12 +1150,12 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>4. Q_débordement (fossé / remblai)</t>
+          <t>4. Q_débordement surface — formules complètes (quand HW &gt; D)</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr"/>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22" ht="35" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>Seuil</t>
@@ -1163,139 +1163,163 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Débute quand HW &gt; D (au-dessus de la clé). y = HW − D</t>
+          <t>Si HW &lt;= D : Q_overflow = 0.  Si HW &gt; D : y = HW - D  (profondeur d'eau AU-DESSUS de la clé)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Géométrie fossé</t>
+          <t>Exemple</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Trapèze: A = (b + z·y)·y ; P = b + 2y√(1+z²) ; R = A/P   avec b=2 m, z=2</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="35" customHeight="1">
+          <t>HW = 1.78 m, D = 1.05 m  →  y = 1.78 - 1.05 = 0.73 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mode surface (défaut)</t>
+          <t>Géométrie trapèze</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Manning: Q = (1/n) A R^(2/3) √S0   avec n≈0.045 (rocher 8–200 mm, écoulement préférentiel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="35" customHeight="1">
+          <t>b = 2 m (fond), z = 2 (talus 2H:1V)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mode porous (option)</t>
+          <t>Aire A</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Wilkins approx.: V_bulk ≈ Cd·n_por·√(g·d50·S0/(1−n_por)) ; Q = A·V_bulk  (beaucoup plus petit — insuffisant seul pour 9 m³/s)</t>
+          <t>A = (b + z*y) * y</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" t="inlineStr"/>
-      <c r="B26" s="8" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Exemple A</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>A = (2 + 2*0.73) * 0.73 = (2 + 1.46) * 0.73 = 3.46 * 0.73 ≈ 2.53 m²</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>5. Régime permanent Q=9 (feuille Resultat_Q9)</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Périmètre mouillé P</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>P = b + 2*y*sqrt(1 + z^2)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Méthode</t>
+          <t>Exemple P</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>On cherche HW tel que Q_pipe(HW)+Q_overflow(HW) = 9  (dichotomie / bisection)</t>
+          <t>P = 2 + 2*0.73*sqrt(1+4) = 2 + 1.46*sqrt(5) ≈ 2 + 1.46*2.236 ≈ 5.26 m</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Résultat typique</t>
+          <t>Rayon hydraulique R</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>WSE≈37.16 m ; Q_pipe≈4.2 ; Q_overflow≈4.8 m³/s</t>
+          <t>R = A / P</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" s="8" t="inlineStr"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Exemple R</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>R ≈ 2.53 / 5.26 ≈ 0.48 m</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>6. Hydrogramme d'entrée (triangle)</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>FORMULE Manning</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Q_overflow = (1/n) * A * R^(2/3) * S0^(1/2)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Montée 0→Tmontée</t>
+          <t>Paramètres</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Q_in(t) = Qpointe · (t / Tmontée)     ex.: 9·(t/40)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
+          <t>n ≈ 0.045 (fossé enroché / rocher 8–200 mm), S0 ≈ 0.0175 (pente du site)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="35" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Descente après pic</t>
+          <t>Exemple Q</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Q_in(t) = Qpointe · (1 − (t−Tmontée)/Tdescente)</t>
+          <t>Q ≈ (1/0.045) * 2.53 * (0.48)^(2/3) * sqrt(0.0175) ≈ 22.3 * 2.53 * 0.61 * 0.132 ≈ 4.5 m³/s (ordre de grandeur)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Exemple</t>
+          <t>Où c'est codé</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>t=20 min → Qin=9·20/40=4.5 ; t=40 → 9 ; t=60 → 9·(1−20/80)=6.75</t>
+          <t>hydraulics.py → overflow_Q() + _manning_Q() + _trapezoid()</t>
         </is>
       </c>
     </row>
     <row r="35" ht="35" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Pond amont A</t>
+          <t>Mode porous (option)</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Surface fictive (m²) ajoutée au stockage: V_pond = A · HW. 0 = seulement tuyau+fossé. 50–500 = bassin/nappé amont simplifié.</t>
+          <t>Wilkins: V_bulk ≈ Cd * n_por * sqrt(g * d50 * S0 / (1 - n_por)) ; Q = A * V_bulk  (beaucoup plus petit — insuffisant seul pour 9 m³/s)</t>
         </is>
       </c>
     </row>
@@ -1306,114 +1330,294 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>7. Routing stockage (feuille Routing_stockage)</t>
+          <t>5. Pourquoi Manning et pas Bernoulli pour le débordement?</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="35" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Bilan</t>
+          <t>Bernoulli EST utilisé</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>dS/dt = Q_in − Q_out(WSE)    (continuité / level-pool)</t>
+          <t>Pour le PONCET (contrôle de sortie): équation d'énergie / Bernoulli avec pertes: HW = TW + (1+Ke)*V^2/(2g) + pertes de frottement Manning</t>
         </is>
       </c>
     </row>
     <row r="39" ht="35" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Stockage S(HW)</t>
+          <t>Pourquoi pas Bernoulli seul au-dessus de D</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>S ≈ V_tuyau(HW)·(aire circulaire partielle × L) + V_fossé(max(0,HW−D)) + A_pond·HW</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
+          <t>Au-dessus de la clé, l'eau ne passe pas par un petit orifice court. Elle s'écoule dans un LONG fossé trapézoïdal rugueux (enrochement). Ce n'est pas un orifice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="35" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Q_out</t>
+          <t>Formule orifice (à éviter ici)</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Q_out = Q_pipe(HW) + Q_overflow(HW)  (+ déversoir large si WSE&gt;37.4)</t>
+          <t>Q = Cd * A * sqrt(2*g*H)  viendrait de Bernoulli sans frottement — OK pour orifice/déversoir COURT, FAUX pour un canal long: ignore L, n, pente → surestime fortement Q</t>
         </is>
       </c>
     </row>
     <row r="41" ht="35" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Numérique</t>
+          <t>Lien Manning ↔ énergie</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Pas de temps subdivisés; estimateur/correcteur sur Q_out. Voir hydraulics.py → route_level_pool()</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
+          <t>Manning EST une forme pratique de Bernoulli/énergie en canal: on remplace les pertes de charge inconnues par une formule empirique de frottement (n, R, S)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="35" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ligne jaune</t>
+          <t>Alternative déversoir</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Pas de temps où WSE est maximal</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" s="8" t="inlineStr"/>
+          <t>Si l'eau débordait seulement sur une crête de route courte, on utiliserait un déversoir (aussi dérivé de Bernoulli). Ici le chemin est un fossé en pente → Manning canal ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="35" customHeight="1">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Résumé</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Pipe = HDS-5 + Bernoulli/énergie+pertes. Overflow fossé = Manning canal ouvert. Les deux reposent sur l'énergie; le frottement décide la formule.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="9" t="inlineStr">
-        <is>
-          <t>8. Fichiers source</t>
-        </is>
-      </c>
+      <c r="A44" t="inlineStr"/>
       <c r="B44" s="8" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>hydraulics.py</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>Toutes les formules hydrauliques</t>
-        </is>
-      </c>
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>6. Régime permanent Q=9 (feuille Resultat_Q9)</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" t="inlineStr">
         <is>
-          <t>build_excel.py</t>
+          <t>Méthode</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Remplit ce classeur à partir de hydraulics.py</t>
+          <t>On cherche HW tel que Q_pipe(HW)+Q_overflow(HW) = 9  (dichotomie / bisection)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
+          <t>Résultat typique</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>WSE≈37.16 m ; Q_pipe≈4.2 ; Q_overflow≈4.8 m³/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" s="8" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>7. Hydrogramme d'entrée (triangle)</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Montée 0→Tmontée</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Q_in(t) = Qpointe * (t / Tmontée)     ex.: 9*(t/40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Descente après pic</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Q_in(t) = Qpointe * (1 - (t-Tmontée)/Tdescente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Exemple</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>t=20 min → Qin=9*20/40=4.5 ; t=40 → 9 ; t=60 → 9*(1-20/80)=6.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="35" customHeight="1">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Pond amont A</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Surface fictive (m²) ajoutée au stockage: V_pond = A * HW. 0 = seulement tuyau+fossé. 50–500 = bassin/nappé amont simplifié.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" s="8" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>8. Routing stockage (feuille Routing_stockage)</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Bilan</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>dS/dt = Q_in - Q_out(WSE)    (continuité / level-pool)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Stockage S(HW)</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>S ≈ V_tuyau(HW) + V_fossé(max(0,HW-D)) + A_pond*HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Q_out</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Q_out = Q_pipe(HW) + Q_overflow(HW)  (+ déversoir large si WSE&gt;37.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="35" customHeight="1">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Numérique</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>Pas de temps subdivisés; estimateur/correcteur sur Q_out. Voir hydraulics.py → route_level_pool()</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Ligne jaune</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Pas de temps où WSE est maximal</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" s="8" t="inlineStr"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>9. Fichiers source</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr"/>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>hydraulics.py</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Toutes les formules hydrauliques</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>build_excel.py</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>Remplit ce classeur à partir de hydraulics.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>run_model.py</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B65" s="8" t="inlineStr">
         <is>
           <t>Affiche le résultat permanent dans le terminal</t>
         </is>
@@ -2758,7 +2962,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>FORMULE triangle: montée Qin=Qpointe*(t/Tmontée); descente Qin=Qpointe*(1-(t-Tmontée)/Tdescente). Ex: t=20 → 9*20/40=4.5. Colonnes jaunes générées par Python; pour changer: modifier B4–B8 puis relancer python build_excel.py. Détails → Formules_explications §§6–7.</t>
+          <t>FORMULE triangle: montée Qin=Qpointe*(t/Tmontée); descente Qin=Qpointe*(1-(t-Tmontée)/Tdescente). Ex: t=20 → 9*20/40=4.5. Colonnes jaunes générées par Python; pour changer: modifier B4–B8 puis relancer python build_excel.py. Détails → Formules_explications §§7–8.</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3279,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Méthode Euler + 1 correcteur; stockage ≈ volume ponceau + fossé trapézoïdal × L + pond amont (50 m²). TW=0.0 m (libre).</t>
+          <t>FORMULE: dS/dt = Qin − Qout(WSE), avec Qout = Q_pipe(HW)+Q_overflow(HW). S = volume tuyau + fossé × L + pond(50 m²)×HW. TW=0.0 m. Voir Formules_explications §7.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify HW (depth) vs WSE (elevation) on Routing sheet
Headers and summary now distinguish profondeur (~1.7 m) from
élévation (~37 m) so users do not confuse HW with WSE.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
+++ b/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
@@ -4902,14 +4902,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Utilise Courbe_de_tarage (formules Parametres). Géométrie OU hydrogramme → WSE max live.</t>
+          <t>IMPORTANT: HW ≈ 1.7 m = PROFONDEUR au-dessus de l'invert. WSE ≈ 37.0 m = ÉLÉVATION absolue = invert(35.36) + HW. Ce n'est pas une erreur: avant vous lisiez WSE (~37); HW (~1.7) est seulement la profondeur.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
-          <t>2S/dt−Q = report Puls. RHS = cible Ind. FORECAST = interpolation.</t>
+          <t>Formule: WSE = Parametres!C9 + HW.  2S/dt−Q = report Puls. RHS = cible Ind.</t>
         </is>
       </c>
     </row>
@@ -4941,17 +4941,17 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>HW (m)</t>
+          <t>HW profondeur (m)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>WSE (m)</t>
+          <t>WSE élévation (m)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>S (m³)</t>
+          <t>S stockage (m³)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add Chicago (Keifer-Chu) hydrograph as default inflow
Build i(t) from IDF a,b,c with Td=60 min for this culvert/ditch,
scale Q(t) to the design peak (e.g. 10 m³/s), keep Triangle as option.
Excel formulas are live; Python chicago_hydrograph kept for validation.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
+++ b/engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,12 +62,16 @@
       <sz val="13"/>
     </font>
     <font>
-      <b val="1"/>
-    </font>
-    <font>
       <i val="1"/>
       <color rgb="0064748B"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="000F5C5C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -133,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,8 +161,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1210,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1284,7 +1289,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>Hydrogramme</t>
@@ -1292,7 +1297,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Hydrogramme_entree!B4–B8</t>
+          <t>Hydrogramme_entree: B3=Chicago|Triangle ; B5=Q pointe ; B9=Td ; B10=r ; B11–B13=IDF</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1320,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>1. Cotes</t>
+          <t>Chicago (détail)</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr"/>
@@ -1323,178 +1328,250 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WSE</t>
+          <t>IDF</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>WSE = Parametres!C9 + HW</t>
+          <t>ī(td)=a/(td+b)^c</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>i(t) avant pic</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>S0 = (invert_amont - invert_aval) / L  (Parametres!C13)</t>
+          <t>i=a*[(1-c)*(tb/r)+b]/(tb/r+b)^(c+1)   tb=tp-t   tp=r*Td</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" s="9" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>i(t) après pic</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>i=a*[(1-c)*(ta/(1-r))+b]/(ta/(1-r)+b)^(c+1)   ta=t-tp</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>2. Courbe de tarage</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17" ht="32" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Q(t)</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Q=Qpointe*i(t)/i_max   i_max=a/b^c</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Création</t>
+          <t>Td choisi</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Pour chaque HW: Q_total = Q_pipe + Q_overflow — formules Excel (plus de valeurs figées Python)</t>
+          <t>60 min pour ce site (ponceau court, Tc~10–20 min)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Q_pipe</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>MIN(entrée HDS-5, sortie Manning/énergie)</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" s="9" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Q_overflow</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Manning surface (défaut) ou Wilkins selon Parametres!C17</t>
-        </is>
-      </c>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>1. Cotes</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ind</t>
+          <t>WSE</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Ind = 2*S/dt + Q_out  (lookup routing)</t>
+          <t>WSE = Parametres!C9 + HW</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" s="9" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S0</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>S0 = (invert_amont - invert_aval) / L  (Parametres!C13)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>3. RHS / 2S/dt−Q</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
       <c r="B22" s="9" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>RHS</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>RHS = (2S/dt - Q)_prev + Qin_prev + Qin_new</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>2. Courbe de tarage</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2S/dt−Q</t>
+          <t>Création</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Terme de report Puls (pas un débit)</t>
+          <t>Pour chaque HW: Q_total = Q_pipe + Q_overflow — formules Excel (plus de valeurs figées Python)</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" s="9" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Q_pipe</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>MIN(entrée HDS-5, sortie Manning/énergie)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>4. Python conservé</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Q_overflow</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Manning surface (défaut) ou Wilkins selon Parametres!C17</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
-          <t>hydraulics.py</t>
+          <t>Ind</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Moteur de référence</t>
+          <t>Ind = 2*S/dt + Q_out  (lookup routing)</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>build_excel.py</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Régénère le .xlsx</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" s="9" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>excel_rating_formulas.py</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Texte des formules de courbe</t>
-        </is>
-      </c>
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>3. RHS / 2S/dt−Q</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
+          <t>RHS</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>RHS = (2S/dt - Q)_prev + Qin_prev + Qin_new</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2S/dt−Q</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Terme de report Puls (pas un débit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" s="9" t="inlineStr"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>4. Python conservé</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>hydraulics.py</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Moteur de référence</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>build_excel.py</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Régénère le .xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>excel_rating_formulas.py</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Texte des formules de courbe</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>run_model.py</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>Test terminal</t>
         </is>
@@ -1511,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1564,46 +1641,77 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3) Orage (pointe, montée, descente, pond)</t>
+          <t>3) Orage Chicago (défaut) ou Triangle</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   → Hydrogramme_entree B4–B8 → Routing_stockage « WSE max »</t>
+          <t xml:space="preserve">   → Hydrogramme_entree: B3=Chicago, B5=Q pointe (ex. 10), B9=Td=60 min</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   → IDF a,b,c en B11–B13 (caler sur votre station)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4) Mode débordement</t>
+          <t xml:space="preserve">   → Routing_stockage « WSE max »</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   → Parametres C17 = surface | porous | both</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Chicago en bref: hyétogramme Keifer–Chu → Q(t)=Qpointe*i(t)/i_max</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Td=60 min choisi pour ce culvert/fossé (voir Hydrogramme_notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4) Mode débordement</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   → Parametres C17 = surface | porous | both</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Python N'EST PAS requis pour ces changements.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Gardez hydraulics.py / build_excel.py pour régénérer le classeur plus tard si besoin.</t>
         </is>
@@ -1672,7 +1780,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3557,33 +3665,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Hydrogramme d'entrée Q(t) — TRIANGLE FORMULES LIVE</t>
+          <t>Hydrogramme d'entrée — Chicago (défaut) ou Triangle — FORMULES LIVE</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Éditez B4–B8 (jaunes). Voir Guide_Sans_Python.</t>
+          <t>Méthode Chicago (Keifer–Chu): hyétogramme IDF → forme de Q(t) calée sur Q pointe. Durée Td=60 min adaptée à ce ponceau/fossé (Tc site typ. 10–20 min). Pour Q=10: mettre 10 dans B5. B3=Chicago ou Triangle.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>Options (éditer ici)</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Chicago | Triangle</t>
         </is>
       </c>
     </row>
@@ -3596,48 +3715,56 @@
       <c r="B4" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="C4" s="17" t="inlineStr">
-        <is>
-          <t>stockage amont simplifié</t>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>stockage amont (ne pas déplacer: Courbe lit B4)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q pointe triangle (m³/s)</t>
+          <t>Q pointe (m³/s)</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>ex. 9 → 12</t>
+        <v>10</v>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>ex. 10 — pic de l'hydrogramme</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Montée (min)</t>
+          <t>Montée triangle (min)</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="C6" s="17" t="inlineStr"/>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>utilisé si B3=Triangle</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Descente (min)</t>
+          <t>Descente triangle (min)</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
         <v>80</v>
       </c>
-      <c r="C7" s="17" t="inlineStr"/>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>utilisé si B3=Triangle</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3648,1223 +3775,1810 @@
       <c r="B8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="17" t="inlineStr"/>
-    </row>
-    <row r="9"/>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>ne pas déplacer: Courbe/Routing lit B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Td Chicago (min)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>durée orage — défaut 60 min pour ce site</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>r (position du pic)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>tp=r*Td ; typ. 0.3–0.5 (urbain ~0.375)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IDF a</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>ī=a/(t+b)^c  [mm/h, t en min] — caler sur VOTRE IDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IDF b</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IDF c</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Chicago: i(t) (col C) puis Q=Qpointe*i/MAX(i) pour garantir le pic. Triangle: montée/descente. Voir Formules_explications + Hydrogramme_notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>i_max utilisé (auto)</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>IF(UPPER($B$3)="CHICAGO",MAX(C17:C136),1)</f>
+        <v/>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>MAX des i Chicago — Q=Qpointe*i/i_max</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>t (min)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Q_in (m³/s)</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>i Chicago (mm/h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="18">
-        <f>IF(A11="","",IF(A11&lt;=$B$6,$B$5*A11/$B$6,MAX(0,$B$5*(1-(A11-$B$6)/$B$7))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5">
-        <f>IF(A11="","",IF(A11+$B$8&gt;$B$6+$B$7,"",A11+$B$8))</f>
-        <v/>
-      </c>
-      <c r="B12" s="18">
-        <f>IF(A12="","",IF(A12&lt;=$B$6,$B$5*A12/$B$6,MAX(0,$B$5*(1-(A12-$B$6)/$B$7))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5">
-        <f>IF(A12="","",IF(A12+$B$8&gt;$B$6+$B$7,"",A12+$B$8))</f>
-        <v/>
-      </c>
-      <c r="B13" s="18">
-        <f>IF(A13="","",IF(A13&lt;=$B$6,$B$5*A13/$B$6,MAX(0,$B$5*(1-(A13-$B$6)/$B$7))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5">
-        <f>IF(A13="","",IF(A13+$B$8&gt;$B$6+$B$7,"",A13+$B$8))</f>
-        <v/>
-      </c>
-      <c r="B14" s="18">
-        <f>IF(A14="","",IF(A14&lt;=$B$6,$B$5*A14/$B$6,MAX(0,$B$5*(1-(A14-$B$6)/$B$7))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5">
-        <f>IF(A14="","",IF(A14+$B$8&gt;$B$6+$B$7,"",A14+$B$8))</f>
-        <v/>
-      </c>
-      <c r="B15" s="18">
-        <f>IF(A15="","",IF(A15&lt;=$B$6,$B$5*A15/$B$6,MAX(0,$B$5*(1-(A15-$B$6)/$B$7))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5">
-        <f>IF(A15="","",IF(A15+$B$8&gt;$B$6+$B$7,"",A15+$B$8))</f>
-        <v/>
-      </c>
-      <c r="B16" s="18">
-        <f>IF(A16="","",IF(A16&lt;=$B$6,$B$5*A16/$B$6,MAX(0,$B$5*(1-(A16-$B$6)/$B$7))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5">
-        <f>IF(A16="","",IF(A16+$B$8&gt;$B$6+$B$7,"",A16+$B$8))</f>
-        <v/>
-      </c>
       <c r="B17" s="18">
-        <f>IF(A17="","",IF(A17&lt;=$B$6,$B$5*A17/$B$6,MAX(0,$B$5*(1-(A17-$B$6)/$B$7))))</f>
+        <f>IF(A17="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C17/$B$15),IF(A17&lt;=$B$6,$B$5*A17/$B$6,MAX(0,$B$5*(1-(A17-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C17" s="18">
+        <f>IF(OR(A17="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A17&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A17))/$B$10)+$B$12)/((((($B$10*$B$9)-A17))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A17-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A17-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5">
-        <f>IF(A17="","",IF(A17+$B$8&gt;$B$6+$B$7,"",A17+$B$8))</f>
+        <f>IF(A17="","",IF(AND(UPPER($B$3)="CHICAGO",A17&lt;($B$10*$B$9),A17+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A17+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A17+$B$8)))</f>
         <v/>
       </c>
       <c r="B18" s="18">
-        <f>IF(A18="","",IF(A18&lt;=$B$6,$B$5*A18/$B$6,MAX(0,$B$5*(1-(A18-$B$6)/$B$7))))</f>
+        <f>IF(A18="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C18/$B$15),IF(A18&lt;=$B$6,$B$5*A18/$B$6,MAX(0,$B$5*(1-(A18-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C18" s="18">
+        <f>IF(OR(A18="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A18&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A18))/$B$10)+$B$12)/((((($B$10*$B$9)-A18))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A18-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A18-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5">
-        <f>IF(A18="","",IF(A18+$B$8&gt;$B$6+$B$7,"",A18+$B$8))</f>
+        <f>IF(A18="","",IF(AND(UPPER($B$3)="CHICAGO",A18&lt;($B$10*$B$9),A18+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A18+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A18+$B$8)))</f>
         <v/>
       </c>
       <c r="B19" s="18">
-        <f>IF(A19="","",IF(A19&lt;=$B$6,$B$5*A19/$B$6,MAX(0,$B$5*(1-(A19-$B$6)/$B$7))))</f>
+        <f>IF(A19="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C19/$B$15),IF(A19&lt;=$B$6,$B$5*A19/$B$6,MAX(0,$B$5*(1-(A19-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C19" s="18">
+        <f>IF(OR(A19="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A19&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A19))/$B$10)+$B$12)/((((($B$10*$B$9)-A19))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A19-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A19-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5">
-        <f>IF(A19="","",IF(A19+$B$8&gt;$B$6+$B$7,"",A19+$B$8))</f>
+        <f>IF(A19="","",IF(AND(UPPER($B$3)="CHICAGO",A19&lt;($B$10*$B$9),A19+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A19+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A19+$B$8)))</f>
         <v/>
       </c>
       <c r="B20" s="18">
-        <f>IF(A20="","",IF(A20&lt;=$B$6,$B$5*A20/$B$6,MAX(0,$B$5*(1-(A20-$B$6)/$B$7))))</f>
+        <f>IF(A20="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C20/$B$15),IF(A20&lt;=$B$6,$B$5*A20/$B$6,MAX(0,$B$5*(1-(A20-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C20" s="18">
+        <f>IF(OR(A20="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A20&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A20))/$B$10)+$B$12)/((((($B$10*$B$9)-A20))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A20-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A20-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5">
-        <f>IF(A20="","",IF(A20+$B$8&gt;$B$6+$B$7,"",A20+$B$8))</f>
+        <f>IF(A20="","",IF(AND(UPPER($B$3)="CHICAGO",A20&lt;($B$10*$B$9),A20+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A20+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A20+$B$8)))</f>
         <v/>
       </c>
       <c r="B21" s="18">
-        <f>IF(A21="","",IF(A21&lt;=$B$6,$B$5*A21/$B$6,MAX(0,$B$5*(1-(A21-$B$6)/$B$7))))</f>
+        <f>IF(A21="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C21/$B$15),IF(A21&lt;=$B$6,$B$5*A21/$B$6,MAX(0,$B$5*(1-(A21-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C21" s="18">
+        <f>IF(OR(A21="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A21&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A21))/$B$10)+$B$12)/((((($B$10*$B$9)-A21))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A21-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A21-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5">
-        <f>IF(A21="","",IF(A21+$B$8&gt;$B$6+$B$7,"",A21+$B$8))</f>
+        <f>IF(A21="","",IF(AND(UPPER($B$3)="CHICAGO",A21&lt;($B$10*$B$9),A21+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A21+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A21+$B$8)))</f>
         <v/>
       </c>
       <c r="B22" s="18">
-        <f>IF(A22="","",IF(A22&lt;=$B$6,$B$5*A22/$B$6,MAX(0,$B$5*(1-(A22-$B$6)/$B$7))))</f>
+        <f>IF(A22="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C22/$B$15),IF(A22&lt;=$B$6,$B$5*A22/$B$6,MAX(0,$B$5*(1-(A22-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C22" s="18">
+        <f>IF(OR(A22="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A22&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A22))/$B$10)+$B$12)/((((($B$10*$B$9)-A22))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A22-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A22-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5">
-        <f>IF(A22="","",IF(A22+$B$8&gt;$B$6+$B$7,"",A22+$B$8))</f>
+        <f>IF(A22="","",IF(AND(UPPER($B$3)="CHICAGO",A22&lt;($B$10*$B$9),A22+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A22+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A22+$B$8)))</f>
         <v/>
       </c>
       <c r="B23" s="18">
-        <f>IF(A23="","",IF(A23&lt;=$B$6,$B$5*A23/$B$6,MAX(0,$B$5*(1-(A23-$B$6)/$B$7))))</f>
+        <f>IF(A23="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C23/$B$15),IF(A23&lt;=$B$6,$B$5*A23/$B$6,MAX(0,$B$5*(1-(A23-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C23" s="18">
+        <f>IF(OR(A23="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A23&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A23))/$B$10)+$B$12)/((((($B$10*$B$9)-A23))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A23-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A23-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5">
-        <f>IF(A23="","",IF(A23+$B$8&gt;$B$6+$B$7,"",A23+$B$8))</f>
+        <f>IF(A23="","",IF(AND(UPPER($B$3)="CHICAGO",A23&lt;($B$10*$B$9),A23+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A23+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A23+$B$8)))</f>
         <v/>
       </c>
       <c r="B24" s="18">
-        <f>IF(A24="","",IF(A24&lt;=$B$6,$B$5*A24/$B$6,MAX(0,$B$5*(1-(A24-$B$6)/$B$7))))</f>
+        <f>IF(A24="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C24/$B$15),IF(A24&lt;=$B$6,$B$5*A24/$B$6,MAX(0,$B$5*(1-(A24-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C24" s="18">
+        <f>IF(OR(A24="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A24&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A24))/$B$10)+$B$12)/((((($B$10*$B$9)-A24))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A24-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A24-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5">
-        <f>IF(A24="","",IF(A24+$B$8&gt;$B$6+$B$7,"",A24+$B$8))</f>
+        <f>IF(A24="","",IF(AND(UPPER($B$3)="CHICAGO",A24&lt;($B$10*$B$9),A24+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A24+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A24+$B$8)))</f>
         <v/>
       </c>
       <c r="B25" s="18">
-        <f>IF(A25="","",IF(A25&lt;=$B$6,$B$5*A25/$B$6,MAX(0,$B$5*(1-(A25-$B$6)/$B$7))))</f>
+        <f>IF(A25="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C25/$B$15),IF(A25&lt;=$B$6,$B$5*A25/$B$6,MAX(0,$B$5*(1-(A25-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C25" s="18">
+        <f>IF(OR(A25="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A25&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A25))/$B$10)+$B$12)/((((($B$10*$B$9)-A25))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A25-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A25-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5">
-        <f>IF(A25="","",IF(A25+$B$8&gt;$B$6+$B$7,"",A25+$B$8))</f>
+        <f>IF(A25="","",IF(AND(UPPER($B$3)="CHICAGO",A25&lt;($B$10*$B$9),A25+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A25+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A25+$B$8)))</f>
         <v/>
       </c>
       <c r="B26" s="18">
-        <f>IF(A26="","",IF(A26&lt;=$B$6,$B$5*A26/$B$6,MAX(0,$B$5*(1-(A26-$B$6)/$B$7))))</f>
+        <f>IF(A26="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C26/$B$15),IF(A26&lt;=$B$6,$B$5*A26/$B$6,MAX(0,$B$5*(1-(A26-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C26" s="18">
+        <f>IF(OR(A26="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A26&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A26))/$B$10)+$B$12)/((((($B$10*$B$9)-A26))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A26-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A26-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5">
-        <f>IF(A26="","",IF(A26+$B$8&gt;$B$6+$B$7,"",A26+$B$8))</f>
+        <f>IF(A26="","",IF(AND(UPPER($B$3)="CHICAGO",A26&lt;($B$10*$B$9),A26+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A26+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A26+$B$8)))</f>
         <v/>
       </c>
       <c r="B27" s="18">
-        <f>IF(A27="","",IF(A27&lt;=$B$6,$B$5*A27/$B$6,MAX(0,$B$5*(1-(A27-$B$6)/$B$7))))</f>
+        <f>IF(A27="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C27/$B$15),IF(A27&lt;=$B$6,$B$5*A27/$B$6,MAX(0,$B$5*(1-(A27-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C27" s="18">
+        <f>IF(OR(A27="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A27&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A27))/$B$10)+$B$12)/((((($B$10*$B$9)-A27))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A27-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A27-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5">
-        <f>IF(A27="","",IF(A27+$B$8&gt;$B$6+$B$7,"",A27+$B$8))</f>
+        <f>IF(A27="","",IF(AND(UPPER($B$3)="CHICAGO",A27&lt;($B$10*$B$9),A27+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A27+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A27+$B$8)))</f>
         <v/>
       </c>
       <c r="B28" s="18">
-        <f>IF(A28="","",IF(A28&lt;=$B$6,$B$5*A28/$B$6,MAX(0,$B$5*(1-(A28-$B$6)/$B$7))))</f>
+        <f>IF(A28="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C28/$B$15),IF(A28&lt;=$B$6,$B$5*A28/$B$6,MAX(0,$B$5*(1-(A28-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C28" s="18">
+        <f>IF(OR(A28="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A28&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A28))/$B$10)+$B$12)/((((($B$10*$B$9)-A28))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A28-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A28-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5">
-        <f>IF(A28="","",IF(A28+$B$8&gt;$B$6+$B$7,"",A28+$B$8))</f>
+        <f>IF(A28="","",IF(AND(UPPER($B$3)="CHICAGO",A28&lt;($B$10*$B$9),A28+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A28+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A28+$B$8)))</f>
         <v/>
       </c>
       <c r="B29" s="18">
-        <f>IF(A29="","",IF(A29&lt;=$B$6,$B$5*A29/$B$6,MAX(0,$B$5*(1-(A29-$B$6)/$B$7))))</f>
+        <f>IF(A29="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C29/$B$15),IF(A29&lt;=$B$6,$B$5*A29/$B$6,MAX(0,$B$5*(1-(A29-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C29" s="18">
+        <f>IF(OR(A29="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A29&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A29))/$B$10)+$B$12)/((((($B$10*$B$9)-A29))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A29-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A29-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5">
-        <f>IF(A29="","",IF(A29+$B$8&gt;$B$6+$B$7,"",A29+$B$8))</f>
+        <f>IF(A29="","",IF(AND(UPPER($B$3)="CHICAGO",A29&lt;($B$10*$B$9),A29+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A29+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A29+$B$8)))</f>
         <v/>
       </c>
       <c r="B30" s="18">
-        <f>IF(A30="","",IF(A30&lt;=$B$6,$B$5*A30/$B$6,MAX(0,$B$5*(1-(A30-$B$6)/$B$7))))</f>
+        <f>IF(A30="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C30/$B$15),IF(A30&lt;=$B$6,$B$5*A30/$B$6,MAX(0,$B$5*(1-(A30-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C30" s="18">
+        <f>IF(OR(A30="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A30&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A30))/$B$10)+$B$12)/((((($B$10*$B$9)-A30))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A30-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A30-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5">
-        <f>IF(A30="","",IF(A30+$B$8&gt;$B$6+$B$7,"",A30+$B$8))</f>
+        <f>IF(A30="","",IF(AND(UPPER($B$3)="CHICAGO",A30&lt;($B$10*$B$9),A30+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A30+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A30+$B$8)))</f>
         <v/>
       </c>
       <c r="B31" s="18">
-        <f>IF(A31="","",IF(A31&lt;=$B$6,$B$5*A31/$B$6,MAX(0,$B$5*(1-(A31-$B$6)/$B$7))))</f>
+        <f>IF(A31="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C31/$B$15),IF(A31&lt;=$B$6,$B$5*A31/$B$6,MAX(0,$B$5*(1-(A31-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C31" s="18">
+        <f>IF(OR(A31="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A31&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A31))/$B$10)+$B$12)/((((($B$10*$B$9)-A31))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A31-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A31-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5">
-        <f>IF(A31="","",IF(A31+$B$8&gt;$B$6+$B$7,"",A31+$B$8))</f>
+        <f>IF(A31="","",IF(AND(UPPER($B$3)="CHICAGO",A31&lt;($B$10*$B$9),A31+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A31+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A31+$B$8)))</f>
         <v/>
       </c>
       <c r="B32" s="18">
-        <f>IF(A32="","",IF(A32&lt;=$B$6,$B$5*A32/$B$6,MAX(0,$B$5*(1-(A32-$B$6)/$B$7))))</f>
+        <f>IF(A32="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C32/$B$15),IF(A32&lt;=$B$6,$B$5*A32/$B$6,MAX(0,$B$5*(1-(A32-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C32" s="18">
+        <f>IF(OR(A32="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A32&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A32))/$B$10)+$B$12)/((((($B$10*$B$9)-A32))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A32-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A32-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5">
-        <f>IF(A32="","",IF(A32+$B$8&gt;$B$6+$B$7,"",A32+$B$8))</f>
+        <f>IF(A32="","",IF(AND(UPPER($B$3)="CHICAGO",A32&lt;($B$10*$B$9),A32+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A32+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A32+$B$8)))</f>
         <v/>
       </c>
       <c r="B33" s="18">
-        <f>IF(A33="","",IF(A33&lt;=$B$6,$B$5*A33/$B$6,MAX(0,$B$5*(1-(A33-$B$6)/$B$7))))</f>
+        <f>IF(A33="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C33/$B$15),IF(A33&lt;=$B$6,$B$5*A33/$B$6,MAX(0,$B$5*(1-(A33-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C33" s="18">
+        <f>IF(OR(A33="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A33&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A33))/$B$10)+$B$12)/((((($B$10*$B$9)-A33))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A33-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A33-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5">
-        <f>IF(A33="","",IF(A33+$B$8&gt;$B$6+$B$7,"",A33+$B$8))</f>
+        <f>IF(A33="","",IF(AND(UPPER($B$3)="CHICAGO",A33&lt;($B$10*$B$9),A33+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A33+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A33+$B$8)))</f>
         <v/>
       </c>
       <c r="B34" s="18">
-        <f>IF(A34="","",IF(A34&lt;=$B$6,$B$5*A34/$B$6,MAX(0,$B$5*(1-(A34-$B$6)/$B$7))))</f>
+        <f>IF(A34="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C34/$B$15),IF(A34&lt;=$B$6,$B$5*A34/$B$6,MAX(0,$B$5*(1-(A34-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C34" s="18">
+        <f>IF(OR(A34="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A34&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A34))/$B$10)+$B$12)/((((($B$10*$B$9)-A34))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A34-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A34-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5">
-        <f>IF(A34="","",IF(A34+$B$8&gt;$B$6+$B$7,"",A34+$B$8))</f>
+        <f>IF(A34="","",IF(AND(UPPER($B$3)="CHICAGO",A34&lt;($B$10*$B$9),A34+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A34+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A34+$B$8)))</f>
         <v/>
       </c>
       <c r="B35" s="18">
-        <f>IF(A35="","",IF(A35&lt;=$B$6,$B$5*A35/$B$6,MAX(0,$B$5*(1-(A35-$B$6)/$B$7))))</f>
+        <f>IF(A35="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C35/$B$15),IF(A35&lt;=$B$6,$B$5*A35/$B$6,MAX(0,$B$5*(1-(A35-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C35" s="18">
+        <f>IF(OR(A35="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A35&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A35))/$B$10)+$B$12)/((((($B$10*$B$9)-A35))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A35-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A35-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5">
-        <f>IF(A35="","",IF(A35+$B$8&gt;$B$6+$B$7,"",A35+$B$8))</f>
+        <f>IF(A35="","",IF(AND(UPPER($B$3)="CHICAGO",A35&lt;($B$10*$B$9),A35+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A35+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A35+$B$8)))</f>
         <v/>
       </c>
       <c r="B36" s="18">
-        <f>IF(A36="","",IF(A36&lt;=$B$6,$B$5*A36/$B$6,MAX(0,$B$5*(1-(A36-$B$6)/$B$7))))</f>
+        <f>IF(A36="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C36/$B$15),IF(A36&lt;=$B$6,$B$5*A36/$B$6,MAX(0,$B$5*(1-(A36-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C36" s="18">
+        <f>IF(OR(A36="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A36&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A36))/$B$10)+$B$12)/((((($B$10*$B$9)-A36))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A36-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A36-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5">
-        <f>IF(A36="","",IF(A36+$B$8&gt;$B$6+$B$7,"",A36+$B$8))</f>
+        <f>IF(A36="","",IF(AND(UPPER($B$3)="CHICAGO",A36&lt;($B$10*$B$9),A36+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A36+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A36+$B$8)))</f>
         <v/>
       </c>
       <c r="B37" s="18">
-        <f>IF(A37="","",IF(A37&lt;=$B$6,$B$5*A37/$B$6,MAX(0,$B$5*(1-(A37-$B$6)/$B$7))))</f>
+        <f>IF(A37="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C37/$B$15),IF(A37&lt;=$B$6,$B$5*A37/$B$6,MAX(0,$B$5*(1-(A37-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C37" s="18">
+        <f>IF(OR(A37="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A37&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A37))/$B$10)+$B$12)/((((($B$10*$B$9)-A37))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A37-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A37-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5">
-        <f>IF(A37="","",IF(A37+$B$8&gt;$B$6+$B$7,"",A37+$B$8))</f>
+        <f>IF(A37="","",IF(AND(UPPER($B$3)="CHICAGO",A37&lt;($B$10*$B$9),A37+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A37+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A37+$B$8)))</f>
         <v/>
       </c>
       <c r="B38" s="18">
-        <f>IF(A38="","",IF(A38&lt;=$B$6,$B$5*A38/$B$6,MAX(0,$B$5*(1-(A38-$B$6)/$B$7))))</f>
+        <f>IF(A38="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C38/$B$15),IF(A38&lt;=$B$6,$B$5*A38/$B$6,MAX(0,$B$5*(1-(A38-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C38" s="18">
+        <f>IF(OR(A38="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A38&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A38))/$B$10)+$B$12)/((((($B$10*$B$9)-A38))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A38-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A38-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5">
-        <f>IF(A38="","",IF(A38+$B$8&gt;$B$6+$B$7,"",A38+$B$8))</f>
+        <f>IF(A38="","",IF(AND(UPPER($B$3)="CHICAGO",A38&lt;($B$10*$B$9),A38+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A38+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A38+$B$8)))</f>
         <v/>
       </c>
       <c r="B39" s="18">
-        <f>IF(A39="","",IF(A39&lt;=$B$6,$B$5*A39/$B$6,MAX(0,$B$5*(1-(A39-$B$6)/$B$7))))</f>
+        <f>IF(A39="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C39/$B$15),IF(A39&lt;=$B$6,$B$5*A39/$B$6,MAX(0,$B$5*(1-(A39-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C39" s="18">
+        <f>IF(OR(A39="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A39&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A39))/$B$10)+$B$12)/((((($B$10*$B$9)-A39))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A39-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A39-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5">
-        <f>IF(A39="","",IF(A39+$B$8&gt;$B$6+$B$7,"",A39+$B$8))</f>
+        <f>IF(A39="","",IF(AND(UPPER($B$3)="CHICAGO",A39&lt;($B$10*$B$9),A39+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A39+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A39+$B$8)))</f>
         <v/>
       </c>
       <c r="B40" s="18">
-        <f>IF(A40="","",IF(A40&lt;=$B$6,$B$5*A40/$B$6,MAX(0,$B$5*(1-(A40-$B$6)/$B$7))))</f>
+        <f>IF(A40="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C40/$B$15),IF(A40&lt;=$B$6,$B$5*A40/$B$6,MAX(0,$B$5*(1-(A40-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C40" s="18">
+        <f>IF(OR(A40="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A40&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A40))/$B$10)+$B$12)/((((($B$10*$B$9)-A40))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A40-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A40-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5">
-        <f>IF(A40="","",IF(A40+$B$8&gt;$B$6+$B$7,"",A40+$B$8))</f>
+        <f>IF(A40="","",IF(AND(UPPER($B$3)="CHICAGO",A40&lt;($B$10*$B$9),A40+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A40+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A40+$B$8)))</f>
         <v/>
       </c>
       <c r="B41" s="18">
-        <f>IF(A41="","",IF(A41&lt;=$B$6,$B$5*A41/$B$6,MAX(0,$B$5*(1-(A41-$B$6)/$B$7))))</f>
+        <f>IF(A41="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C41/$B$15),IF(A41&lt;=$B$6,$B$5*A41/$B$6,MAX(0,$B$5*(1-(A41-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C41" s="18">
+        <f>IF(OR(A41="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A41&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A41))/$B$10)+$B$12)/((((($B$10*$B$9)-A41))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A41-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A41-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5">
-        <f>IF(A41="","",IF(A41+$B$8&gt;$B$6+$B$7,"",A41+$B$8))</f>
+        <f>IF(A41="","",IF(AND(UPPER($B$3)="CHICAGO",A41&lt;($B$10*$B$9),A41+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A41+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A41+$B$8)))</f>
         <v/>
       </c>
       <c r="B42" s="18">
-        <f>IF(A42="","",IF(A42&lt;=$B$6,$B$5*A42/$B$6,MAX(0,$B$5*(1-(A42-$B$6)/$B$7))))</f>
+        <f>IF(A42="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C42/$B$15),IF(A42&lt;=$B$6,$B$5*A42/$B$6,MAX(0,$B$5*(1-(A42-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C42" s="18">
+        <f>IF(OR(A42="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A42&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A42))/$B$10)+$B$12)/((((($B$10*$B$9)-A42))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A42-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A42-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5">
-        <f>IF(A42="","",IF(A42+$B$8&gt;$B$6+$B$7,"",A42+$B$8))</f>
+        <f>IF(A42="","",IF(AND(UPPER($B$3)="CHICAGO",A42&lt;($B$10*$B$9),A42+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A42+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A42+$B$8)))</f>
         <v/>
       </c>
       <c r="B43" s="18">
-        <f>IF(A43="","",IF(A43&lt;=$B$6,$B$5*A43/$B$6,MAX(0,$B$5*(1-(A43-$B$6)/$B$7))))</f>
+        <f>IF(A43="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C43/$B$15),IF(A43&lt;=$B$6,$B$5*A43/$B$6,MAX(0,$B$5*(1-(A43-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C43" s="18">
+        <f>IF(OR(A43="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A43&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A43))/$B$10)+$B$12)/((((($B$10*$B$9)-A43))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A43-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A43-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5">
-        <f>IF(A43="","",IF(A43+$B$8&gt;$B$6+$B$7,"",A43+$B$8))</f>
+        <f>IF(A43="","",IF(AND(UPPER($B$3)="CHICAGO",A43&lt;($B$10*$B$9),A43+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A43+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A43+$B$8)))</f>
         <v/>
       </c>
       <c r="B44" s="18">
-        <f>IF(A44="","",IF(A44&lt;=$B$6,$B$5*A44/$B$6,MAX(0,$B$5*(1-(A44-$B$6)/$B$7))))</f>
+        <f>IF(A44="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C44/$B$15),IF(A44&lt;=$B$6,$B$5*A44/$B$6,MAX(0,$B$5*(1-(A44-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C44" s="18">
+        <f>IF(OR(A44="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A44&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A44))/$B$10)+$B$12)/((((($B$10*$B$9)-A44))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A44-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A44-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5">
-        <f>IF(A44="","",IF(A44+$B$8&gt;$B$6+$B$7,"",A44+$B$8))</f>
+        <f>IF(A44="","",IF(AND(UPPER($B$3)="CHICAGO",A44&lt;($B$10*$B$9),A44+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A44+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A44+$B$8)))</f>
         <v/>
       </c>
       <c r="B45" s="18">
-        <f>IF(A45="","",IF(A45&lt;=$B$6,$B$5*A45/$B$6,MAX(0,$B$5*(1-(A45-$B$6)/$B$7))))</f>
+        <f>IF(A45="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C45/$B$15),IF(A45&lt;=$B$6,$B$5*A45/$B$6,MAX(0,$B$5*(1-(A45-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C45" s="18">
+        <f>IF(OR(A45="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A45&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A45))/$B$10)+$B$12)/((((($B$10*$B$9)-A45))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A45-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A45-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5">
-        <f>IF(A45="","",IF(A45+$B$8&gt;$B$6+$B$7,"",A45+$B$8))</f>
+        <f>IF(A45="","",IF(AND(UPPER($B$3)="CHICAGO",A45&lt;($B$10*$B$9),A45+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A45+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A45+$B$8)))</f>
         <v/>
       </c>
       <c r="B46" s="18">
-        <f>IF(A46="","",IF(A46&lt;=$B$6,$B$5*A46/$B$6,MAX(0,$B$5*(1-(A46-$B$6)/$B$7))))</f>
+        <f>IF(A46="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C46/$B$15),IF(A46&lt;=$B$6,$B$5*A46/$B$6,MAX(0,$B$5*(1-(A46-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C46" s="18">
+        <f>IF(OR(A46="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A46&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A46))/$B$10)+$B$12)/((((($B$10*$B$9)-A46))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A46-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A46-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5">
-        <f>IF(A46="","",IF(A46+$B$8&gt;$B$6+$B$7,"",A46+$B$8))</f>
+        <f>IF(A46="","",IF(AND(UPPER($B$3)="CHICAGO",A46&lt;($B$10*$B$9),A46+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A46+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A46+$B$8)))</f>
         <v/>
       </c>
       <c r="B47" s="18">
-        <f>IF(A47="","",IF(A47&lt;=$B$6,$B$5*A47/$B$6,MAX(0,$B$5*(1-(A47-$B$6)/$B$7))))</f>
+        <f>IF(A47="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C47/$B$15),IF(A47&lt;=$B$6,$B$5*A47/$B$6,MAX(0,$B$5*(1-(A47-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C47" s="18">
+        <f>IF(OR(A47="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A47&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A47))/$B$10)+$B$12)/((((($B$10*$B$9)-A47))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A47-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A47-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5">
-        <f>IF(A47="","",IF(A47+$B$8&gt;$B$6+$B$7,"",A47+$B$8))</f>
+        <f>IF(A47="","",IF(AND(UPPER($B$3)="CHICAGO",A47&lt;($B$10*$B$9),A47+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A47+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A47+$B$8)))</f>
         <v/>
       </c>
       <c r="B48" s="18">
-        <f>IF(A48="","",IF(A48&lt;=$B$6,$B$5*A48/$B$6,MAX(0,$B$5*(1-(A48-$B$6)/$B$7))))</f>
+        <f>IF(A48="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C48/$B$15),IF(A48&lt;=$B$6,$B$5*A48/$B$6,MAX(0,$B$5*(1-(A48-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C48" s="18">
+        <f>IF(OR(A48="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A48&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A48))/$B$10)+$B$12)/((((($B$10*$B$9)-A48))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A48-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A48-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5">
-        <f>IF(A48="","",IF(A48+$B$8&gt;$B$6+$B$7,"",A48+$B$8))</f>
+        <f>IF(A48="","",IF(AND(UPPER($B$3)="CHICAGO",A48&lt;($B$10*$B$9),A48+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A48+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A48+$B$8)))</f>
         <v/>
       </c>
       <c r="B49" s="18">
-        <f>IF(A49="","",IF(A49&lt;=$B$6,$B$5*A49/$B$6,MAX(0,$B$5*(1-(A49-$B$6)/$B$7))))</f>
+        <f>IF(A49="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C49/$B$15),IF(A49&lt;=$B$6,$B$5*A49/$B$6,MAX(0,$B$5*(1-(A49-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C49" s="18">
+        <f>IF(OR(A49="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A49&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A49))/$B$10)+$B$12)/((((($B$10*$B$9)-A49))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A49-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A49-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5">
-        <f>IF(A49="","",IF(A49+$B$8&gt;$B$6+$B$7,"",A49+$B$8))</f>
+        <f>IF(A49="","",IF(AND(UPPER($B$3)="CHICAGO",A49&lt;($B$10*$B$9),A49+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A49+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A49+$B$8)))</f>
         <v/>
       </c>
       <c r="B50" s="18">
-        <f>IF(A50="","",IF(A50&lt;=$B$6,$B$5*A50/$B$6,MAX(0,$B$5*(1-(A50-$B$6)/$B$7))))</f>
+        <f>IF(A50="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C50/$B$15),IF(A50&lt;=$B$6,$B$5*A50/$B$6,MAX(0,$B$5*(1-(A50-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C50" s="18">
+        <f>IF(OR(A50="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A50&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A50))/$B$10)+$B$12)/((((($B$10*$B$9)-A50))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A50-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A50-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5">
-        <f>IF(A50="","",IF(A50+$B$8&gt;$B$6+$B$7,"",A50+$B$8))</f>
+        <f>IF(A50="","",IF(AND(UPPER($B$3)="CHICAGO",A50&lt;($B$10*$B$9),A50+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A50+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A50+$B$8)))</f>
         <v/>
       </c>
       <c r="B51" s="18">
-        <f>IF(A51="","",IF(A51&lt;=$B$6,$B$5*A51/$B$6,MAX(0,$B$5*(1-(A51-$B$6)/$B$7))))</f>
+        <f>IF(A51="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C51/$B$15),IF(A51&lt;=$B$6,$B$5*A51/$B$6,MAX(0,$B$5*(1-(A51-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C51" s="18">
+        <f>IF(OR(A51="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A51&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A51))/$B$10)+$B$12)/((((($B$10*$B$9)-A51))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A51-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A51-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5">
-        <f>IF(A51="","",IF(A51+$B$8&gt;$B$6+$B$7,"",A51+$B$8))</f>
+        <f>IF(A51="","",IF(AND(UPPER($B$3)="CHICAGO",A51&lt;($B$10*$B$9),A51+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A51+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A51+$B$8)))</f>
         <v/>
       </c>
       <c r="B52" s="18">
-        <f>IF(A52="","",IF(A52&lt;=$B$6,$B$5*A52/$B$6,MAX(0,$B$5*(1-(A52-$B$6)/$B$7))))</f>
+        <f>IF(A52="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C52/$B$15),IF(A52&lt;=$B$6,$B$5*A52/$B$6,MAX(0,$B$5*(1-(A52-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C52" s="18">
+        <f>IF(OR(A52="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A52&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A52))/$B$10)+$B$12)/((((($B$10*$B$9)-A52))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A52-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A52-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5">
-        <f>IF(A52="","",IF(A52+$B$8&gt;$B$6+$B$7,"",A52+$B$8))</f>
+        <f>IF(A52="","",IF(AND(UPPER($B$3)="CHICAGO",A52&lt;($B$10*$B$9),A52+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A52+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A52+$B$8)))</f>
         <v/>
       </c>
       <c r="B53" s="18">
-        <f>IF(A53="","",IF(A53&lt;=$B$6,$B$5*A53/$B$6,MAX(0,$B$5*(1-(A53-$B$6)/$B$7))))</f>
+        <f>IF(A53="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C53/$B$15),IF(A53&lt;=$B$6,$B$5*A53/$B$6,MAX(0,$B$5*(1-(A53-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C53" s="18">
+        <f>IF(OR(A53="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A53&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A53))/$B$10)+$B$12)/((((($B$10*$B$9)-A53))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A53-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A53-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5">
-        <f>IF(A53="","",IF(A53+$B$8&gt;$B$6+$B$7,"",A53+$B$8))</f>
+        <f>IF(A53="","",IF(AND(UPPER($B$3)="CHICAGO",A53&lt;($B$10*$B$9),A53+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A53+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A53+$B$8)))</f>
         <v/>
       </c>
       <c r="B54" s="18">
-        <f>IF(A54="","",IF(A54&lt;=$B$6,$B$5*A54/$B$6,MAX(0,$B$5*(1-(A54-$B$6)/$B$7))))</f>
+        <f>IF(A54="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C54/$B$15),IF(A54&lt;=$B$6,$B$5*A54/$B$6,MAX(0,$B$5*(1-(A54-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C54" s="18">
+        <f>IF(OR(A54="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A54&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A54))/$B$10)+$B$12)/((((($B$10*$B$9)-A54))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A54-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A54-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5">
-        <f>IF(A54="","",IF(A54+$B$8&gt;$B$6+$B$7,"",A54+$B$8))</f>
+        <f>IF(A54="","",IF(AND(UPPER($B$3)="CHICAGO",A54&lt;($B$10*$B$9),A54+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A54+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A54+$B$8)))</f>
         <v/>
       </c>
       <c r="B55" s="18">
-        <f>IF(A55="","",IF(A55&lt;=$B$6,$B$5*A55/$B$6,MAX(0,$B$5*(1-(A55-$B$6)/$B$7))))</f>
+        <f>IF(A55="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C55/$B$15),IF(A55&lt;=$B$6,$B$5*A55/$B$6,MAX(0,$B$5*(1-(A55-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C55" s="18">
+        <f>IF(OR(A55="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A55&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A55))/$B$10)+$B$12)/((((($B$10*$B$9)-A55))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A55-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A55-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5">
-        <f>IF(A55="","",IF(A55+$B$8&gt;$B$6+$B$7,"",A55+$B$8))</f>
+        <f>IF(A55="","",IF(AND(UPPER($B$3)="CHICAGO",A55&lt;($B$10*$B$9),A55+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A55+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A55+$B$8)))</f>
         <v/>
       </c>
       <c r="B56" s="18">
-        <f>IF(A56="","",IF(A56&lt;=$B$6,$B$5*A56/$B$6,MAX(0,$B$5*(1-(A56-$B$6)/$B$7))))</f>
+        <f>IF(A56="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C56/$B$15),IF(A56&lt;=$B$6,$B$5*A56/$B$6,MAX(0,$B$5*(1-(A56-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C56" s="18">
+        <f>IF(OR(A56="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A56&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A56))/$B$10)+$B$12)/((((($B$10*$B$9)-A56))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A56-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A56-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5">
-        <f>IF(A56="","",IF(A56+$B$8&gt;$B$6+$B$7,"",A56+$B$8))</f>
+        <f>IF(A56="","",IF(AND(UPPER($B$3)="CHICAGO",A56&lt;($B$10*$B$9),A56+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A56+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A56+$B$8)))</f>
         <v/>
       </c>
       <c r="B57" s="18">
-        <f>IF(A57="","",IF(A57&lt;=$B$6,$B$5*A57/$B$6,MAX(0,$B$5*(1-(A57-$B$6)/$B$7))))</f>
+        <f>IF(A57="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C57/$B$15),IF(A57&lt;=$B$6,$B$5*A57/$B$6,MAX(0,$B$5*(1-(A57-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C57" s="18">
+        <f>IF(OR(A57="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A57&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A57))/$B$10)+$B$12)/((((($B$10*$B$9)-A57))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A57-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A57-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5">
-        <f>IF(A57="","",IF(A57+$B$8&gt;$B$6+$B$7,"",A57+$B$8))</f>
+        <f>IF(A57="","",IF(AND(UPPER($B$3)="CHICAGO",A57&lt;($B$10*$B$9),A57+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A57+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A57+$B$8)))</f>
         <v/>
       </c>
       <c r="B58" s="18">
-        <f>IF(A58="","",IF(A58&lt;=$B$6,$B$5*A58/$B$6,MAX(0,$B$5*(1-(A58-$B$6)/$B$7))))</f>
+        <f>IF(A58="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C58/$B$15),IF(A58&lt;=$B$6,$B$5*A58/$B$6,MAX(0,$B$5*(1-(A58-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C58" s="18">
+        <f>IF(OR(A58="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A58&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A58))/$B$10)+$B$12)/((((($B$10*$B$9)-A58))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A58-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A58-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5">
-        <f>IF(A58="","",IF(A58+$B$8&gt;$B$6+$B$7,"",A58+$B$8))</f>
+        <f>IF(A58="","",IF(AND(UPPER($B$3)="CHICAGO",A58&lt;($B$10*$B$9),A58+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A58+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A58+$B$8)))</f>
         <v/>
       </c>
       <c r="B59" s="18">
-        <f>IF(A59="","",IF(A59&lt;=$B$6,$B$5*A59/$B$6,MAX(0,$B$5*(1-(A59-$B$6)/$B$7))))</f>
+        <f>IF(A59="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C59/$B$15),IF(A59&lt;=$B$6,$B$5*A59/$B$6,MAX(0,$B$5*(1-(A59-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C59" s="18">
+        <f>IF(OR(A59="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A59&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A59))/$B$10)+$B$12)/((((($B$10*$B$9)-A59))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A59-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A59-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5">
-        <f>IF(A59="","",IF(A59+$B$8&gt;$B$6+$B$7,"",A59+$B$8))</f>
+        <f>IF(A59="","",IF(AND(UPPER($B$3)="CHICAGO",A59&lt;($B$10*$B$9),A59+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A59+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A59+$B$8)))</f>
         <v/>
       </c>
       <c r="B60" s="18">
-        <f>IF(A60="","",IF(A60&lt;=$B$6,$B$5*A60/$B$6,MAX(0,$B$5*(1-(A60-$B$6)/$B$7))))</f>
+        <f>IF(A60="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C60/$B$15),IF(A60&lt;=$B$6,$B$5*A60/$B$6,MAX(0,$B$5*(1-(A60-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C60" s="18">
+        <f>IF(OR(A60="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A60&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A60))/$B$10)+$B$12)/((((($B$10*$B$9)-A60))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A60-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A60-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5">
-        <f>IF(A60="","",IF(A60+$B$8&gt;$B$6+$B$7,"",A60+$B$8))</f>
+        <f>IF(A60="","",IF(AND(UPPER($B$3)="CHICAGO",A60&lt;($B$10*$B$9),A60+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A60+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A60+$B$8)))</f>
         <v/>
       </c>
       <c r="B61" s="18">
-        <f>IF(A61="","",IF(A61&lt;=$B$6,$B$5*A61/$B$6,MAX(0,$B$5*(1-(A61-$B$6)/$B$7))))</f>
+        <f>IF(A61="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C61/$B$15),IF(A61&lt;=$B$6,$B$5*A61/$B$6,MAX(0,$B$5*(1-(A61-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C61" s="18">
+        <f>IF(OR(A61="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A61&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A61))/$B$10)+$B$12)/((((($B$10*$B$9)-A61))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A61-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A61-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5">
-        <f>IF(A61="","",IF(A61+$B$8&gt;$B$6+$B$7,"",A61+$B$8))</f>
+        <f>IF(A61="","",IF(AND(UPPER($B$3)="CHICAGO",A61&lt;($B$10*$B$9),A61+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A61+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A61+$B$8)))</f>
         <v/>
       </c>
       <c r="B62" s="18">
-        <f>IF(A62="","",IF(A62&lt;=$B$6,$B$5*A62/$B$6,MAX(0,$B$5*(1-(A62-$B$6)/$B$7))))</f>
+        <f>IF(A62="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C62/$B$15),IF(A62&lt;=$B$6,$B$5*A62/$B$6,MAX(0,$B$5*(1-(A62-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C62" s="18">
+        <f>IF(OR(A62="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A62&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A62))/$B$10)+$B$12)/((((($B$10*$B$9)-A62))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A62-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A62-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5">
-        <f>IF(A62="","",IF(A62+$B$8&gt;$B$6+$B$7,"",A62+$B$8))</f>
+        <f>IF(A62="","",IF(AND(UPPER($B$3)="CHICAGO",A62&lt;($B$10*$B$9),A62+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A62+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A62+$B$8)))</f>
         <v/>
       </c>
       <c r="B63" s="18">
-        <f>IF(A63="","",IF(A63&lt;=$B$6,$B$5*A63/$B$6,MAX(0,$B$5*(1-(A63-$B$6)/$B$7))))</f>
+        <f>IF(A63="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C63/$B$15),IF(A63&lt;=$B$6,$B$5*A63/$B$6,MAX(0,$B$5*(1-(A63-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C63" s="18">
+        <f>IF(OR(A63="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A63&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A63))/$B$10)+$B$12)/((((($B$10*$B$9)-A63))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A63-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A63-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5">
-        <f>IF(A63="","",IF(A63+$B$8&gt;$B$6+$B$7,"",A63+$B$8))</f>
+        <f>IF(A63="","",IF(AND(UPPER($B$3)="CHICAGO",A63&lt;($B$10*$B$9),A63+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A63+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A63+$B$8)))</f>
         <v/>
       </c>
       <c r="B64" s="18">
-        <f>IF(A64="","",IF(A64&lt;=$B$6,$B$5*A64/$B$6,MAX(0,$B$5*(1-(A64-$B$6)/$B$7))))</f>
+        <f>IF(A64="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C64/$B$15),IF(A64&lt;=$B$6,$B$5*A64/$B$6,MAX(0,$B$5*(1-(A64-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C64" s="18">
+        <f>IF(OR(A64="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A64&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A64))/$B$10)+$B$12)/((((($B$10*$B$9)-A64))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A64-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A64-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5">
-        <f>IF(A64="","",IF(A64+$B$8&gt;$B$6+$B$7,"",A64+$B$8))</f>
+        <f>IF(A64="","",IF(AND(UPPER($B$3)="CHICAGO",A64&lt;($B$10*$B$9),A64+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A64+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A64+$B$8)))</f>
         <v/>
       </c>
       <c r="B65" s="18">
-        <f>IF(A65="","",IF(A65&lt;=$B$6,$B$5*A65/$B$6,MAX(0,$B$5*(1-(A65-$B$6)/$B$7))))</f>
+        <f>IF(A65="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C65/$B$15),IF(A65&lt;=$B$6,$B$5*A65/$B$6,MAX(0,$B$5*(1-(A65-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C65" s="18">
+        <f>IF(OR(A65="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A65&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A65))/$B$10)+$B$12)/((((($B$10*$B$9)-A65))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A65-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A65-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5">
-        <f>IF(A65="","",IF(A65+$B$8&gt;$B$6+$B$7,"",A65+$B$8))</f>
+        <f>IF(A65="","",IF(AND(UPPER($B$3)="CHICAGO",A65&lt;($B$10*$B$9),A65+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A65+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A65+$B$8)))</f>
         <v/>
       </c>
       <c r="B66" s="18">
-        <f>IF(A66="","",IF(A66&lt;=$B$6,$B$5*A66/$B$6,MAX(0,$B$5*(1-(A66-$B$6)/$B$7))))</f>
+        <f>IF(A66="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C66/$B$15),IF(A66&lt;=$B$6,$B$5*A66/$B$6,MAX(0,$B$5*(1-(A66-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C66" s="18">
+        <f>IF(OR(A66="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A66&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A66))/$B$10)+$B$12)/((((($B$10*$B$9)-A66))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A66-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A66-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5">
-        <f>IF(A66="","",IF(A66+$B$8&gt;$B$6+$B$7,"",A66+$B$8))</f>
+        <f>IF(A66="","",IF(AND(UPPER($B$3)="CHICAGO",A66&lt;($B$10*$B$9),A66+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A66+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A66+$B$8)))</f>
         <v/>
       </c>
       <c r="B67" s="18">
-        <f>IF(A67="","",IF(A67&lt;=$B$6,$B$5*A67/$B$6,MAX(0,$B$5*(1-(A67-$B$6)/$B$7))))</f>
+        <f>IF(A67="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C67/$B$15),IF(A67&lt;=$B$6,$B$5*A67/$B$6,MAX(0,$B$5*(1-(A67-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C67" s="18">
+        <f>IF(OR(A67="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A67&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A67))/$B$10)+$B$12)/((((($B$10*$B$9)-A67))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A67-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A67-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5">
-        <f>IF(A67="","",IF(A67+$B$8&gt;$B$6+$B$7,"",A67+$B$8))</f>
+        <f>IF(A67="","",IF(AND(UPPER($B$3)="CHICAGO",A67&lt;($B$10*$B$9),A67+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A67+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A67+$B$8)))</f>
         <v/>
       </c>
       <c r="B68" s="18">
-        <f>IF(A68="","",IF(A68&lt;=$B$6,$B$5*A68/$B$6,MAX(0,$B$5*(1-(A68-$B$6)/$B$7))))</f>
+        <f>IF(A68="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C68/$B$15),IF(A68&lt;=$B$6,$B$5*A68/$B$6,MAX(0,$B$5*(1-(A68-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C68" s="18">
+        <f>IF(OR(A68="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A68&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A68))/$B$10)+$B$12)/((((($B$10*$B$9)-A68))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A68-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A68-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5">
-        <f>IF(A68="","",IF(A68+$B$8&gt;$B$6+$B$7,"",A68+$B$8))</f>
+        <f>IF(A68="","",IF(AND(UPPER($B$3)="CHICAGO",A68&lt;($B$10*$B$9),A68+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A68+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A68+$B$8)))</f>
         <v/>
       </c>
       <c r="B69" s="18">
-        <f>IF(A69="","",IF(A69&lt;=$B$6,$B$5*A69/$B$6,MAX(0,$B$5*(1-(A69-$B$6)/$B$7))))</f>
+        <f>IF(A69="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C69/$B$15),IF(A69&lt;=$B$6,$B$5*A69/$B$6,MAX(0,$B$5*(1-(A69-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C69" s="18">
+        <f>IF(OR(A69="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A69&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A69))/$B$10)+$B$12)/((((($B$10*$B$9)-A69))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A69-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A69-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5">
-        <f>IF(A69="","",IF(A69+$B$8&gt;$B$6+$B$7,"",A69+$B$8))</f>
+        <f>IF(A69="","",IF(AND(UPPER($B$3)="CHICAGO",A69&lt;($B$10*$B$9),A69+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A69+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A69+$B$8)))</f>
         <v/>
       </c>
       <c r="B70" s="18">
-        <f>IF(A70="","",IF(A70&lt;=$B$6,$B$5*A70/$B$6,MAX(0,$B$5*(1-(A70-$B$6)/$B$7))))</f>
+        <f>IF(A70="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C70/$B$15),IF(A70&lt;=$B$6,$B$5*A70/$B$6,MAX(0,$B$5*(1-(A70-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C70" s="18">
+        <f>IF(OR(A70="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A70&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A70))/$B$10)+$B$12)/((((($B$10*$B$9)-A70))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A70-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A70-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5">
-        <f>IF(A70="","",IF(A70+$B$8&gt;$B$6+$B$7,"",A70+$B$8))</f>
+        <f>IF(A70="","",IF(AND(UPPER($B$3)="CHICAGO",A70&lt;($B$10*$B$9),A70+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A70+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A70+$B$8)))</f>
         <v/>
       </c>
       <c r="B71" s="18">
-        <f>IF(A71="","",IF(A71&lt;=$B$6,$B$5*A71/$B$6,MAX(0,$B$5*(1-(A71-$B$6)/$B$7))))</f>
+        <f>IF(A71="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C71/$B$15),IF(A71&lt;=$B$6,$B$5*A71/$B$6,MAX(0,$B$5*(1-(A71-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C71" s="18">
+        <f>IF(OR(A71="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A71&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A71))/$B$10)+$B$12)/((((($B$10*$B$9)-A71))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A71-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A71-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5">
-        <f>IF(A71="","",IF(A71+$B$8&gt;$B$6+$B$7,"",A71+$B$8))</f>
+        <f>IF(A71="","",IF(AND(UPPER($B$3)="CHICAGO",A71&lt;($B$10*$B$9),A71+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A71+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A71+$B$8)))</f>
         <v/>
       </c>
       <c r="B72" s="18">
-        <f>IF(A72="","",IF(A72&lt;=$B$6,$B$5*A72/$B$6,MAX(0,$B$5*(1-(A72-$B$6)/$B$7))))</f>
+        <f>IF(A72="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C72/$B$15),IF(A72&lt;=$B$6,$B$5*A72/$B$6,MAX(0,$B$5*(1-(A72-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C72" s="18">
+        <f>IF(OR(A72="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A72&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A72))/$B$10)+$B$12)/((((($B$10*$B$9)-A72))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A72-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A72-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5">
-        <f>IF(A72="","",IF(A72+$B$8&gt;$B$6+$B$7,"",A72+$B$8))</f>
+        <f>IF(A72="","",IF(AND(UPPER($B$3)="CHICAGO",A72&lt;($B$10*$B$9),A72+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A72+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A72+$B$8)))</f>
         <v/>
       </c>
       <c r="B73" s="18">
-        <f>IF(A73="","",IF(A73&lt;=$B$6,$B$5*A73/$B$6,MAX(0,$B$5*(1-(A73-$B$6)/$B$7))))</f>
+        <f>IF(A73="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C73/$B$15),IF(A73&lt;=$B$6,$B$5*A73/$B$6,MAX(0,$B$5*(1-(A73-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C73" s="18">
+        <f>IF(OR(A73="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A73&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A73))/$B$10)+$B$12)/((((($B$10*$B$9)-A73))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A73-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A73-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5">
-        <f>IF(A73="","",IF(A73+$B$8&gt;$B$6+$B$7,"",A73+$B$8))</f>
+        <f>IF(A73="","",IF(AND(UPPER($B$3)="CHICAGO",A73&lt;($B$10*$B$9),A73+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A73+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A73+$B$8)))</f>
         <v/>
       </c>
       <c r="B74" s="18">
-        <f>IF(A74="","",IF(A74&lt;=$B$6,$B$5*A74/$B$6,MAX(0,$B$5*(1-(A74-$B$6)/$B$7))))</f>
+        <f>IF(A74="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C74/$B$15),IF(A74&lt;=$B$6,$B$5*A74/$B$6,MAX(0,$B$5*(1-(A74-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C74" s="18">
+        <f>IF(OR(A74="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A74&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A74))/$B$10)+$B$12)/((((($B$10*$B$9)-A74))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A74-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A74-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5">
-        <f>IF(A74="","",IF(A74+$B$8&gt;$B$6+$B$7,"",A74+$B$8))</f>
+        <f>IF(A74="","",IF(AND(UPPER($B$3)="CHICAGO",A74&lt;($B$10*$B$9),A74+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A74+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A74+$B$8)))</f>
         <v/>
       </c>
       <c r="B75" s="18">
-        <f>IF(A75="","",IF(A75&lt;=$B$6,$B$5*A75/$B$6,MAX(0,$B$5*(1-(A75-$B$6)/$B$7))))</f>
+        <f>IF(A75="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C75/$B$15),IF(A75&lt;=$B$6,$B$5*A75/$B$6,MAX(0,$B$5*(1-(A75-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C75" s="18">
+        <f>IF(OR(A75="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A75&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A75))/$B$10)+$B$12)/((((($B$10*$B$9)-A75))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A75-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A75-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5">
-        <f>IF(A75="","",IF(A75+$B$8&gt;$B$6+$B$7,"",A75+$B$8))</f>
+        <f>IF(A75="","",IF(AND(UPPER($B$3)="CHICAGO",A75&lt;($B$10*$B$9),A75+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A75+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A75+$B$8)))</f>
         <v/>
       </c>
       <c r="B76" s="18">
-        <f>IF(A76="","",IF(A76&lt;=$B$6,$B$5*A76/$B$6,MAX(0,$B$5*(1-(A76-$B$6)/$B$7))))</f>
+        <f>IF(A76="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C76/$B$15),IF(A76&lt;=$B$6,$B$5*A76/$B$6,MAX(0,$B$5*(1-(A76-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C76" s="18">
+        <f>IF(OR(A76="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A76&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A76))/$B$10)+$B$12)/((((($B$10*$B$9)-A76))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A76-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A76-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5">
-        <f>IF(A76="","",IF(A76+$B$8&gt;$B$6+$B$7,"",A76+$B$8))</f>
+        <f>IF(A76="","",IF(AND(UPPER($B$3)="CHICAGO",A76&lt;($B$10*$B$9),A76+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A76+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A76+$B$8)))</f>
         <v/>
       </c>
       <c r="B77" s="18">
-        <f>IF(A77="","",IF(A77&lt;=$B$6,$B$5*A77/$B$6,MAX(0,$B$5*(1-(A77-$B$6)/$B$7))))</f>
+        <f>IF(A77="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C77/$B$15),IF(A77&lt;=$B$6,$B$5*A77/$B$6,MAX(0,$B$5*(1-(A77-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C77" s="18">
+        <f>IF(OR(A77="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A77&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A77))/$B$10)+$B$12)/((((($B$10*$B$9)-A77))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A77-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A77-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5">
-        <f>IF(A77="","",IF(A77+$B$8&gt;$B$6+$B$7,"",A77+$B$8))</f>
+        <f>IF(A77="","",IF(AND(UPPER($B$3)="CHICAGO",A77&lt;($B$10*$B$9),A77+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A77+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A77+$B$8)))</f>
         <v/>
       </c>
       <c r="B78" s="18">
-        <f>IF(A78="","",IF(A78&lt;=$B$6,$B$5*A78/$B$6,MAX(0,$B$5*(1-(A78-$B$6)/$B$7))))</f>
+        <f>IF(A78="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C78/$B$15),IF(A78&lt;=$B$6,$B$5*A78/$B$6,MAX(0,$B$5*(1-(A78-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C78" s="18">
+        <f>IF(OR(A78="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A78&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A78))/$B$10)+$B$12)/((((($B$10*$B$9)-A78))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A78-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A78-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5">
-        <f>IF(A78="","",IF(A78+$B$8&gt;$B$6+$B$7,"",A78+$B$8))</f>
+        <f>IF(A78="","",IF(AND(UPPER($B$3)="CHICAGO",A78&lt;($B$10*$B$9),A78+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A78+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A78+$B$8)))</f>
         <v/>
       </c>
       <c r="B79" s="18">
-        <f>IF(A79="","",IF(A79&lt;=$B$6,$B$5*A79/$B$6,MAX(0,$B$5*(1-(A79-$B$6)/$B$7))))</f>
+        <f>IF(A79="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C79/$B$15),IF(A79&lt;=$B$6,$B$5*A79/$B$6,MAX(0,$B$5*(1-(A79-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C79" s="18">
+        <f>IF(OR(A79="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A79&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A79))/$B$10)+$B$12)/((((($B$10*$B$9)-A79))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A79-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A79-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5">
-        <f>IF(A79="","",IF(A79+$B$8&gt;$B$6+$B$7,"",A79+$B$8))</f>
+        <f>IF(A79="","",IF(AND(UPPER($B$3)="CHICAGO",A79&lt;($B$10*$B$9),A79+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A79+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A79+$B$8)))</f>
         <v/>
       </c>
       <c r="B80" s="18">
-        <f>IF(A80="","",IF(A80&lt;=$B$6,$B$5*A80/$B$6,MAX(0,$B$5*(1-(A80-$B$6)/$B$7))))</f>
+        <f>IF(A80="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C80/$B$15),IF(A80&lt;=$B$6,$B$5*A80/$B$6,MAX(0,$B$5*(1-(A80-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C80" s="18">
+        <f>IF(OR(A80="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A80&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A80))/$B$10)+$B$12)/((((($B$10*$B$9)-A80))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A80-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A80-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5">
-        <f>IF(A80="","",IF(A80+$B$8&gt;$B$6+$B$7,"",A80+$B$8))</f>
+        <f>IF(A80="","",IF(AND(UPPER($B$3)="CHICAGO",A80&lt;($B$10*$B$9),A80+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A80+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A80+$B$8)))</f>
         <v/>
       </c>
       <c r="B81" s="18">
-        <f>IF(A81="","",IF(A81&lt;=$B$6,$B$5*A81/$B$6,MAX(0,$B$5*(1-(A81-$B$6)/$B$7))))</f>
+        <f>IF(A81="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C81/$B$15),IF(A81&lt;=$B$6,$B$5*A81/$B$6,MAX(0,$B$5*(1-(A81-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C81" s="18">
+        <f>IF(OR(A81="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A81&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A81))/$B$10)+$B$12)/((((($B$10*$B$9)-A81))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A81-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A81-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5">
-        <f>IF(A81="","",IF(A81+$B$8&gt;$B$6+$B$7,"",A81+$B$8))</f>
+        <f>IF(A81="","",IF(AND(UPPER($B$3)="CHICAGO",A81&lt;($B$10*$B$9),A81+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A81+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A81+$B$8)))</f>
         <v/>
       </c>
       <c r="B82" s="18">
-        <f>IF(A82="","",IF(A82&lt;=$B$6,$B$5*A82/$B$6,MAX(0,$B$5*(1-(A82-$B$6)/$B$7))))</f>
+        <f>IF(A82="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C82/$B$15),IF(A82&lt;=$B$6,$B$5*A82/$B$6,MAX(0,$B$5*(1-(A82-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C82" s="18">
+        <f>IF(OR(A82="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A82&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A82))/$B$10)+$B$12)/((((($B$10*$B$9)-A82))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A82-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A82-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5">
-        <f>IF(A82="","",IF(A82+$B$8&gt;$B$6+$B$7,"",A82+$B$8))</f>
+        <f>IF(A82="","",IF(AND(UPPER($B$3)="CHICAGO",A82&lt;($B$10*$B$9),A82+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A82+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A82+$B$8)))</f>
         <v/>
       </c>
       <c r="B83" s="18">
-        <f>IF(A83="","",IF(A83&lt;=$B$6,$B$5*A83/$B$6,MAX(0,$B$5*(1-(A83-$B$6)/$B$7))))</f>
+        <f>IF(A83="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C83/$B$15),IF(A83&lt;=$B$6,$B$5*A83/$B$6,MAX(0,$B$5*(1-(A83-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C83" s="18">
+        <f>IF(OR(A83="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A83&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A83))/$B$10)+$B$12)/((((($B$10*$B$9)-A83))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A83-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A83-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5">
-        <f>IF(A83="","",IF(A83+$B$8&gt;$B$6+$B$7,"",A83+$B$8))</f>
+        <f>IF(A83="","",IF(AND(UPPER($B$3)="CHICAGO",A83&lt;($B$10*$B$9),A83+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A83+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A83+$B$8)))</f>
         <v/>
       </c>
       <c r="B84" s="18">
-        <f>IF(A84="","",IF(A84&lt;=$B$6,$B$5*A84/$B$6,MAX(0,$B$5*(1-(A84-$B$6)/$B$7))))</f>
+        <f>IF(A84="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C84/$B$15),IF(A84&lt;=$B$6,$B$5*A84/$B$6,MAX(0,$B$5*(1-(A84-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C84" s="18">
+        <f>IF(OR(A84="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A84&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A84))/$B$10)+$B$12)/((((($B$10*$B$9)-A84))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A84-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A84-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5">
-        <f>IF(A84="","",IF(A84+$B$8&gt;$B$6+$B$7,"",A84+$B$8))</f>
+        <f>IF(A84="","",IF(AND(UPPER($B$3)="CHICAGO",A84&lt;($B$10*$B$9),A84+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A84+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A84+$B$8)))</f>
         <v/>
       </c>
       <c r="B85" s="18">
-        <f>IF(A85="","",IF(A85&lt;=$B$6,$B$5*A85/$B$6,MAX(0,$B$5*(1-(A85-$B$6)/$B$7))))</f>
+        <f>IF(A85="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C85/$B$15),IF(A85&lt;=$B$6,$B$5*A85/$B$6,MAX(0,$B$5*(1-(A85-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C85" s="18">
+        <f>IF(OR(A85="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A85&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A85))/$B$10)+$B$12)/((((($B$10*$B$9)-A85))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A85-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A85-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5">
-        <f>IF(A85="","",IF(A85+$B$8&gt;$B$6+$B$7,"",A85+$B$8))</f>
+        <f>IF(A85="","",IF(AND(UPPER($B$3)="CHICAGO",A85&lt;($B$10*$B$9),A85+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A85+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A85+$B$8)))</f>
         <v/>
       </c>
       <c r="B86" s="18">
-        <f>IF(A86="","",IF(A86&lt;=$B$6,$B$5*A86/$B$6,MAX(0,$B$5*(1-(A86-$B$6)/$B$7))))</f>
+        <f>IF(A86="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C86/$B$15),IF(A86&lt;=$B$6,$B$5*A86/$B$6,MAX(0,$B$5*(1-(A86-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C86" s="18">
+        <f>IF(OR(A86="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A86&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A86))/$B$10)+$B$12)/((((($B$10*$B$9)-A86))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A86-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A86-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5">
-        <f>IF(A86="","",IF(A86+$B$8&gt;$B$6+$B$7,"",A86+$B$8))</f>
+        <f>IF(A86="","",IF(AND(UPPER($B$3)="CHICAGO",A86&lt;($B$10*$B$9),A86+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A86+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A86+$B$8)))</f>
         <v/>
       </c>
       <c r="B87" s="18">
-        <f>IF(A87="","",IF(A87&lt;=$B$6,$B$5*A87/$B$6,MAX(0,$B$5*(1-(A87-$B$6)/$B$7))))</f>
+        <f>IF(A87="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C87/$B$15),IF(A87&lt;=$B$6,$B$5*A87/$B$6,MAX(0,$B$5*(1-(A87-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C87" s="18">
+        <f>IF(OR(A87="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A87&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A87))/$B$10)+$B$12)/((((($B$10*$B$9)-A87))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A87-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A87-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5">
-        <f>IF(A87="","",IF(A87+$B$8&gt;$B$6+$B$7,"",A87+$B$8))</f>
+        <f>IF(A87="","",IF(AND(UPPER($B$3)="CHICAGO",A87&lt;($B$10*$B$9),A87+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A87+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A87+$B$8)))</f>
         <v/>
       </c>
       <c r="B88" s="18">
-        <f>IF(A88="","",IF(A88&lt;=$B$6,$B$5*A88/$B$6,MAX(0,$B$5*(1-(A88-$B$6)/$B$7))))</f>
+        <f>IF(A88="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C88/$B$15),IF(A88&lt;=$B$6,$B$5*A88/$B$6,MAX(0,$B$5*(1-(A88-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C88" s="18">
+        <f>IF(OR(A88="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A88&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A88))/$B$10)+$B$12)/((((($B$10*$B$9)-A88))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A88-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A88-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5">
-        <f>IF(A88="","",IF(A88+$B$8&gt;$B$6+$B$7,"",A88+$B$8))</f>
+        <f>IF(A88="","",IF(AND(UPPER($B$3)="CHICAGO",A88&lt;($B$10*$B$9),A88+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A88+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A88+$B$8)))</f>
         <v/>
       </c>
       <c r="B89" s="18">
-        <f>IF(A89="","",IF(A89&lt;=$B$6,$B$5*A89/$B$6,MAX(0,$B$5*(1-(A89-$B$6)/$B$7))))</f>
+        <f>IF(A89="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C89/$B$15),IF(A89&lt;=$B$6,$B$5*A89/$B$6,MAX(0,$B$5*(1-(A89-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C89" s="18">
+        <f>IF(OR(A89="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A89&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A89))/$B$10)+$B$12)/((((($B$10*$B$9)-A89))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A89-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A89-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5">
-        <f>IF(A89="","",IF(A89+$B$8&gt;$B$6+$B$7,"",A89+$B$8))</f>
+        <f>IF(A89="","",IF(AND(UPPER($B$3)="CHICAGO",A89&lt;($B$10*$B$9),A89+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A89+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A89+$B$8)))</f>
         <v/>
       </c>
       <c r="B90" s="18">
-        <f>IF(A90="","",IF(A90&lt;=$B$6,$B$5*A90/$B$6,MAX(0,$B$5*(1-(A90-$B$6)/$B$7))))</f>
+        <f>IF(A90="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C90/$B$15),IF(A90&lt;=$B$6,$B$5*A90/$B$6,MAX(0,$B$5*(1-(A90-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C90" s="18">
+        <f>IF(OR(A90="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A90&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A90))/$B$10)+$B$12)/((((($B$10*$B$9)-A90))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A90-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A90-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5">
-        <f>IF(A90="","",IF(A90+$B$8&gt;$B$6+$B$7,"",A90+$B$8))</f>
+        <f>IF(A90="","",IF(AND(UPPER($B$3)="CHICAGO",A90&lt;($B$10*$B$9),A90+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A90+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A90+$B$8)))</f>
         <v/>
       </c>
       <c r="B91" s="18">
-        <f>IF(A91="","",IF(A91&lt;=$B$6,$B$5*A91/$B$6,MAX(0,$B$5*(1-(A91-$B$6)/$B$7))))</f>
+        <f>IF(A91="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C91/$B$15),IF(A91&lt;=$B$6,$B$5*A91/$B$6,MAX(0,$B$5*(1-(A91-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C91" s="18">
+        <f>IF(OR(A91="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A91&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A91))/$B$10)+$B$12)/((((($B$10*$B$9)-A91))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A91-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A91-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5">
-        <f>IF(A91="","",IF(A91+$B$8&gt;$B$6+$B$7,"",A91+$B$8))</f>
+        <f>IF(A91="","",IF(AND(UPPER($B$3)="CHICAGO",A91&lt;($B$10*$B$9),A91+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A91+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A91+$B$8)))</f>
         <v/>
       </c>
       <c r="B92" s="18">
-        <f>IF(A92="","",IF(A92&lt;=$B$6,$B$5*A92/$B$6,MAX(0,$B$5*(1-(A92-$B$6)/$B$7))))</f>
+        <f>IF(A92="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C92/$B$15),IF(A92&lt;=$B$6,$B$5*A92/$B$6,MAX(0,$B$5*(1-(A92-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C92" s="18">
+        <f>IF(OR(A92="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A92&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A92))/$B$10)+$B$12)/((((($B$10*$B$9)-A92))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A92-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A92-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5">
-        <f>IF(A92="","",IF(A92+$B$8&gt;$B$6+$B$7,"",A92+$B$8))</f>
+        <f>IF(A92="","",IF(AND(UPPER($B$3)="CHICAGO",A92&lt;($B$10*$B$9),A92+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A92+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A92+$B$8)))</f>
         <v/>
       </c>
       <c r="B93" s="18">
-        <f>IF(A93="","",IF(A93&lt;=$B$6,$B$5*A93/$B$6,MAX(0,$B$5*(1-(A93-$B$6)/$B$7))))</f>
+        <f>IF(A93="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C93/$B$15),IF(A93&lt;=$B$6,$B$5*A93/$B$6,MAX(0,$B$5*(1-(A93-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C93" s="18">
+        <f>IF(OR(A93="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A93&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A93))/$B$10)+$B$12)/((((($B$10*$B$9)-A93))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A93-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A93-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5">
-        <f>IF(A93="","",IF(A93+$B$8&gt;$B$6+$B$7,"",A93+$B$8))</f>
+        <f>IF(A93="","",IF(AND(UPPER($B$3)="CHICAGO",A93&lt;($B$10*$B$9),A93+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A93+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A93+$B$8)))</f>
         <v/>
       </c>
       <c r="B94" s="18">
-        <f>IF(A94="","",IF(A94&lt;=$B$6,$B$5*A94/$B$6,MAX(0,$B$5*(1-(A94-$B$6)/$B$7))))</f>
+        <f>IF(A94="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C94/$B$15),IF(A94&lt;=$B$6,$B$5*A94/$B$6,MAX(0,$B$5*(1-(A94-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C94" s="18">
+        <f>IF(OR(A94="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A94&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A94))/$B$10)+$B$12)/((((($B$10*$B$9)-A94))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A94-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A94-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5">
-        <f>IF(A94="","",IF(A94+$B$8&gt;$B$6+$B$7,"",A94+$B$8))</f>
+        <f>IF(A94="","",IF(AND(UPPER($B$3)="CHICAGO",A94&lt;($B$10*$B$9),A94+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A94+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A94+$B$8)))</f>
         <v/>
       </c>
       <c r="B95" s="18">
-        <f>IF(A95="","",IF(A95&lt;=$B$6,$B$5*A95/$B$6,MAX(0,$B$5*(1-(A95-$B$6)/$B$7))))</f>
+        <f>IF(A95="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C95/$B$15),IF(A95&lt;=$B$6,$B$5*A95/$B$6,MAX(0,$B$5*(1-(A95-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C95" s="18">
+        <f>IF(OR(A95="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A95&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A95))/$B$10)+$B$12)/((((($B$10*$B$9)-A95))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A95-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A95-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5">
-        <f>IF(A95="","",IF(A95+$B$8&gt;$B$6+$B$7,"",A95+$B$8))</f>
+        <f>IF(A95="","",IF(AND(UPPER($B$3)="CHICAGO",A95&lt;($B$10*$B$9),A95+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A95+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A95+$B$8)))</f>
         <v/>
       </c>
       <c r="B96" s="18">
-        <f>IF(A96="","",IF(A96&lt;=$B$6,$B$5*A96/$B$6,MAX(0,$B$5*(1-(A96-$B$6)/$B$7))))</f>
+        <f>IF(A96="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C96/$B$15),IF(A96&lt;=$B$6,$B$5*A96/$B$6,MAX(0,$B$5*(1-(A96-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C96" s="18">
+        <f>IF(OR(A96="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A96&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A96))/$B$10)+$B$12)/((((($B$10*$B$9)-A96))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A96-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A96-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5">
-        <f>IF(A96="","",IF(A96+$B$8&gt;$B$6+$B$7,"",A96+$B$8))</f>
+        <f>IF(A96="","",IF(AND(UPPER($B$3)="CHICAGO",A96&lt;($B$10*$B$9),A96+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A96+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A96+$B$8)))</f>
         <v/>
       </c>
       <c r="B97" s="18">
-        <f>IF(A97="","",IF(A97&lt;=$B$6,$B$5*A97/$B$6,MAX(0,$B$5*(1-(A97-$B$6)/$B$7))))</f>
+        <f>IF(A97="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C97/$B$15),IF(A97&lt;=$B$6,$B$5*A97/$B$6,MAX(0,$B$5*(1-(A97-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C97" s="18">
+        <f>IF(OR(A97="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A97&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A97))/$B$10)+$B$12)/((((($B$10*$B$9)-A97))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A97-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A97-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5">
-        <f>IF(A97="","",IF(A97+$B$8&gt;$B$6+$B$7,"",A97+$B$8))</f>
+        <f>IF(A97="","",IF(AND(UPPER($B$3)="CHICAGO",A97&lt;($B$10*$B$9),A97+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A97+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A97+$B$8)))</f>
         <v/>
       </c>
       <c r="B98" s="18">
-        <f>IF(A98="","",IF(A98&lt;=$B$6,$B$5*A98/$B$6,MAX(0,$B$5*(1-(A98-$B$6)/$B$7))))</f>
+        <f>IF(A98="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C98/$B$15),IF(A98&lt;=$B$6,$B$5*A98/$B$6,MAX(0,$B$5*(1-(A98-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C98" s="18">
+        <f>IF(OR(A98="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A98&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A98))/$B$10)+$B$12)/((((($B$10*$B$9)-A98))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A98-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A98-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5">
-        <f>IF(A98="","",IF(A98+$B$8&gt;$B$6+$B$7,"",A98+$B$8))</f>
+        <f>IF(A98="","",IF(AND(UPPER($B$3)="CHICAGO",A98&lt;($B$10*$B$9),A98+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A98+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A98+$B$8)))</f>
         <v/>
       </c>
       <c r="B99" s="18">
-        <f>IF(A99="","",IF(A99&lt;=$B$6,$B$5*A99/$B$6,MAX(0,$B$5*(1-(A99-$B$6)/$B$7))))</f>
+        <f>IF(A99="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C99/$B$15),IF(A99&lt;=$B$6,$B$5*A99/$B$6,MAX(0,$B$5*(1-(A99-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C99" s="18">
+        <f>IF(OR(A99="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A99&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A99))/$B$10)+$B$12)/((((($B$10*$B$9)-A99))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A99-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A99-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5">
-        <f>IF(A99="","",IF(A99+$B$8&gt;$B$6+$B$7,"",A99+$B$8))</f>
+        <f>IF(A99="","",IF(AND(UPPER($B$3)="CHICAGO",A99&lt;($B$10*$B$9),A99+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A99+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A99+$B$8)))</f>
         <v/>
       </c>
       <c r="B100" s="18">
-        <f>IF(A100="","",IF(A100&lt;=$B$6,$B$5*A100/$B$6,MAX(0,$B$5*(1-(A100-$B$6)/$B$7))))</f>
+        <f>IF(A100="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C100/$B$15),IF(A100&lt;=$B$6,$B$5*A100/$B$6,MAX(0,$B$5*(1-(A100-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C100" s="18">
+        <f>IF(OR(A100="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A100&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A100))/$B$10)+$B$12)/((((($B$10*$B$9)-A100))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A100-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A100-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5">
-        <f>IF(A100="","",IF(A100+$B$8&gt;$B$6+$B$7,"",A100+$B$8))</f>
+        <f>IF(A100="","",IF(AND(UPPER($B$3)="CHICAGO",A100&lt;($B$10*$B$9),A100+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A100+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A100+$B$8)))</f>
         <v/>
       </c>
       <c r="B101" s="18">
-        <f>IF(A101="","",IF(A101&lt;=$B$6,$B$5*A101/$B$6,MAX(0,$B$5*(1-(A101-$B$6)/$B$7))))</f>
+        <f>IF(A101="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C101/$B$15),IF(A101&lt;=$B$6,$B$5*A101/$B$6,MAX(0,$B$5*(1-(A101-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C101" s="18">
+        <f>IF(OR(A101="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A101&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A101))/$B$10)+$B$12)/((((($B$10*$B$9)-A101))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A101-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A101-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5">
-        <f>IF(A101="","",IF(A101+$B$8&gt;$B$6+$B$7,"",A101+$B$8))</f>
+        <f>IF(A101="","",IF(AND(UPPER($B$3)="CHICAGO",A101&lt;($B$10*$B$9),A101+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A101+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A101+$B$8)))</f>
         <v/>
       </c>
       <c r="B102" s="18">
-        <f>IF(A102="","",IF(A102&lt;=$B$6,$B$5*A102/$B$6,MAX(0,$B$5*(1-(A102-$B$6)/$B$7))))</f>
+        <f>IF(A102="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C102/$B$15),IF(A102&lt;=$B$6,$B$5*A102/$B$6,MAX(0,$B$5*(1-(A102-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C102" s="18">
+        <f>IF(OR(A102="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A102&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A102))/$B$10)+$B$12)/((((($B$10*$B$9)-A102))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A102-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A102-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5">
-        <f>IF(A102="","",IF(A102+$B$8&gt;$B$6+$B$7,"",A102+$B$8))</f>
+        <f>IF(A102="","",IF(AND(UPPER($B$3)="CHICAGO",A102&lt;($B$10*$B$9),A102+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A102+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A102+$B$8)))</f>
         <v/>
       </c>
       <c r="B103" s="18">
-        <f>IF(A103="","",IF(A103&lt;=$B$6,$B$5*A103/$B$6,MAX(0,$B$5*(1-(A103-$B$6)/$B$7))))</f>
+        <f>IF(A103="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C103/$B$15),IF(A103&lt;=$B$6,$B$5*A103/$B$6,MAX(0,$B$5*(1-(A103-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C103" s="18">
+        <f>IF(OR(A103="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A103&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A103))/$B$10)+$B$12)/((((($B$10*$B$9)-A103))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A103-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A103-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5">
-        <f>IF(A103="","",IF(A103+$B$8&gt;$B$6+$B$7,"",A103+$B$8))</f>
+        <f>IF(A103="","",IF(AND(UPPER($B$3)="CHICAGO",A103&lt;($B$10*$B$9),A103+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A103+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A103+$B$8)))</f>
         <v/>
       </c>
       <c r="B104" s="18">
-        <f>IF(A104="","",IF(A104&lt;=$B$6,$B$5*A104/$B$6,MAX(0,$B$5*(1-(A104-$B$6)/$B$7))))</f>
+        <f>IF(A104="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C104/$B$15),IF(A104&lt;=$B$6,$B$5*A104/$B$6,MAX(0,$B$5*(1-(A104-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C104" s="18">
+        <f>IF(OR(A104="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A104&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A104))/$B$10)+$B$12)/((((($B$10*$B$9)-A104))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A104-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A104-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5">
-        <f>IF(A104="","",IF(A104+$B$8&gt;$B$6+$B$7,"",A104+$B$8))</f>
+        <f>IF(A104="","",IF(AND(UPPER($B$3)="CHICAGO",A104&lt;($B$10*$B$9),A104+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A104+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A104+$B$8)))</f>
         <v/>
       </c>
       <c r="B105" s="18">
-        <f>IF(A105="","",IF(A105&lt;=$B$6,$B$5*A105/$B$6,MAX(0,$B$5*(1-(A105-$B$6)/$B$7))))</f>
+        <f>IF(A105="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C105/$B$15),IF(A105&lt;=$B$6,$B$5*A105/$B$6,MAX(0,$B$5*(1-(A105-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C105" s="18">
+        <f>IF(OR(A105="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A105&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A105))/$B$10)+$B$12)/((((($B$10*$B$9)-A105))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A105-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A105-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5">
-        <f>IF(A105="","",IF(A105+$B$8&gt;$B$6+$B$7,"",A105+$B$8))</f>
+        <f>IF(A105="","",IF(AND(UPPER($B$3)="CHICAGO",A105&lt;($B$10*$B$9),A105+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A105+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A105+$B$8)))</f>
         <v/>
       </c>
       <c r="B106" s="18">
-        <f>IF(A106="","",IF(A106&lt;=$B$6,$B$5*A106/$B$6,MAX(0,$B$5*(1-(A106-$B$6)/$B$7))))</f>
+        <f>IF(A106="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C106/$B$15),IF(A106&lt;=$B$6,$B$5*A106/$B$6,MAX(0,$B$5*(1-(A106-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C106" s="18">
+        <f>IF(OR(A106="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A106&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A106))/$B$10)+$B$12)/((((($B$10*$B$9)-A106))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A106-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A106-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5">
-        <f>IF(A106="","",IF(A106+$B$8&gt;$B$6+$B$7,"",A106+$B$8))</f>
+        <f>IF(A106="","",IF(AND(UPPER($B$3)="CHICAGO",A106&lt;($B$10*$B$9),A106+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A106+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A106+$B$8)))</f>
         <v/>
       </c>
       <c r="B107" s="18">
-        <f>IF(A107="","",IF(A107&lt;=$B$6,$B$5*A107/$B$6,MAX(0,$B$5*(1-(A107-$B$6)/$B$7))))</f>
+        <f>IF(A107="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C107/$B$15),IF(A107&lt;=$B$6,$B$5*A107/$B$6,MAX(0,$B$5*(1-(A107-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C107" s="18">
+        <f>IF(OR(A107="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A107&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A107))/$B$10)+$B$12)/((((($B$10*$B$9)-A107))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A107-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A107-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="5">
-        <f>IF(A107="","",IF(A107+$B$8&gt;$B$6+$B$7,"",A107+$B$8))</f>
+        <f>IF(A107="","",IF(AND(UPPER($B$3)="CHICAGO",A107&lt;($B$10*$B$9),A107+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A107+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A107+$B$8)))</f>
         <v/>
       </c>
       <c r="B108" s="18">
-        <f>IF(A108="","",IF(A108&lt;=$B$6,$B$5*A108/$B$6,MAX(0,$B$5*(1-(A108-$B$6)/$B$7))))</f>
+        <f>IF(A108="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C108/$B$15),IF(A108&lt;=$B$6,$B$5*A108/$B$6,MAX(0,$B$5*(1-(A108-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C108" s="18">
+        <f>IF(OR(A108="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A108&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A108))/$B$10)+$B$12)/((((($B$10*$B$9)-A108))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A108-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A108-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5">
-        <f>IF(A108="","",IF(A108+$B$8&gt;$B$6+$B$7,"",A108+$B$8))</f>
+        <f>IF(A108="","",IF(AND(UPPER($B$3)="CHICAGO",A108&lt;($B$10*$B$9),A108+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A108+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A108+$B$8)))</f>
         <v/>
       </c>
       <c r="B109" s="18">
-        <f>IF(A109="","",IF(A109&lt;=$B$6,$B$5*A109/$B$6,MAX(0,$B$5*(1-(A109-$B$6)/$B$7))))</f>
+        <f>IF(A109="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C109/$B$15),IF(A109&lt;=$B$6,$B$5*A109/$B$6,MAX(0,$B$5*(1-(A109-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C109" s="18">
+        <f>IF(OR(A109="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A109&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A109))/$B$10)+$B$12)/((((($B$10*$B$9)-A109))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A109-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A109-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="5">
-        <f>IF(A109="","",IF(A109+$B$8&gt;$B$6+$B$7,"",A109+$B$8))</f>
+        <f>IF(A109="","",IF(AND(UPPER($B$3)="CHICAGO",A109&lt;($B$10*$B$9),A109+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A109+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A109+$B$8)))</f>
         <v/>
       </c>
       <c r="B110" s="18">
-        <f>IF(A110="","",IF(A110&lt;=$B$6,$B$5*A110/$B$6,MAX(0,$B$5*(1-(A110-$B$6)/$B$7))))</f>
+        <f>IF(A110="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C110/$B$15),IF(A110&lt;=$B$6,$B$5*A110/$B$6,MAX(0,$B$5*(1-(A110-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C110" s="18">
+        <f>IF(OR(A110="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A110&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A110))/$B$10)+$B$12)/((((($B$10*$B$9)-A110))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A110-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A110-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5">
-        <f>IF(A110="","",IF(A110+$B$8&gt;$B$6+$B$7,"",A110+$B$8))</f>
+        <f>IF(A110="","",IF(AND(UPPER($B$3)="CHICAGO",A110&lt;($B$10*$B$9),A110+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A110+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A110+$B$8)))</f>
         <v/>
       </c>
       <c r="B111" s="18">
-        <f>IF(A111="","",IF(A111&lt;=$B$6,$B$5*A111/$B$6,MAX(0,$B$5*(1-(A111-$B$6)/$B$7))))</f>
+        <f>IF(A111="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C111/$B$15),IF(A111&lt;=$B$6,$B$5*A111/$B$6,MAX(0,$B$5*(1-(A111-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C111" s="18">
+        <f>IF(OR(A111="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A111&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A111))/$B$10)+$B$12)/((((($B$10*$B$9)-A111))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A111-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A111-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="5">
-        <f>IF(A111="","",IF(A111+$B$8&gt;$B$6+$B$7,"",A111+$B$8))</f>
+        <f>IF(A111="","",IF(AND(UPPER($B$3)="CHICAGO",A111&lt;($B$10*$B$9),A111+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A111+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A111+$B$8)))</f>
         <v/>
       </c>
       <c r="B112" s="18">
-        <f>IF(A112="","",IF(A112&lt;=$B$6,$B$5*A112/$B$6,MAX(0,$B$5*(1-(A112-$B$6)/$B$7))))</f>
+        <f>IF(A112="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C112/$B$15),IF(A112&lt;=$B$6,$B$5*A112/$B$6,MAX(0,$B$5*(1-(A112-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C112" s="18">
+        <f>IF(OR(A112="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A112&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A112))/$B$10)+$B$12)/((((($B$10*$B$9)-A112))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A112-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A112-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5">
-        <f>IF(A112="","",IF(A112+$B$8&gt;$B$6+$B$7,"",A112+$B$8))</f>
+        <f>IF(A112="","",IF(AND(UPPER($B$3)="CHICAGO",A112&lt;($B$10*$B$9),A112+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A112+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A112+$B$8)))</f>
         <v/>
       </c>
       <c r="B113" s="18">
-        <f>IF(A113="","",IF(A113&lt;=$B$6,$B$5*A113/$B$6,MAX(0,$B$5*(1-(A113-$B$6)/$B$7))))</f>
+        <f>IF(A113="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C113/$B$15),IF(A113&lt;=$B$6,$B$5*A113/$B$6,MAX(0,$B$5*(1-(A113-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C113" s="18">
+        <f>IF(OR(A113="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A113&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A113))/$B$10)+$B$12)/((((($B$10*$B$9)-A113))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A113-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A113-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="5">
-        <f>IF(A113="","",IF(A113+$B$8&gt;$B$6+$B$7,"",A113+$B$8))</f>
+        <f>IF(A113="","",IF(AND(UPPER($B$3)="CHICAGO",A113&lt;($B$10*$B$9),A113+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A113+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A113+$B$8)))</f>
         <v/>
       </c>
       <c r="B114" s="18">
-        <f>IF(A114="","",IF(A114&lt;=$B$6,$B$5*A114/$B$6,MAX(0,$B$5*(1-(A114-$B$6)/$B$7))))</f>
+        <f>IF(A114="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C114/$B$15),IF(A114&lt;=$B$6,$B$5*A114/$B$6,MAX(0,$B$5*(1-(A114-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C114" s="18">
+        <f>IF(OR(A114="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A114&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A114))/$B$10)+$B$12)/((((($B$10*$B$9)-A114))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A114-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A114-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5">
-        <f>IF(A114="","",IF(A114+$B$8&gt;$B$6+$B$7,"",A114+$B$8))</f>
+        <f>IF(A114="","",IF(AND(UPPER($B$3)="CHICAGO",A114&lt;($B$10*$B$9),A114+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A114+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A114+$B$8)))</f>
         <v/>
       </c>
       <c r="B115" s="18">
-        <f>IF(A115="","",IF(A115&lt;=$B$6,$B$5*A115/$B$6,MAX(0,$B$5*(1-(A115-$B$6)/$B$7))))</f>
+        <f>IF(A115="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C115/$B$15),IF(A115&lt;=$B$6,$B$5*A115/$B$6,MAX(0,$B$5*(1-(A115-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C115" s="18">
+        <f>IF(OR(A115="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A115&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A115))/$B$10)+$B$12)/((((($B$10*$B$9)-A115))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A115-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A115-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5">
-        <f>IF(A115="","",IF(A115+$B$8&gt;$B$6+$B$7,"",A115+$B$8))</f>
+        <f>IF(A115="","",IF(AND(UPPER($B$3)="CHICAGO",A115&lt;($B$10*$B$9),A115+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A115+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A115+$B$8)))</f>
         <v/>
       </c>
       <c r="B116" s="18">
-        <f>IF(A116="","",IF(A116&lt;=$B$6,$B$5*A116/$B$6,MAX(0,$B$5*(1-(A116-$B$6)/$B$7))))</f>
+        <f>IF(A116="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C116/$B$15),IF(A116&lt;=$B$6,$B$5*A116/$B$6,MAX(0,$B$5*(1-(A116-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C116" s="18">
+        <f>IF(OR(A116="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A116&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A116))/$B$10)+$B$12)/((((($B$10*$B$9)-A116))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A116-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A116-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5">
-        <f>IF(A116="","",IF(A116+$B$8&gt;$B$6+$B$7,"",A116+$B$8))</f>
+        <f>IF(A116="","",IF(AND(UPPER($B$3)="CHICAGO",A116&lt;($B$10*$B$9),A116+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A116+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A116+$B$8)))</f>
         <v/>
       </c>
       <c r="B117" s="18">
-        <f>IF(A117="","",IF(A117&lt;=$B$6,$B$5*A117/$B$6,MAX(0,$B$5*(1-(A117-$B$6)/$B$7))))</f>
+        <f>IF(A117="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C117/$B$15),IF(A117&lt;=$B$6,$B$5*A117/$B$6,MAX(0,$B$5*(1-(A117-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C117" s="18">
+        <f>IF(OR(A117="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A117&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A117))/$B$10)+$B$12)/((((($B$10*$B$9)-A117))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A117-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A117-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="5">
-        <f>IF(A117="","",IF(A117+$B$8&gt;$B$6+$B$7,"",A117+$B$8))</f>
+        <f>IF(A117="","",IF(AND(UPPER($B$3)="CHICAGO",A117&lt;($B$10*$B$9),A117+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A117+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A117+$B$8)))</f>
         <v/>
       </c>
       <c r="B118" s="18">
-        <f>IF(A118="","",IF(A118&lt;=$B$6,$B$5*A118/$B$6,MAX(0,$B$5*(1-(A118-$B$6)/$B$7))))</f>
+        <f>IF(A118="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C118/$B$15),IF(A118&lt;=$B$6,$B$5*A118/$B$6,MAX(0,$B$5*(1-(A118-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C118" s="18">
+        <f>IF(OR(A118="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A118&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A118))/$B$10)+$B$12)/((((($B$10*$B$9)-A118))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A118-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A118-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5">
-        <f>IF(A118="","",IF(A118+$B$8&gt;$B$6+$B$7,"",A118+$B$8))</f>
+        <f>IF(A118="","",IF(AND(UPPER($B$3)="CHICAGO",A118&lt;($B$10*$B$9),A118+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A118+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A118+$B$8)))</f>
         <v/>
       </c>
       <c r="B119" s="18">
-        <f>IF(A119="","",IF(A119&lt;=$B$6,$B$5*A119/$B$6,MAX(0,$B$5*(1-(A119-$B$6)/$B$7))))</f>
+        <f>IF(A119="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C119/$B$15),IF(A119&lt;=$B$6,$B$5*A119/$B$6,MAX(0,$B$5*(1-(A119-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C119" s="18">
+        <f>IF(OR(A119="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A119&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A119))/$B$10)+$B$12)/((((($B$10*$B$9)-A119))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A119-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A119-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="5">
-        <f>IF(A119="","",IF(A119+$B$8&gt;$B$6+$B$7,"",A119+$B$8))</f>
+        <f>IF(A119="","",IF(AND(UPPER($B$3)="CHICAGO",A119&lt;($B$10*$B$9),A119+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A119+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A119+$B$8)))</f>
         <v/>
       </c>
       <c r="B120" s="18">
-        <f>IF(A120="","",IF(A120&lt;=$B$6,$B$5*A120/$B$6,MAX(0,$B$5*(1-(A120-$B$6)/$B$7))))</f>
+        <f>IF(A120="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C120/$B$15),IF(A120&lt;=$B$6,$B$5*A120/$B$6,MAX(0,$B$5*(1-(A120-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C120" s="18">
+        <f>IF(OR(A120="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A120&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A120))/$B$10)+$B$12)/((((($B$10*$B$9)-A120))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A120-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A120-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5">
-        <f>IF(A120="","",IF(A120+$B$8&gt;$B$6+$B$7,"",A120+$B$8))</f>
+        <f>IF(A120="","",IF(AND(UPPER($B$3)="CHICAGO",A120&lt;($B$10*$B$9),A120+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A120+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A120+$B$8)))</f>
         <v/>
       </c>
       <c r="B121" s="18">
-        <f>IF(A121="","",IF(A121&lt;=$B$6,$B$5*A121/$B$6,MAX(0,$B$5*(1-(A121-$B$6)/$B$7))))</f>
+        <f>IF(A121="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C121/$B$15),IF(A121&lt;=$B$6,$B$5*A121/$B$6,MAX(0,$B$5*(1-(A121-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C121" s="18">
+        <f>IF(OR(A121="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A121&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A121))/$B$10)+$B$12)/((((($B$10*$B$9)-A121))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A121-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A121-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="5">
-        <f>IF(A121="","",IF(A121+$B$8&gt;$B$6+$B$7,"",A121+$B$8))</f>
+        <f>IF(A121="","",IF(AND(UPPER($B$3)="CHICAGO",A121&lt;($B$10*$B$9),A121+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A121+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A121+$B$8)))</f>
         <v/>
       </c>
       <c r="B122" s="18">
-        <f>IF(A122="","",IF(A122&lt;=$B$6,$B$5*A122/$B$6,MAX(0,$B$5*(1-(A122-$B$6)/$B$7))))</f>
+        <f>IF(A122="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C122/$B$15),IF(A122&lt;=$B$6,$B$5*A122/$B$6,MAX(0,$B$5*(1-(A122-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C122" s="18">
+        <f>IF(OR(A122="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A122&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A122))/$B$10)+$B$12)/((((($B$10*$B$9)-A122))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A122-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A122-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5">
-        <f>IF(A122="","",IF(A122+$B$8&gt;$B$6+$B$7,"",A122+$B$8))</f>
+        <f>IF(A122="","",IF(AND(UPPER($B$3)="CHICAGO",A122&lt;($B$10*$B$9),A122+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A122+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A122+$B$8)))</f>
         <v/>
       </c>
       <c r="B123" s="18">
-        <f>IF(A123="","",IF(A123&lt;=$B$6,$B$5*A123/$B$6,MAX(0,$B$5*(1-(A123-$B$6)/$B$7))))</f>
+        <f>IF(A123="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C123/$B$15),IF(A123&lt;=$B$6,$B$5*A123/$B$6,MAX(0,$B$5*(1-(A123-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C123" s="18">
+        <f>IF(OR(A123="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A123&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A123))/$B$10)+$B$12)/((((($B$10*$B$9)-A123))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A123-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A123-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="5">
-        <f>IF(A123="","",IF(A123+$B$8&gt;$B$6+$B$7,"",A123+$B$8))</f>
+        <f>IF(A123="","",IF(AND(UPPER($B$3)="CHICAGO",A123&lt;($B$10*$B$9),A123+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A123+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A123+$B$8)))</f>
         <v/>
       </c>
       <c r="B124" s="18">
-        <f>IF(A124="","",IF(A124&lt;=$B$6,$B$5*A124/$B$6,MAX(0,$B$5*(1-(A124-$B$6)/$B$7))))</f>
+        <f>IF(A124="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C124/$B$15),IF(A124&lt;=$B$6,$B$5*A124/$B$6,MAX(0,$B$5*(1-(A124-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C124" s="18">
+        <f>IF(OR(A124="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A124&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A124))/$B$10)+$B$12)/((((($B$10*$B$9)-A124))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A124-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A124-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5">
-        <f>IF(A124="","",IF(A124+$B$8&gt;$B$6+$B$7,"",A124+$B$8))</f>
+        <f>IF(A124="","",IF(AND(UPPER($B$3)="CHICAGO",A124&lt;($B$10*$B$9),A124+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A124+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A124+$B$8)))</f>
         <v/>
       </c>
       <c r="B125" s="18">
-        <f>IF(A125="","",IF(A125&lt;=$B$6,$B$5*A125/$B$6,MAX(0,$B$5*(1-(A125-$B$6)/$B$7))))</f>
+        <f>IF(A125="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C125/$B$15),IF(A125&lt;=$B$6,$B$5*A125/$B$6,MAX(0,$B$5*(1-(A125-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C125" s="18">
+        <f>IF(OR(A125="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A125&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A125))/$B$10)+$B$12)/((((($B$10*$B$9)-A125))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A125-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A125-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="5">
-        <f>IF(A125="","",IF(A125+$B$8&gt;$B$6+$B$7,"",A125+$B$8))</f>
+        <f>IF(A125="","",IF(AND(UPPER($B$3)="CHICAGO",A125&lt;($B$10*$B$9),A125+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A125+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A125+$B$8)))</f>
         <v/>
       </c>
       <c r="B126" s="18">
-        <f>IF(A126="","",IF(A126&lt;=$B$6,$B$5*A126/$B$6,MAX(0,$B$5*(1-(A126-$B$6)/$B$7))))</f>
+        <f>IF(A126="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C126/$B$15),IF(A126&lt;=$B$6,$B$5*A126/$B$6,MAX(0,$B$5*(1-(A126-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C126" s="18">
+        <f>IF(OR(A126="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A126&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A126))/$B$10)+$B$12)/((((($B$10*$B$9)-A126))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A126-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A126-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5">
-        <f>IF(A126="","",IF(A126+$B$8&gt;$B$6+$B$7,"",A126+$B$8))</f>
+        <f>IF(A126="","",IF(AND(UPPER($B$3)="CHICAGO",A126&lt;($B$10*$B$9),A126+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A126+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A126+$B$8)))</f>
         <v/>
       </c>
       <c r="B127" s="18">
-        <f>IF(A127="","",IF(A127&lt;=$B$6,$B$5*A127/$B$6,MAX(0,$B$5*(1-(A127-$B$6)/$B$7))))</f>
+        <f>IF(A127="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C127/$B$15),IF(A127&lt;=$B$6,$B$5*A127/$B$6,MAX(0,$B$5*(1-(A127-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C127" s="18">
+        <f>IF(OR(A127="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A127&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A127))/$B$10)+$B$12)/((((($B$10*$B$9)-A127))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A127-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A127-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="5">
-        <f>IF(A127="","",IF(A127+$B$8&gt;$B$6+$B$7,"",A127+$B$8))</f>
+        <f>IF(A127="","",IF(AND(UPPER($B$3)="CHICAGO",A127&lt;($B$10*$B$9),A127+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A127+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A127+$B$8)))</f>
         <v/>
       </c>
       <c r="B128" s="18">
-        <f>IF(A128="","",IF(A128&lt;=$B$6,$B$5*A128/$B$6,MAX(0,$B$5*(1-(A128-$B$6)/$B$7))))</f>
+        <f>IF(A128="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C128/$B$15),IF(A128&lt;=$B$6,$B$5*A128/$B$6,MAX(0,$B$5*(1-(A128-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C128" s="18">
+        <f>IF(OR(A128="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A128&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A128))/$B$10)+$B$12)/((((($B$10*$B$9)-A128))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A128-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A128-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5">
-        <f>IF(A128="","",IF(A128+$B$8&gt;$B$6+$B$7,"",A128+$B$8))</f>
+        <f>IF(A128="","",IF(AND(UPPER($B$3)="CHICAGO",A128&lt;($B$10*$B$9),A128+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A128+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A128+$B$8)))</f>
         <v/>
       </c>
       <c r="B129" s="18">
-        <f>IF(A129="","",IF(A129&lt;=$B$6,$B$5*A129/$B$6,MAX(0,$B$5*(1-(A129-$B$6)/$B$7))))</f>
+        <f>IF(A129="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C129/$B$15),IF(A129&lt;=$B$6,$B$5*A129/$B$6,MAX(0,$B$5*(1-(A129-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C129" s="18">
+        <f>IF(OR(A129="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A129&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A129))/$B$10)+$B$12)/((((($B$10*$B$9)-A129))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A129-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A129-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="5">
-        <f>IF(A129="","",IF(A129+$B$8&gt;$B$6+$B$7,"",A129+$B$8))</f>
+        <f>IF(A129="","",IF(AND(UPPER($B$3)="CHICAGO",A129&lt;($B$10*$B$9),A129+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A129+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A129+$B$8)))</f>
         <v/>
       </c>
       <c r="B130" s="18">
-        <f>IF(A130="","",IF(A130&lt;=$B$6,$B$5*A130/$B$6,MAX(0,$B$5*(1-(A130-$B$6)/$B$7))))</f>
+        <f>IF(A130="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C130/$B$15),IF(A130&lt;=$B$6,$B$5*A130/$B$6,MAX(0,$B$5*(1-(A130-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C130" s="18">
+        <f>IF(OR(A130="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A130&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A130))/$B$10)+$B$12)/((((($B$10*$B$9)-A130))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A130-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A130-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5">
+        <f>IF(A130="","",IF(AND(UPPER($B$3)="CHICAGO",A130&lt;($B$10*$B$9),A130+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A130+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A130+$B$8)))</f>
+        <v/>
+      </c>
+      <c r="B131" s="18">
+        <f>IF(A131="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C131/$B$15),IF(A131&lt;=$B$6,$B$5*A131/$B$6,MAX(0,$B$5*(1-(A131-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C131" s="18">
+        <f>IF(OR(A131="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A131&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A131))/$B$10)+$B$12)/((((($B$10*$B$9)-A131))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A131-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A131-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5">
+        <f>IF(A131="","",IF(AND(UPPER($B$3)="CHICAGO",A131&lt;($B$10*$B$9),A131+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A131+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A131+$B$8)))</f>
+        <v/>
+      </c>
+      <c r="B132" s="18">
+        <f>IF(A132="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C132/$B$15),IF(A132&lt;=$B$6,$B$5*A132/$B$6,MAX(0,$B$5*(1-(A132-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C132" s="18">
+        <f>IF(OR(A132="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A132&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A132))/$B$10)+$B$12)/((((($B$10*$B$9)-A132))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A132-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A132-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5">
+        <f>IF(A132="","",IF(AND(UPPER($B$3)="CHICAGO",A132&lt;($B$10*$B$9),A132+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A132+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A132+$B$8)))</f>
+        <v/>
+      </c>
+      <c r="B133" s="18">
+        <f>IF(A133="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C133/$B$15),IF(A133&lt;=$B$6,$B$5*A133/$B$6,MAX(0,$B$5*(1-(A133-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C133" s="18">
+        <f>IF(OR(A133="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A133&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A133))/$B$10)+$B$12)/((((($B$10*$B$9)-A133))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A133-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A133-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5">
+        <f>IF(A133="","",IF(AND(UPPER($B$3)="CHICAGO",A133&lt;($B$10*$B$9),A133+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A133+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A133+$B$8)))</f>
+        <v/>
+      </c>
+      <c r="B134" s="18">
+        <f>IF(A134="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C134/$B$15),IF(A134&lt;=$B$6,$B$5*A134/$B$6,MAX(0,$B$5*(1-(A134-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C134" s="18">
+        <f>IF(OR(A134="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A134&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A134))/$B$10)+$B$12)/((((($B$10*$B$9)-A134))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A134-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A134-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5">
+        <f>IF(A134="","",IF(AND(UPPER($B$3)="CHICAGO",A134&lt;($B$10*$B$9),A134+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A134+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A134+$B$8)))</f>
+        <v/>
+      </c>
+      <c r="B135" s="18">
+        <f>IF(A135="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C135/$B$15),IF(A135&lt;=$B$6,$B$5*A135/$B$6,MAX(0,$B$5*(1-(A135-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C135" s="18">
+        <f>IF(OR(A135="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A135&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A135))/$B$10)+$B$12)/((((($B$10*$B$9)-A135))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A135-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A135-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5">
+        <f>IF(A135="","",IF(AND(UPPER($B$3)="CHICAGO",A135&lt;($B$10*$B$9),A135+$B$8&gt;($B$10*$B$9)),($B$10*$B$9),IF(A135+$B$8&gt;(IF(UPPER($B$3)="CHICAGO",$B$9,$B$6+$B$7)),"",A135+$B$8)))</f>
+        <v/>
+      </c>
+      <c r="B136" s="18">
+        <f>IF(A136="","",IF(UPPER($B$3)="CHICAGO",IF($B$15&lt;=0,0,$B$5*C136/$B$15),IF(A136&lt;=$B$6,$B$5*A136/$B$6,MAX(0,$B$5*(1-(A136-$B$6)/$B$7)))))</f>
+        <v/>
+      </c>
+      <c r="C136" s="18">
+        <f>IF(OR(A136="",UPPER($B$3)&lt;&gt;"CHICAGO"),"",IF(A136&lt;=($B$10*$B$9),$B$11*((1-$B$13)*(((($B$10*$B$9)-A136))/$B$10)+$B$12)/((((($B$10*$B$9)-A136))/$B$10)+$B$12)^($B$13+1),$B$11*((1-$B$13)*(((A136-($B$10*$B$9)))/(1-$B$10))+$B$12)/((((A136-($B$10*$B$9)))/(1-$B$10))+$B$12)^($B$13+1)))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4876,7 +5590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K130"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4895,19 +5609,19 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Routing stockage — Puls LIVE (WSE max = niveau d'eau max)</t>
+          <t>Routing stockage — Puls LIVE (lit Hydrogramme_entree, y compris Chicago)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IMPORTANT: HW ≈ 1.7 m = PROFONDEUR au-dessus de l'invert. WSE ≈ 37.0 m = ÉLÉVATION absolue = invert(35.36) + HW. Ce n'est pas une erreur: avant vous lisiez WSE (~37); HW (~1.7) est seulement la profondeur.</t>
+          <t>IMPORTANT: HW = PROFONDEUR (~1.7 m). WSE = ÉLÉVATION = invert + HW (~37 m). Q_in vient de Hydrogramme_entree (Chicago ou Triangle).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Formule: WSE = Parametres!C9 + HW.  2S/dt−Q = report Puls. RHS = cible Ind.</t>
         </is>
@@ -4972,11 +5686,11 @@
     </row>
     <row r="5">
       <c r="A5" s="5">
-        <f>Hydrogramme_entree!A11</f>
+        <f>Hydrogramme_entree!A17</f>
         <v/>
       </c>
       <c r="B5" s="12">
-        <f>Hydrogramme_entree!B11</f>
+        <f>Hydrogramme_entree!B17</f>
         <v/>
       </c>
       <c r="C5" s="12" t="n">
@@ -5010,11 +5724,11 @@
     </row>
     <row r="6">
       <c r="A6" s="5">
-        <f>Hydrogramme_entree!A12</f>
+        <f>Hydrogramme_entree!A18</f>
         <v/>
       </c>
       <c r="B6" s="12">
-        <f>Hydrogramme_entree!B12</f>
+        <f>Hydrogramme_entree!B18</f>
         <v/>
       </c>
       <c r="C6" s="12">
@@ -5056,11 +5770,11 @@
     </row>
     <row r="7">
       <c r="A7" s="5">
-        <f>Hydrogramme_entree!A13</f>
+        <f>Hydrogramme_entree!A19</f>
         <v/>
       </c>
       <c r="B7" s="12">
-        <f>Hydrogramme_entree!B13</f>
+        <f>Hydrogramme_entree!B19</f>
         <v/>
       </c>
       <c r="C7" s="12">
@@ -5102,11 +5816,11 @@
     </row>
     <row r="8">
       <c r="A8" s="5">
-        <f>Hydrogramme_entree!A14</f>
+        <f>Hydrogramme_entree!A20</f>
         <v/>
       </c>
       <c r="B8" s="12">
-        <f>Hydrogramme_entree!B14</f>
+        <f>Hydrogramme_entree!B20</f>
         <v/>
       </c>
       <c r="C8" s="12">
@@ -5148,11 +5862,11 @@
     </row>
     <row r="9">
       <c r="A9" s="5">
-        <f>Hydrogramme_entree!A15</f>
+        <f>Hydrogramme_entree!A21</f>
         <v/>
       </c>
       <c r="B9" s="12">
-        <f>Hydrogramme_entree!B15</f>
+        <f>Hydrogramme_entree!B21</f>
         <v/>
       </c>
       <c r="C9" s="12">
@@ -5194,11 +5908,11 @@
     </row>
     <row r="10">
       <c r="A10" s="5">
-        <f>Hydrogramme_entree!A16</f>
+        <f>Hydrogramme_entree!A22</f>
         <v/>
       </c>
       <c r="B10" s="12">
-        <f>Hydrogramme_entree!B16</f>
+        <f>Hydrogramme_entree!B22</f>
         <v/>
       </c>
       <c r="C10" s="12">
@@ -5240,11 +5954,11 @@
     </row>
     <row r="11">
       <c r="A11" s="5">
-        <f>Hydrogramme_entree!A17</f>
+        <f>Hydrogramme_entree!A23</f>
         <v/>
       </c>
       <c r="B11" s="12">
-        <f>Hydrogramme_entree!B17</f>
+        <f>Hydrogramme_entree!B23</f>
         <v/>
       </c>
       <c r="C11" s="12">
@@ -5286,11 +6000,11 @@
     </row>
     <row r="12">
       <c r="A12" s="5">
-        <f>Hydrogramme_entree!A18</f>
+        <f>Hydrogramme_entree!A24</f>
         <v/>
       </c>
       <c r="B12" s="12">
-        <f>Hydrogramme_entree!B18</f>
+        <f>Hydrogramme_entree!B24</f>
         <v/>
       </c>
       <c r="C12" s="12">
@@ -5332,11 +6046,11 @@
     </row>
     <row r="13">
       <c r="A13" s="5">
-        <f>Hydrogramme_entree!A19</f>
+        <f>Hydrogramme_entree!A25</f>
         <v/>
       </c>
       <c r="B13" s="12">
-        <f>Hydrogramme_entree!B19</f>
+        <f>Hydrogramme_entree!B25</f>
         <v/>
       </c>
       <c r="C13" s="12">
@@ -5378,11 +6092,11 @@
     </row>
     <row r="14">
       <c r="A14" s="5">
-        <f>Hydrogramme_entree!A20</f>
+        <f>Hydrogramme_entree!A26</f>
         <v/>
       </c>
       <c r="B14" s="12">
-        <f>Hydrogramme_entree!B20</f>
+        <f>Hydrogramme_entree!B26</f>
         <v/>
       </c>
       <c r="C14" s="12">
@@ -5424,11 +6138,11 @@
     </row>
     <row r="15">
       <c r="A15" s="5">
-        <f>Hydrogramme_entree!A21</f>
+        <f>Hydrogramme_entree!A27</f>
         <v/>
       </c>
       <c r="B15" s="12">
-        <f>Hydrogramme_entree!B21</f>
+        <f>Hydrogramme_entree!B27</f>
         <v/>
       </c>
       <c r="C15" s="12">
@@ -5470,11 +6184,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5">
-        <f>Hydrogramme_entree!A22</f>
+        <f>Hydrogramme_entree!A28</f>
         <v/>
       </c>
       <c r="B16" s="12">
-        <f>Hydrogramme_entree!B22</f>
+        <f>Hydrogramme_entree!B28</f>
         <v/>
       </c>
       <c r="C16" s="12">
@@ -5516,11 +6230,11 @@
     </row>
     <row r="17">
       <c r="A17" s="5">
-        <f>Hydrogramme_entree!A23</f>
+        <f>Hydrogramme_entree!A29</f>
         <v/>
       </c>
       <c r="B17" s="12">
-        <f>Hydrogramme_entree!B23</f>
+        <f>Hydrogramme_entree!B29</f>
         <v/>
       </c>
       <c r="C17" s="12">
@@ -5562,11 +6276,11 @@
     </row>
     <row r="18">
       <c r="A18" s="5">
-        <f>Hydrogramme_entree!A24</f>
+        <f>Hydrogramme_entree!A30</f>
         <v/>
       </c>
       <c r="B18" s="12">
-        <f>Hydrogramme_entree!B24</f>
+        <f>Hydrogramme_entree!B30</f>
         <v/>
       </c>
       <c r="C18" s="12">
@@ -5608,11 +6322,11 @@
     </row>
     <row r="19">
       <c r="A19" s="5">
-        <f>Hydrogramme_entree!A25</f>
+        <f>Hydrogramme_entree!A31</f>
         <v/>
       </c>
       <c r="B19" s="12">
-        <f>Hydrogramme_entree!B25</f>
+        <f>Hydrogramme_entree!B31</f>
         <v/>
       </c>
       <c r="C19" s="12">
@@ -5654,11 +6368,11 @@
     </row>
     <row r="20">
       <c r="A20" s="5">
-        <f>Hydrogramme_entree!A26</f>
+        <f>Hydrogramme_entree!A32</f>
         <v/>
       </c>
       <c r="B20" s="12">
-        <f>Hydrogramme_entree!B26</f>
+        <f>Hydrogramme_entree!B32</f>
         <v/>
       </c>
       <c r="C20" s="12">
@@ -5700,11 +6414,11 @@
     </row>
     <row r="21">
       <c r="A21" s="5">
-        <f>Hydrogramme_entree!A27</f>
+        <f>Hydrogramme_entree!A33</f>
         <v/>
       </c>
       <c r="B21" s="12">
-        <f>Hydrogramme_entree!B27</f>
+        <f>Hydrogramme_entree!B33</f>
         <v/>
       </c>
       <c r="C21" s="12">
@@ -5746,11 +6460,11 @@
     </row>
     <row r="22">
       <c r="A22" s="5">
-        <f>Hydrogramme_entree!A28</f>
+        <f>Hydrogramme_entree!A34</f>
         <v/>
       </c>
       <c r="B22" s="12">
-        <f>Hydrogramme_entree!B28</f>
+        <f>Hydrogramme_entree!B34</f>
         <v/>
       </c>
       <c r="C22" s="12">
@@ -5792,11 +6506,11 @@
     </row>
     <row r="23">
       <c r="A23" s="5">
-        <f>Hydrogramme_entree!A29</f>
+        <f>Hydrogramme_entree!A35</f>
         <v/>
       </c>
       <c r="B23" s="12">
-        <f>Hydrogramme_entree!B29</f>
+        <f>Hydrogramme_entree!B35</f>
         <v/>
       </c>
       <c r="C23" s="12">
@@ -5838,11 +6552,11 @@
     </row>
     <row r="24">
       <c r="A24" s="5">
-        <f>Hydrogramme_entree!A30</f>
+        <f>Hydrogramme_entree!A36</f>
         <v/>
       </c>
       <c r="B24" s="12">
-        <f>Hydrogramme_entree!B30</f>
+        <f>Hydrogramme_entree!B36</f>
         <v/>
       </c>
       <c r="C24" s="12">
@@ -5884,11 +6598,11 @@
     </row>
     <row r="25">
       <c r="A25" s="5">
-        <f>Hydrogramme_entree!A31</f>
+        <f>Hydrogramme_entree!A37</f>
         <v/>
       </c>
       <c r="B25" s="12">
-        <f>Hydrogramme_entree!B31</f>
+        <f>Hydrogramme_entree!B37</f>
         <v/>
       </c>
       <c r="C25" s="12">
@@ -5930,11 +6644,11 @@
     </row>
     <row r="26">
       <c r="A26" s="5">
-        <f>Hydrogramme_entree!A32</f>
+        <f>Hydrogramme_entree!A38</f>
         <v/>
       </c>
       <c r="B26" s="12">
-        <f>Hydrogramme_entree!B32</f>
+        <f>Hydrogramme_entree!B38</f>
         <v/>
       </c>
       <c r="C26" s="12">
@@ -5976,11 +6690,11 @@
     </row>
     <row r="27">
       <c r="A27" s="5">
-        <f>Hydrogramme_entree!A33</f>
+        <f>Hydrogramme_entree!A39</f>
         <v/>
       </c>
       <c r="B27" s="12">
-        <f>Hydrogramme_entree!B33</f>
+        <f>Hydrogramme_entree!B39</f>
         <v/>
       </c>
       <c r="C27" s="12">
@@ -6022,11 +6736,11 @@
     </row>
     <row r="28">
       <c r="A28" s="5">
-        <f>Hydrogramme_entree!A34</f>
+        <f>Hydrogramme_entree!A40</f>
         <v/>
       </c>
       <c r="B28" s="12">
-        <f>Hydrogramme_entree!B34</f>
+        <f>Hydrogramme_entree!B40</f>
         <v/>
       </c>
       <c r="C28" s="12">
@@ -6068,11 +6782,11 @@
     </row>
     <row r="29">
       <c r="A29" s="5">
-        <f>Hydrogramme_entree!A35</f>
+        <f>Hydrogramme_entree!A41</f>
         <v/>
       </c>
       <c r="B29" s="12">
-        <f>Hydrogramme_entree!B35</f>
+        <f>Hydrogramme_entree!B41</f>
         <v/>
       </c>
       <c r="C29" s="12">
@@ -6114,11 +6828,11 @@
     </row>
     <row r="30">
       <c r="A30" s="5">
-        <f>Hydrogramme_entree!A36</f>
+        <f>Hydrogramme_entree!A42</f>
         <v/>
       </c>
       <c r="B30" s="12">
-        <f>Hydrogramme_entree!B36</f>
+        <f>Hydrogramme_entree!B42</f>
         <v/>
       </c>
       <c r="C30" s="12">
@@ -6160,11 +6874,11 @@
     </row>
     <row r="31">
       <c r="A31" s="5">
-        <f>Hydrogramme_entree!A37</f>
+        <f>Hydrogramme_entree!A43</f>
         <v/>
       </c>
       <c r="B31" s="12">
-        <f>Hydrogramme_entree!B37</f>
+        <f>Hydrogramme_entree!B43</f>
         <v/>
       </c>
       <c r="C31" s="12">
@@ -6206,11 +6920,11 @@
     </row>
     <row r="32">
       <c r="A32" s="5">
-        <f>Hydrogramme_entree!A38</f>
+        <f>Hydrogramme_entree!A44</f>
         <v/>
       </c>
       <c r="B32" s="12">
-        <f>Hydrogramme_entree!B38</f>
+        <f>Hydrogramme_entree!B44</f>
         <v/>
       </c>
       <c r="C32" s="12">
@@ -6252,11 +6966,11 @@
     </row>
     <row r="33">
       <c r="A33" s="5">
-        <f>Hydrogramme_entree!A39</f>
+        <f>Hydrogramme_entree!A45</f>
         <v/>
       </c>
       <c r="B33" s="12">
-        <f>Hydrogramme_entree!B39</f>
+        <f>Hydrogramme_entree!B45</f>
         <v/>
       </c>
       <c r="C33" s="12">
@@ -6298,11 +7012,11 @@
     </row>
     <row r="34">
       <c r="A34" s="5">
-        <f>Hydrogramme_entree!A40</f>
+        <f>Hydrogramme_entree!A46</f>
         <v/>
       </c>
       <c r="B34" s="12">
-        <f>Hydrogramme_entree!B40</f>
+        <f>Hydrogramme_entree!B46</f>
         <v/>
       </c>
       <c r="C34" s="12">
@@ -6344,11 +7058,11 @@
     </row>
     <row r="35">
       <c r="A35" s="5">
-        <f>Hydrogramme_entree!A41</f>
+        <f>Hydrogramme_entree!A47</f>
         <v/>
       </c>
       <c r="B35" s="12">
-        <f>Hydrogramme_entree!B41</f>
+        <f>Hydrogramme_entree!B47</f>
         <v/>
       </c>
       <c r="C35" s="12">
@@ -6390,11 +7104,11 @@
     </row>
     <row r="36">
       <c r="A36" s="5">
-        <f>Hydrogramme_entree!A42</f>
+        <f>Hydrogramme_entree!A48</f>
         <v/>
       </c>
       <c r="B36" s="12">
-        <f>Hydrogramme_entree!B42</f>
+        <f>Hydrogramme_entree!B48</f>
         <v/>
       </c>
       <c r="C36" s="12">
@@ -6436,11 +7150,11 @@
     </row>
     <row r="37">
       <c r="A37" s="5">
-        <f>Hydrogramme_entree!A43</f>
+        <f>Hydrogramme_entree!A49</f>
         <v/>
       </c>
       <c r="B37" s="12">
-        <f>Hydrogramme_entree!B43</f>
+        <f>Hydrogramme_entree!B49</f>
         <v/>
       </c>
       <c r="C37" s="12">
@@ -6482,11 +7196,11 @@
     </row>
     <row r="38">
       <c r="A38" s="5">
-        <f>Hydrogramme_entree!A44</f>
+        <f>Hydrogramme_entree!A50</f>
         <v/>
       </c>
       <c r="B38" s="12">
-        <f>Hydrogramme_entree!B44</f>
+        <f>Hydrogramme_entree!B50</f>
         <v/>
       </c>
       <c r="C38" s="12">
@@ -6528,11 +7242,11 @@
     </row>
     <row r="39">
       <c r="A39" s="5">
-        <f>Hydrogramme_entree!A45</f>
+        <f>Hydrogramme_entree!A51</f>
         <v/>
       </c>
       <c r="B39" s="12">
-        <f>Hydrogramme_entree!B45</f>
+        <f>Hydrogramme_entree!B51</f>
         <v/>
       </c>
       <c r="C39" s="12">
@@ -6574,11 +7288,11 @@
     </row>
     <row r="40">
       <c r="A40" s="5">
-        <f>Hydrogramme_entree!A46</f>
+        <f>Hydrogramme_entree!A52</f>
         <v/>
       </c>
       <c r="B40" s="12">
-        <f>Hydrogramme_entree!B46</f>
+        <f>Hydrogramme_entree!B52</f>
         <v/>
       </c>
       <c r="C40" s="12">
@@ -6620,11 +7334,11 @@
     </row>
     <row r="41">
       <c r="A41" s="5">
-        <f>Hydrogramme_entree!A47</f>
+        <f>Hydrogramme_entree!A53</f>
         <v/>
       </c>
       <c r="B41" s="12">
-        <f>Hydrogramme_entree!B47</f>
+        <f>Hydrogramme_entree!B53</f>
         <v/>
       </c>
       <c r="C41" s="12">
@@ -6666,11 +7380,11 @@
     </row>
     <row r="42">
       <c r="A42" s="5">
-        <f>Hydrogramme_entree!A48</f>
+        <f>Hydrogramme_entree!A54</f>
         <v/>
       </c>
       <c r="B42" s="12">
-        <f>Hydrogramme_entree!B48</f>
+        <f>Hydrogramme_entree!B54</f>
         <v/>
       </c>
       <c r="C42" s="12">
@@ -6712,11 +7426,11 @@
     </row>
     <row r="43">
       <c r="A43" s="5">
-        <f>Hydrogramme_entree!A49</f>
+        <f>Hydrogramme_entree!A55</f>
         <v/>
       </c>
       <c r="B43" s="12">
-        <f>Hydrogramme_entree!B49</f>
+        <f>Hydrogramme_entree!B55</f>
         <v/>
       </c>
       <c r="C43" s="12">
@@ -6758,11 +7472,11 @@
     </row>
     <row r="44">
       <c r="A44" s="5">
-        <f>Hydrogramme_entree!A50</f>
+        <f>Hydrogramme_entree!A56</f>
         <v/>
       </c>
       <c r="B44" s="12">
-        <f>Hydrogramme_entree!B50</f>
+        <f>Hydrogramme_entree!B56</f>
         <v/>
       </c>
       <c r="C44" s="12">
@@ -6804,11 +7518,11 @@
     </row>
     <row r="45">
       <c r="A45" s="5">
-        <f>Hydrogramme_entree!A51</f>
+        <f>Hydrogramme_entree!A57</f>
         <v/>
       </c>
       <c r="B45" s="12">
-        <f>Hydrogramme_entree!B51</f>
+        <f>Hydrogramme_entree!B57</f>
         <v/>
       </c>
       <c r="C45" s="12">
@@ -6850,11 +7564,11 @@
     </row>
     <row r="46">
       <c r="A46" s="5">
-        <f>Hydrogramme_entree!A52</f>
+        <f>Hydrogramme_entree!A58</f>
         <v/>
       </c>
       <c r="B46" s="12">
-        <f>Hydrogramme_entree!B52</f>
+        <f>Hydrogramme_entree!B58</f>
         <v/>
       </c>
       <c r="C46" s="12">
@@ -6896,11 +7610,11 @@
     </row>
     <row r="47">
       <c r="A47" s="5">
-        <f>Hydrogramme_entree!A53</f>
+        <f>Hydrogramme_entree!A59</f>
         <v/>
       </c>
       <c r="B47" s="12">
-        <f>Hydrogramme_entree!B53</f>
+        <f>Hydrogramme_entree!B59</f>
         <v/>
       </c>
       <c r="C47" s="12">
@@ -6942,11 +7656,11 @@
     </row>
     <row r="48">
       <c r="A48" s="5">
-        <f>Hydrogramme_entree!A54</f>
+        <f>Hydrogramme_entree!A60</f>
         <v/>
       </c>
       <c r="B48" s="12">
-        <f>Hydrogramme_entree!B54</f>
+        <f>Hydrogramme_entree!B60</f>
         <v/>
       </c>
       <c r="C48" s="12">
@@ -6988,11 +7702,11 @@
     </row>
     <row r="49">
       <c r="A49" s="5">
-        <f>Hydrogramme_entree!A55</f>
+        <f>Hydrogramme_entree!A61</f>
         <v/>
       </c>
       <c r="B49" s="12">
-        <f>Hydrogramme_entree!B55</f>
+        <f>Hydrogramme_entree!B61</f>
         <v/>
       </c>
       <c r="C49" s="12">
@@ -7034,11 +7748,11 @@
     </row>
     <row r="50">
       <c r="A50" s="5">
-        <f>Hydrogramme_entree!A56</f>
+        <f>Hydrogramme_entree!A62</f>
         <v/>
       </c>
       <c r="B50" s="12">
-        <f>Hydrogramme_entree!B56</f>
+        <f>Hydrogramme_entree!B62</f>
         <v/>
       </c>
       <c r="C50" s="12">
@@ -7080,11 +7794,11 @@
     </row>
     <row r="51">
       <c r="A51" s="5">
-        <f>Hydrogramme_entree!A57</f>
+        <f>Hydrogramme_entree!A63</f>
         <v/>
       </c>
       <c r="B51" s="12">
-        <f>Hydrogramme_entree!B57</f>
+        <f>Hydrogramme_entree!B63</f>
         <v/>
       </c>
       <c r="C51" s="12">
@@ -7126,11 +7840,11 @@
     </row>
     <row r="52">
       <c r="A52" s="5">
-        <f>Hydrogramme_entree!A58</f>
+        <f>Hydrogramme_entree!A64</f>
         <v/>
       </c>
       <c r="B52" s="12">
-        <f>Hydrogramme_entree!B58</f>
+        <f>Hydrogramme_entree!B64</f>
         <v/>
       </c>
       <c r="C52" s="12">
@@ -7172,11 +7886,11 @@
     </row>
     <row r="53">
       <c r="A53" s="5">
-        <f>Hydrogramme_entree!A59</f>
+        <f>Hydrogramme_entree!A65</f>
         <v/>
       </c>
       <c r="B53" s="12">
-        <f>Hydrogramme_entree!B59</f>
+        <f>Hydrogramme_entree!B65</f>
         <v/>
       </c>
       <c r="C53" s="12">
@@ -7218,11 +7932,11 @@
     </row>
     <row r="54">
       <c r="A54" s="5">
-        <f>Hydrogramme_entree!A60</f>
+        <f>Hydrogramme_entree!A66</f>
         <v/>
       </c>
       <c r="B54" s="12">
-        <f>Hydrogramme_entree!B60</f>
+        <f>Hydrogramme_entree!B66</f>
         <v/>
       </c>
       <c r="C54" s="12">
@@ -7264,11 +7978,11 @@
     </row>
     <row r="55">
       <c r="A55" s="5">
-        <f>Hydrogramme_entree!A61</f>
+        <f>Hydrogramme_entree!A67</f>
         <v/>
       </c>
       <c r="B55" s="12">
-        <f>Hydrogramme_entree!B61</f>
+        <f>Hydrogramme_entree!B67</f>
         <v/>
       </c>
       <c r="C55" s="12">
@@ -7310,11 +8024,11 @@
     </row>
     <row r="56">
       <c r="A56" s="5">
-        <f>Hydrogramme_entree!A62</f>
+        <f>Hydrogramme_entree!A68</f>
         <v/>
       </c>
       <c r="B56" s="12">
-        <f>Hydrogramme_entree!B62</f>
+        <f>Hydrogramme_entree!B68</f>
         <v/>
       </c>
       <c r="C56" s="12">
@@ -7356,11 +8070,11 @@
     </row>
     <row r="57">
       <c r="A57" s="5">
-        <f>Hydrogramme_entree!A63</f>
+        <f>Hydrogramme_entree!A69</f>
         <v/>
       </c>
       <c r="B57" s="12">
-        <f>Hydrogramme_entree!B63</f>
+        <f>Hydrogramme_entree!B69</f>
         <v/>
       </c>
       <c r="C57" s="12">
@@ -7402,11 +8116,11 @@
     </row>
     <row r="58">
       <c r="A58" s="5">
-        <f>Hydrogramme_entree!A64</f>
+        <f>Hydrogramme_entree!A70</f>
         <v/>
       </c>
       <c r="B58" s="12">
-        <f>Hydrogramme_entree!B64</f>
+        <f>Hydrogramme_entree!B70</f>
         <v/>
       </c>
       <c r="C58" s="12">
@@ -7448,11 +8162,11 @@
     </row>
     <row r="59">
       <c r="A59" s="5">
-        <f>Hydrogramme_entree!A65</f>
+        <f>Hydrogramme_entree!A71</f>
         <v/>
       </c>
       <c r="B59" s="12">
-        <f>Hydrogramme_entree!B65</f>
+        <f>Hydrogramme_entree!B71</f>
         <v/>
       </c>
       <c r="C59" s="12">
@@ -7494,11 +8208,11 @@
     </row>
     <row r="60">
       <c r="A60" s="5">
-        <f>Hydrogramme_entree!A66</f>
+        <f>Hydrogramme_entree!A72</f>
         <v/>
       </c>
       <c r="B60" s="12">
-        <f>Hydrogramme_entree!B66</f>
+        <f>Hydrogramme_entree!B72</f>
         <v/>
       </c>
       <c r="C60" s="12">
@@ -7540,11 +8254,11 @@
     </row>
     <row r="61">
       <c r="A61" s="5">
-        <f>Hydrogramme_entree!A67</f>
+        <f>Hydrogramme_entree!A73</f>
         <v/>
       </c>
       <c r="B61" s="12">
-        <f>Hydrogramme_entree!B67</f>
+        <f>Hydrogramme_entree!B73</f>
         <v/>
       </c>
       <c r="C61" s="12">
@@ -7586,11 +8300,11 @@
     </row>
     <row r="62">
       <c r="A62" s="5">
-        <f>Hydrogramme_entree!A68</f>
+        <f>Hydrogramme_entree!A74</f>
         <v/>
       </c>
       <c r="B62" s="12">
-        <f>Hydrogramme_entree!B68</f>
+        <f>Hydrogramme_entree!B74</f>
         <v/>
       </c>
       <c r="C62" s="12">
@@ -7632,11 +8346,11 @@
     </row>
     <row r="63">
       <c r="A63" s="5">
-        <f>Hydrogramme_entree!A69</f>
+        <f>Hydrogramme_entree!A75</f>
         <v/>
       </c>
       <c r="B63" s="12">
-        <f>Hydrogramme_entree!B69</f>
+        <f>Hydrogramme_entree!B75</f>
         <v/>
       </c>
       <c r="C63" s="12">
@@ -7678,11 +8392,11 @@
     </row>
     <row r="64">
       <c r="A64" s="5">
-        <f>Hydrogramme_entree!A70</f>
+        <f>Hydrogramme_entree!A76</f>
         <v/>
       </c>
       <c r="B64" s="12">
-        <f>Hydrogramme_entree!B70</f>
+        <f>Hydrogramme_entree!B76</f>
         <v/>
       </c>
       <c r="C64" s="12">
@@ -7724,11 +8438,11 @@
     </row>
     <row r="65">
       <c r="A65" s="5">
-        <f>Hydrogramme_entree!A71</f>
+        <f>Hydrogramme_entree!A77</f>
         <v/>
       </c>
       <c r="B65" s="12">
-        <f>Hydrogramme_entree!B71</f>
+        <f>Hydrogramme_entree!B77</f>
         <v/>
       </c>
       <c r="C65" s="12">
@@ -7770,11 +8484,11 @@
     </row>
     <row r="66">
       <c r="A66" s="5">
-        <f>Hydrogramme_entree!A72</f>
+        <f>Hydrogramme_entree!A78</f>
         <v/>
       </c>
       <c r="B66" s="12">
-        <f>Hydrogramme_entree!B72</f>
+        <f>Hydrogramme_entree!B78</f>
         <v/>
       </c>
       <c r="C66" s="12">
@@ -7816,11 +8530,11 @@
     </row>
     <row r="67">
       <c r="A67" s="5">
-        <f>Hydrogramme_entree!A73</f>
+        <f>Hydrogramme_entree!A79</f>
         <v/>
       </c>
       <c r="B67" s="12">
-        <f>Hydrogramme_entree!B73</f>
+        <f>Hydrogramme_entree!B79</f>
         <v/>
       </c>
       <c r="C67" s="12">
@@ -7862,11 +8576,11 @@
     </row>
     <row r="68">
       <c r="A68" s="5">
-        <f>Hydrogramme_entree!A74</f>
+        <f>Hydrogramme_entree!A80</f>
         <v/>
       </c>
       <c r="B68" s="12">
-        <f>Hydrogramme_entree!B74</f>
+        <f>Hydrogramme_entree!B80</f>
         <v/>
       </c>
       <c r="C68" s="12">
@@ -7908,11 +8622,11 @@
     </row>
     <row r="69">
       <c r="A69" s="5">
-        <f>Hydrogramme_entree!A75</f>
+        <f>Hydrogramme_entree!A81</f>
         <v/>
       </c>
       <c r="B69" s="12">
-        <f>Hydrogramme_entree!B75</f>
+        <f>Hydrogramme_entree!B81</f>
         <v/>
       </c>
       <c r="C69" s="12">
@@ -7954,11 +8668,11 @@
     </row>
     <row r="70">
       <c r="A70" s="5">
-        <f>Hydrogramme_entree!A76</f>
+        <f>Hydrogramme_entree!A82</f>
         <v/>
       </c>
       <c r="B70" s="12">
-        <f>Hydrogramme_entree!B76</f>
+        <f>Hydrogramme_entree!B82</f>
         <v/>
       </c>
       <c r="C70" s="12">
@@ -8000,11 +8714,11 @@
     </row>
     <row r="71">
       <c r="A71" s="5">
-        <f>Hydrogramme_entree!A77</f>
+        <f>Hydrogramme_entree!A83</f>
         <v/>
       </c>
       <c r="B71" s="12">
-        <f>Hydrogramme_entree!B77</f>
+        <f>Hydrogramme_entree!B83</f>
         <v/>
       </c>
       <c r="C71" s="12">
@@ -8046,11 +8760,11 @@
     </row>
     <row r="72">
       <c r="A72" s="5">
-        <f>Hydrogramme_entree!A78</f>
+        <f>Hydrogramme_entree!A84</f>
         <v/>
       </c>
       <c r="B72" s="12">
-        <f>Hydrogramme_entree!B78</f>
+        <f>Hydrogramme_entree!B84</f>
         <v/>
       </c>
       <c r="C72" s="12">
@@ -8092,11 +8806,11 @@
     </row>
     <row r="73">
       <c r="A73" s="5">
-        <f>Hydrogramme_entree!A79</f>
+        <f>Hydrogramme_entree!A85</f>
         <v/>
       </c>
       <c r="B73" s="12">
-        <f>Hydrogramme_entree!B79</f>
+        <f>Hydrogramme_entree!B85</f>
         <v/>
       </c>
       <c r="C73" s="12">
@@ -8138,11 +8852,11 @@
     </row>
     <row r="74">
       <c r="A74" s="5">
-        <f>Hydrogramme_entree!A80</f>
+        <f>Hydrogramme_entree!A86</f>
         <v/>
       </c>
       <c r="B74" s="12">
-        <f>Hydrogramme_entree!B80</f>
+        <f>Hydrogramme_entree!B86</f>
         <v/>
       </c>
       <c r="C74" s="12">
@@ -8184,11 +8898,11 @@
     </row>
     <row r="75">
       <c r="A75" s="5">
-        <f>Hydrogramme_entree!A81</f>
+        <f>Hydrogramme_entree!A87</f>
         <v/>
       </c>
       <c r="B75" s="12">
-        <f>Hydrogramme_entree!B81</f>
+        <f>Hydrogramme_entree!B87</f>
         <v/>
       </c>
       <c r="C75" s="12">
@@ -8230,11 +8944,11 @@
     </row>
     <row r="76">
       <c r="A76" s="5">
-        <f>Hydrogramme_entree!A82</f>
+        <f>Hydrogramme_entree!A88</f>
         <v/>
       </c>
       <c r="B76" s="12">
-        <f>Hydrogramme_entree!B82</f>
+        <f>Hydrogramme_entree!B88</f>
         <v/>
       </c>
       <c r="C76" s="12">
@@ -8276,11 +8990,11 @@
     </row>
     <row r="77">
       <c r="A77" s="5">
-        <f>Hydrogramme_entree!A83</f>
+        <f>Hydrogramme_entree!A89</f>
         <v/>
       </c>
       <c r="B77" s="12">
-        <f>Hydrogramme_entree!B83</f>
+        <f>Hydrogramme_entree!B89</f>
         <v/>
       </c>
       <c r="C77" s="12">
@@ -8322,11 +9036,11 @@
     </row>
     <row r="78">
       <c r="A78" s="5">
-        <f>Hydrogramme_entree!A84</f>
+        <f>Hydrogramme_entree!A90</f>
         <v/>
       </c>
       <c r="B78" s="12">
-        <f>Hydrogramme_entree!B84</f>
+        <f>Hydrogramme_entree!B90</f>
         <v/>
       </c>
       <c r="C78" s="12">
@@ -8368,11 +9082,11 @@
     </row>
     <row r="79">
       <c r="A79" s="5">
-        <f>Hydrogramme_entree!A85</f>
+        <f>Hydrogramme_entree!A91</f>
         <v/>
       </c>
       <c r="B79" s="12">
-        <f>Hydrogramme_entree!B85</f>
+        <f>Hydrogramme_entree!B91</f>
         <v/>
       </c>
       <c r="C79" s="12">
@@ -8414,11 +9128,11 @@
     </row>
     <row r="80">
       <c r="A80" s="5">
-        <f>Hydrogramme_entree!A86</f>
+        <f>Hydrogramme_entree!A92</f>
         <v/>
       </c>
       <c r="B80" s="12">
-        <f>Hydrogramme_entree!B86</f>
+        <f>Hydrogramme_entree!B92</f>
         <v/>
       </c>
       <c r="C80" s="12">
@@ -8460,11 +9174,11 @@
     </row>
     <row r="81">
       <c r="A81" s="5">
-        <f>Hydrogramme_entree!A87</f>
+        <f>Hydrogramme_entree!A93</f>
         <v/>
       </c>
       <c r="B81" s="12">
-        <f>Hydrogramme_entree!B87</f>
+        <f>Hydrogramme_entree!B93</f>
         <v/>
       </c>
       <c r="C81" s="12">
@@ -8506,11 +9220,11 @@
     </row>
     <row r="82">
       <c r="A82" s="5">
-        <f>Hydrogramme_entree!A88</f>
+        <f>Hydrogramme_entree!A94</f>
         <v/>
       </c>
       <c r="B82" s="12">
-        <f>Hydrogramme_entree!B88</f>
+        <f>Hydrogramme_entree!B94</f>
         <v/>
       </c>
       <c r="C82" s="12">
@@ -8552,11 +9266,11 @@
     </row>
     <row r="83">
       <c r="A83" s="5">
-        <f>Hydrogramme_entree!A89</f>
+        <f>Hydrogramme_entree!A95</f>
         <v/>
       </c>
       <c r="B83" s="12">
-        <f>Hydrogramme_entree!B89</f>
+        <f>Hydrogramme_entree!B95</f>
         <v/>
       </c>
       <c r="C83" s="12">
@@ -8598,11 +9312,11 @@
     </row>
     <row r="84">
       <c r="A84" s="5">
-        <f>Hydrogramme_entree!A90</f>
+        <f>Hydrogramme_entree!A96</f>
         <v/>
       </c>
       <c r="B84" s="12">
-        <f>Hydrogramme_entree!B90</f>
+        <f>Hydrogramme_entree!B96</f>
         <v/>
       </c>
       <c r="C84" s="12">
@@ -8644,11 +9358,11 @@
     </row>
     <row r="85">
       <c r="A85" s="5">
-        <f>Hydrogramme_entree!A91</f>
+        <f>Hydrogramme_entree!A97</f>
         <v/>
       </c>
       <c r="B85" s="12">
-        <f>Hydrogramme_entree!B91</f>
+        <f>Hydrogramme_entree!B97</f>
         <v/>
       </c>
       <c r="C85" s="12">
@@ -8690,11 +9404,11 @@
     </row>
     <row r="86">
       <c r="A86" s="5">
-        <f>Hydrogramme_entree!A92</f>
+        <f>Hydrogramme_entree!A98</f>
         <v/>
       </c>
       <c r="B86" s="12">
-        <f>Hydrogramme_entree!B92</f>
+        <f>Hydrogramme_entree!B98</f>
         <v/>
       </c>
       <c r="C86" s="12">
@@ -8736,11 +9450,11 @@
     </row>
     <row r="87">
       <c r="A87" s="5">
-        <f>Hydrogramme_entree!A93</f>
+        <f>Hydrogramme_entree!A99</f>
         <v/>
       </c>
       <c r="B87" s="12">
-        <f>Hydrogramme_entree!B93</f>
+        <f>Hydrogramme_entree!B99</f>
         <v/>
       </c>
       <c r="C87" s="12">
@@ -8782,11 +9496,11 @@
     </row>
     <row r="88">
       <c r="A88" s="5">
-        <f>Hydrogramme_entree!A94</f>
+        <f>Hydrogramme_entree!A100</f>
         <v/>
       </c>
       <c r="B88" s="12">
-        <f>Hydrogramme_entree!B94</f>
+        <f>Hydrogramme_entree!B100</f>
         <v/>
       </c>
       <c r="C88" s="12">
@@ -8828,11 +9542,11 @@
     </row>
     <row r="89">
       <c r="A89" s="5">
-        <f>Hydrogramme_entree!A95</f>
+        <f>Hydrogramme_entree!A101</f>
         <v/>
       </c>
       <c r="B89" s="12">
-        <f>Hydrogramme_entree!B95</f>
+        <f>Hydrogramme_entree!B101</f>
         <v/>
       </c>
       <c r="C89" s="12">
@@ -8874,11 +9588,11 @@
     </row>
     <row r="90">
       <c r="A90" s="5">
-        <f>Hydrogramme_entree!A96</f>
+        <f>Hydrogramme_entree!A102</f>
         <v/>
       </c>
       <c r="B90" s="12">
-        <f>Hydrogramme_entree!B96</f>
+        <f>Hydrogramme_entree!B102</f>
         <v/>
       </c>
       <c r="C90" s="12">
@@ -8920,11 +9634,11 @@
     </row>
     <row r="91">
       <c r="A91" s="5">
-        <f>Hydrogramme_entree!A97</f>
+        <f>Hydrogramme_entree!A103</f>
         <v/>
       </c>
       <c r="B91" s="12">
-        <f>Hydrogramme_entree!B97</f>
+        <f>Hydrogramme_entree!B103</f>
         <v/>
       </c>
       <c r="C91" s="12">
@@ -8966,11 +9680,11 @@
     </row>
     <row r="92">
       <c r="A92" s="5">
-        <f>Hydrogramme_entree!A98</f>
+        <f>Hydrogramme_entree!A104</f>
         <v/>
       </c>
       <c r="B92" s="12">
-        <f>Hydrogramme_entree!B98</f>
+        <f>Hydrogramme_entree!B104</f>
         <v/>
       </c>
       <c r="C92" s="12">
@@ -9012,11 +9726,11 @@
     </row>
     <row r="93">
       <c r="A93" s="5">
-        <f>Hydrogramme_entree!A99</f>
+        <f>Hydrogramme_entree!A105</f>
         <v/>
       </c>
       <c r="B93" s="12">
-        <f>Hydrogramme_entree!B99</f>
+        <f>Hydrogramme_entree!B105</f>
         <v/>
       </c>
       <c r="C93" s="12">
@@ -9058,11 +9772,11 @@
     </row>
     <row r="94">
       <c r="A94" s="5">
-        <f>Hydrogramme_entree!A100</f>
+        <f>Hydrogramme_entree!A106</f>
         <v/>
       </c>
       <c r="B94" s="12">
-        <f>Hydrogramme_entree!B100</f>
+        <f>Hydrogramme_entree!B106</f>
         <v/>
       </c>
       <c r="C94" s="12">
@@ -9104,11 +9818,11 @@
     </row>
     <row r="95">
       <c r="A95" s="5">
-        <f>Hydrogramme_entree!A101</f>
+        <f>Hydrogramme_entree!A107</f>
         <v/>
       </c>
       <c r="B95" s="12">
-        <f>Hydrogramme_entree!B101</f>
+        <f>Hydrogramme_entree!B107</f>
         <v/>
       </c>
       <c r="C95" s="12">
@@ -9150,11 +9864,11 @@
     </row>
     <row r="96">
       <c r="A96" s="5">
-        <f>Hydrogramme_entree!A102</f>
+        <f>Hydrogramme_entree!A108</f>
         <v/>
       </c>
       <c r="B96" s="12">
-        <f>Hydrogramme_entree!B102</f>
+        <f>Hydrogramme_entree!B108</f>
         <v/>
       </c>
       <c r="C96" s="12">
@@ -9196,11 +9910,11 @@
     </row>
     <row r="97">
       <c r="A97" s="5">
-        <f>Hydrogramme_entree!A103</f>
+        <f>Hydrogramme_entree!A109</f>
         <v/>
       </c>
       <c r="B97" s="12">
-        <f>Hydrogramme_entree!B103</f>
+        <f>Hydrogramme_entree!B109</f>
         <v/>
       </c>
       <c r="C97" s="12">
@@ -9242,11 +9956,11 @@
     </row>
     <row r="98">
       <c r="A98" s="5">
-        <f>Hydrogramme_entree!A104</f>
+        <f>Hydrogramme_entree!A110</f>
         <v/>
       </c>
       <c r="B98" s="12">
-        <f>Hydrogramme_entree!B104</f>
+        <f>Hydrogramme_entree!B110</f>
         <v/>
       </c>
       <c r="C98" s="12">
@@ -9288,11 +10002,11 @@
     </row>
     <row r="99">
       <c r="A99" s="5">
-        <f>Hydrogramme_entree!A105</f>
+        <f>Hydrogramme_entree!A111</f>
         <v/>
       </c>
       <c r="B99" s="12">
-        <f>Hydrogramme_entree!B105</f>
+        <f>Hydrogramme_entree!B111</f>
         <v/>
       </c>
       <c r="C99" s="12">
@@ -9334,11 +10048,11 @@
     </row>
     <row r="100">
       <c r="A100" s="5">
-        <f>Hydrogramme_entree!A106</f>
+        <f>Hydrogramme_entree!A112</f>
         <v/>
       </c>
       <c r="B100" s="12">
-        <f>Hydrogramme_entree!B106</f>
+        <f>Hydrogramme_entree!B112</f>
         <v/>
       </c>
       <c r="C100" s="12">
@@ -9380,11 +10094,11 @@
     </row>
     <row r="101">
       <c r="A101" s="5">
-        <f>Hydrogramme_entree!A107</f>
+        <f>Hydrogramme_entree!A113</f>
         <v/>
       </c>
       <c r="B101" s="12">
-        <f>Hydrogramme_entree!B107</f>
+        <f>Hydrogramme_entree!B113</f>
         <v/>
       </c>
       <c r="C101" s="12">
@@ -9426,11 +10140,11 @@
     </row>
     <row r="102">
       <c r="A102" s="5">
-        <f>Hydrogramme_entree!A108</f>
+        <f>Hydrogramme_entree!A114</f>
         <v/>
       </c>
       <c r="B102" s="12">
-        <f>Hydrogramme_entree!B108</f>
+        <f>Hydrogramme_entree!B114</f>
         <v/>
       </c>
       <c r="C102" s="12">
@@ -9472,11 +10186,11 @@
     </row>
     <row r="103">
       <c r="A103" s="5">
-        <f>Hydrogramme_entree!A109</f>
+        <f>Hydrogramme_entree!A115</f>
         <v/>
       </c>
       <c r="B103" s="12">
-        <f>Hydrogramme_entree!B109</f>
+        <f>Hydrogramme_entree!B115</f>
         <v/>
       </c>
       <c r="C103" s="12">
@@ -9518,11 +10232,11 @@
     </row>
     <row r="104">
       <c r="A104" s="5">
-        <f>Hydrogramme_entree!A110</f>
+        <f>Hydrogramme_entree!A116</f>
         <v/>
       </c>
       <c r="B104" s="12">
-        <f>Hydrogramme_entree!B110</f>
+        <f>Hydrogramme_entree!B116</f>
         <v/>
       </c>
       <c r="C104" s="12">
@@ -9564,11 +10278,11 @@
     </row>
     <row r="105">
       <c r="A105" s="5">
-        <f>Hydrogramme_entree!A111</f>
+        <f>Hydrogramme_entree!A117</f>
         <v/>
       </c>
       <c r="B105" s="12">
-        <f>Hydrogramme_entree!B111</f>
+        <f>Hydrogramme_entree!B117</f>
         <v/>
       </c>
       <c r="C105" s="12">
@@ -9610,11 +10324,11 @@
     </row>
     <row r="106">
       <c r="A106" s="5">
-        <f>Hydrogramme_entree!A112</f>
+        <f>Hydrogramme_entree!A118</f>
         <v/>
       </c>
       <c r="B106" s="12">
-        <f>Hydrogramme_entree!B112</f>
+        <f>Hydrogramme_entree!B118</f>
         <v/>
       </c>
       <c r="C106" s="12">
@@ -9656,11 +10370,11 @@
     </row>
     <row r="107">
       <c r="A107" s="5">
-        <f>Hydrogramme_entree!A113</f>
+        <f>Hydrogramme_entree!A119</f>
         <v/>
       </c>
       <c r="B107" s="12">
-        <f>Hydrogramme_entree!B113</f>
+        <f>Hydrogramme_entree!B119</f>
         <v/>
       </c>
       <c r="C107" s="12">
@@ -9702,11 +10416,11 @@
     </row>
     <row r="108">
       <c r="A108" s="5">
-        <f>Hydrogramme_entree!A114</f>
+        <f>Hydrogramme_entree!A120</f>
         <v/>
       </c>
       <c r="B108" s="12">
-        <f>Hydrogramme_entree!B114</f>
+        <f>Hydrogramme_entree!B120</f>
         <v/>
       </c>
       <c r="C108" s="12">
@@ -9748,11 +10462,11 @@
     </row>
     <row r="109">
       <c r="A109" s="5">
-        <f>Hydrogramme_entree!A115</f>
+        <f>Hydrogramme_entree!A121</f>
         <v/>
       </c>
       <c r="B109" s="12">
-        <f>Hydrogramme_entree!B115</f>
+        <f>Hydrogramme_entree!B121</f>
         <v/>
       </c>
       <c r="C109" s="12">
@@ -9794,11 +10508,11 @@
     </row>
     <row r="110">
       <c r="A110" s="5">
-        <f>Hydrogramme_entree!A116</f>
+        <f>Hydrogramme_entree!A122</f>
         <v/>
       </c>
       <c r="B110" s="12">
-        <f>Hydrogramme_entree!B116</f>
+        <f>Hydrogramme_entree!B122</f>
         <v/>
       </c>
       <c r="C110" s="12">
@@ -9840,11 +10554,11 @@
     </row>
     <row r="111">
       <c r="A111" s="5">
-        <f>Hydrogramme_entree!A117</f>
+        <f>Hydrogramme_entree!A123</f>
         <v/>
       </c>
       <c r="B111" s="12">
-        <f>Hydrogramme_entree!B117</f>
+        <f>Hydrogramme_entree!B123</f>
         <v/>
       </c>
       <c r="C111" s="12">
@@ -9886,11 +10600,11 @@
     </row>
     <row r="112">
       <c r="A112" s="5">
-        <f>Hydrogramme_entree!A118</f>
+        <f>Hydrogramme_entree!A124</f>
         <v/>
       </c>
       <c r="B112" s="12">
-        <f>Hydrogramme_entree!B118</f>
+        <f>Hydrogramme_entree!B124</f>
         <v/>
       </c>
       <c r="C112" s="12">
@@ -9932,11 +10646,11 @@
     </row>
     <row r="113">
       <c r="A113" s="5">
-        <f>Hydrogramme_entree!A119</f>
+        <f>Hydrogramme_entree!A125</f>
         <v/>
       </c>
       <c r="B113" s="12">
-        <f>Hydrogramme_entree!B119</f>
+        <f>Hydrogramme_entree!B125</f>
         <v/>
       </c>
       <c r="C113" s="12">
@@ -9978,11 +10692,11 @@
     </row>
     <row r="114">
       <c r="A114" s="5">
-        <f>Hydrogramme_entree!A120</f>
+        <f>Hydrogramme_entree!A126</f>
         <v/>
       </c>
       <c r="B114" s="12">
-        <f>Hydrogramme_entree!B120</f>
+        <f>Hydrogramme_entree!B126</f>
         <v/>
       </c>
       <c r="C114" s="12">
@@ -10024,11 +10738,11 @@
     </row>
     <row r="115">
       <c r="A115" s="5">
-        <f>Hydrogramme_entree!A121</f>
+        <f>Hydrogramme_entree!A127</f>
         <v/>
       </c>
       <c r="B115" s="12">
-        <f>Hydrogramme_entree!B121</f>
+        <f>Hydrogramme_entree!B127</f>
         <v/>
       </c>
       <c r="C115" s="12">
@@ -10070,11 +10784,11 @@
     </row>
     <row r="116">
       <c r="A116" s="5">
-        <f>Hydrogramme_entree!A122</f>
+        <f>Hydrogramme_entree!A128</f>
         <v/>
       </c>
       <c r="B116" s="12">
-        <f>Hydrogramme_entree!B122</f>
+        <f>Hydrogramme_entree!B128</f>
         <v/>
       </c>
       <c r="C116" s="12">
@@ -10116,11 +10830,11 @@
     </row>
     <row r="117">
       <c r="A117" s="5">
-        <f>Hydrogramme_entree!A123</f>
+        <f>Hydrogramme_entree!A129</f>
         <v/>
       </c>
       <c r="B117" s="12">
-        <f>Hydrogramme_entree!B123</f>
+        <f>Hydrogramme_entree!B129</f>
         <v/>
       </c>
       <c r="C117" s="12">
@@ -10162,11 +10876,11 @@
     </row>
     <row r="118">
       <c r="A118" s="5">
-        <f>Hydrogramme_entree!A124</f>
+        <f>Hydrogramme_entree!A130</f>
         <v/>
       </c>
       <c r="B118" s="12">
-        <f>Hydrogramme_entree!B124</f>
+        <f>Hydrogramme_entree!B130</f>
         <v/>
       </c>
       <c r="C118" s="12">
@@ -10208,11 +10922,11 @@
     </row>
     <row r="119">
       <c r="A119" s="5">
-        <f>Hydrogramme_entree!A125</f>
+        <f>Hydrogramme_entree!A131</f>
         <v/>
       </c>
       <c r="B119" s="12">
-        <f>Hydrogramme_entree!B125</f>
+        <f>Hydrogramme_entree!B131</f>
         <v/>
       </c>
       <c r="C119" s="12">
@@ -10254,11 +10968,11 @@
     </row>
     <row r="120">
       <c r="A120" s="5">
-        <f>Hydrogramme_entree!A126</f>
+        <f>Hydrogramme_entree!A132</f>
         <v/>
       </c>
       <c r="B120" s="12">
-        <f>Hydrogramme_entree!B126</f>
+        <f>Hydrogramme_entree!B132</f>
         <v/>
       </c>
       <c r="C120" s="12">
@@ -10300,11 +11014,11 @@
     </row>
     <row r="121">
       <c r="A121" s="5">
-        <f>Hydrogramme_entree!A127</f>
+        <f>Hydrogramme_entree!A133</f>
         <v/>
       </c>
       <c r="B121" s="12">
-        <f>Hydrogramme_entree!B127</f>
+        <f>Hydrogramme_entree!B133</f>
         <v/>
       </c>
       <c r="C121" s="12">
@@ -10346,11 +11060,11 @@
     </row>
     <row r="122">
       <c r="A122" s="5">
-        <f>Hydrogramme_entree!A128</f>
+        <f>Hydrogramme_entree!A134</f>
         <v/>
       </c>
       <c r="B122" s="12">
-        <f>Hydrogramme_entree!B128</f>
+        <f>Hydrogramme_entree!B134</f>
         <v/>
       </c>
       <c r="C122" s="12">
@@ -10392,11 +11106,11 @@
     </row>
     <row r="123">
       <c r="A123" s="5">
-        <f>Hydrogramme_entree!A129</f>
+        <f>Hydrogramme_entree!A135</f>
         <v/>
       </c>
       <c r="B123" s="12">
-        <f>Hydrogramme_entree!B129</f>
+        <f>Hydrogramme_entree!B135</f>
         <v/>
       </c>
       <c r="C123" s="12">
@@ -10438,11 +11152,11 @@
     </row>
     <row r="124">
       <c r="A124" s="5">
-        <f>Hydrogramme_entree!A130</f>
+        <f>Hydrogramme_entree!A136</f>
         <v/>
       </c>
       <c r="B124" s="12">
-        <f>Hydrogramme_entree!B130</f>
+        <f>Hydrogramme_entree!B136</f>
         <v/>
       </c>
       <c r="C124" s="12">
@@ -10484,7 +11198,7 @@
     </row>
     <row r="125"/>
     <row r="126">
-      <c r="A126" s="16" t="inlineStr">
+      <c r="A126" s="19" t="inlineStr">
         <is>
           <t>Résumé (live)</t>
         </is>
@@ -10493,53 +11207,74 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>WSE max</t>
-        </is>
-      </c>
-      <c r="B127" s="19">
+          <t>WSE max (élévation)</t>
+        </is>
+      </c>
+      <c r="B127" s="20">
         <f>MAX(G5:G124)</f>
         <v/>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>m  ← niveau d'eau maximum</t>
+          <t>m  ← comparer à 37.4 m</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>S max</t>
+          <t>HW max (profondeur)</t>
         </is>
       </c>
       <c r="B128">
-        <f>MAX(H5:H124)</f>
-        <v/>
+        <f>MAX(F5:F124)</f>
+        <v/>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>m  ← au-dessus de l'invert (≈ WSE−35.36)</t>
+        </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Q_in max</t>
+          <t>S max</t>
         </is>
       </c>
       <c r="B129">
-        <f>MAX(B5:B124)</f>
-        <v/>
+        <f>MAX(H5:H124)</f>
+        <v/>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
+          <t>Q_in max</t>
+        </is>
+      </c>
+      <c r="B130">
+        <f>MAX(B5:B124)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
           <t>Réf. Python au build</t>
         </is>
       </c>
-      <c r="B130" t="n">
-        <v>37.143</v>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>m (validation optionnelle)</t>
+      <c r="B131" t="n">
+        <v>37.122</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>m WSE (validation optionnelle)</t>
         </is>
       </c>
     </row>
@@ -10563,16 +11298,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Notes hydrogramme</t>
+          <t>Chicago vs Triangle — et comment c'est construit</t>
         </is>
       </c>
     </row>
@@ -10580,23 +11315,131 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Qin triangle: montée Qpointe*t/Montée ; descente Qpointe*(1-(t-Montée)/Descente)</t>
-        </is>
+      <c r="A3">
+        <f>== MÉTHODE CHICAGO (Keifer–Chu) — défaut du classeur ===</f>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Géométrie: Parametres (live). Orage: Hydrogramme_entree. WSE max: Routing_stockage.</t>
+          <t>1) IDF: intensité moyenne ī(td) = a / (td + b)^c   (td en minutes, ī en mm/h)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Python optionnel: build_excel.py / hydraulics.py / run_model.py</t>
+          <t>2) Hyétogramme: intensité INSTANTANÉE i(t) avant/après le pic tp = r*Td</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Avant pic (tb = tp − t):  i = a * [(1−c)*(tb/r) + b] / (tb/r + b)^(c+1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Après pic (ta = t − tp):  i = a * [(1−c)*(ta/(1−r)) + b] / (ta/(1−r) + b)^(c+1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3) Pic d'intensité: i_max = a / b^c</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4) Hydrogramme calé sur un débit donné:  Q(t) = Q_pointe * i(t) / i_max</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   → pour Q_pointe = 10 m³/s, le maximum de Q_in est exactement 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Durée Td = 60 min (choix pour ce ponceau + fossé):</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - temps de parcours dans le tuyau (L=50.9 m) ≈ quelques minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Tc typique petit bassin urbain/industriel ≈ 10–20 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - règle pratique: Td ≥ ~2–3 × Tc → 60 min est adéquat (120 min si bassin plus grand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Coeffs a,b,c: remplacer par ceux de VOTRE courbe IDF (période de retour du projet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>La forme de Q(t) dépend surtout de b, c, r, Td ; a s'annule dans i/i_max.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <f>== TRIANGLE (option) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mettre B3 = Triangle. Qin = montée/descente linéaires (B6, B7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Routing: feuille Routing_stockage lit la colonne Q_in (inchangée).</t>
         </is>
       </c>
     </row>
@@ -10624,7 +11467,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Comparaison modes (instantané Python au build — pédagogique)</t>
         </is>
@@ -10644,7 +11487,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4"/>
@@ -10686,29 +11529,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>porous</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Seulement pores du remblai — faible débit</t>
         </is>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="22" t="n">
         <v>37.4</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="22" t="n">
         <v>4.422</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="22" t="n">
         <v>0.16</v>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="F6" s="22" t="n">
         <v>4.582</v>
       </c>
-      <c r="G6" s="21" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>Non / limite</t>
         </is>
@@ -10726,16 +11569,16 @@
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>37.157</v>
+        <v>37.229</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>4.235</v>
+        <v>4.291</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>4.764</v>
+        <v>5.709</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
@@ -10744,29 +11587,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Poreux + surface</t>
         </is>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="22" t="n">
         <v>37.4</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="22" t="n">
         <v>4.422</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="22" t="n">
         <v>0.16</v>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="22" t="n">
         <v>4.582</v>
       </c>
-      <c r="G8" s="21" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>Non / limite</t>
         </is>

</xml_diff>